<commit_message>
Devis 2027 : devis en portrait A4, forfait avec prix des lignes affichés ou masqués
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Devis_Enedril_2027.xlsx
+++ b/devis_2027/Devis_Enedril_2027.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'4 Devis'!$A$1:$L$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'4 Devis'!$A$1:$K$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,7 +29,7 @@
     <numFmt numFmtId="166" formatCode="#,##0;-#,##0;;@"/>
     <numFmt numFmtId="167" formatCode="#,##0.00 &quot;€&quot;"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="35">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -142,7 +142,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="17"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -159,7 +159,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0008203F"/>
-      <sz val="8"/>
+      <sz val="7.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -169,42 +169,54 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00E2231A"/>
+      <color rgb="0051647A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000B1B2E"/>
       <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000B1B2E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="0051647A"/>
-      <sz val="10"/>
+      <color rgb="00E2231A"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000B1B2E"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="22"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="20"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="0008203F"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="0051647A"/>
-      <sz val="8.5"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -215,7 +227,7 @@
     <font>
       <name val="Calibri"/>
       <color rgb="0051647A"/>
-      <sz val="8"/>
+      <sz val="7.5"/>
     </font>
   </fonts>
   <fills count="8">
@@ -298,11 +310,6 @@
       </top>
     </border>
     <border>
-      <top style="thin">
-        <color rgb="00D5DEE8"/>
-      </top>
-    </border>
-    <border>
       <right style="thin">
         <color rgb="00D5DEE8"/>
       </right>
@@ -315,7 +322,6 @@
         <color rgb="00D5DEE8"/>
       </left>
     </border>
-    <border/>
     <border>
       <right style="thin">
         <color rgb="00D5DEE8"/>
@@ -337,11 +343,17 @@
         <color rgb="00D5DEE8"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00D5DEE8"/>
+      </top>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -409,6 +421,9 @@
     <xf numFmtId="167" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -433,64 +448,76 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" shrinkToFit="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -658,7 +685,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1428750" cy="323850"/>
+    <ext cx="1333500" cy="304800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2066,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2371,34 +2398,52 @@
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="20" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Afficher les prix des lignes du forfait sur le devis</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Oui : chaque ligne garde ses tarifs ; Non : elles s’affichent « incl. ». Dans les deux cas le prix final du forfait apparaît dans le bandeau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>Rappels</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="27" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>Transport « Coût réel +15 % » : aucun montant affiché. Choisir « Forfait » pour imposer un prix.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="27" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>Lignes couvertes par le forfait : mettre « Oui » dans « Inclus au forfait » (onglet 2). Elles s’affichent « incl. » sur le devis.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="D15:H17"/>
+    <mergeCell ref="D18:H18"/>
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="B12:H12"/>
   </mergeCells>
-  <dataValidations count="12">
+  <dataValidations count="13">
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="stop">
       <formula1>=Listes!$G$2:$G$12</formula1>
     </dataValidation>
@@ -2435,6 +2480,9 @@
     <dataValidation sqref="G13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="stop">
       <formula1>=Listes!$N$2:$N$12</formula1>
     </dataValidation>
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur" error="Choisir une valeur de la liste." type="list" errorStyle="stop">
+      <formula1>=Listes!$G$2:$G$12</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2448,45 +2496,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="1.5" customWidth="1" min="12" max="12"/>
-    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col width="4.5" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="5.5" customWidth="1" min="4" max="4"/>
+    <col width="10.5" customWidth="1" min="5" max="5"/>
+    <col width="10.5" customWidth="1" min="6" max="6"/>
+    <col width="10.5" customWidth="1" min="7" max="7"/>
+    <col width="12.5" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="1.5" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="28">
+      <c r="D1" s="29">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("title",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="L1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="1" t="n"/>
       <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="29">
+      <c r="D2" s="30">
         <f>"N° "&amp;'1 Affaire'!$C$6&amp;"   ·   "&amp;IF('1 Affaire'!$C$7="","",TEXT('1 Affaire'!$C$7,"dd/mm/yyyy"))</f>
         <v/>
       </c>
-      <c r="L2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
     </row>
     <row r="3" ht="5" customHeight="1">
       <c r="A3" s="4" t="n"/>
@@ -2500,1581 +2545,1494 @@
       <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
-      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="15" customHeight="1">
-      <c r="B5" s="30">
+      <c r="B5" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("client",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("offer",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
-      <c r="G5" s="30">
+      <c r="H5" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("date",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
-      <c r="I5" s="30">
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="B6" s="32">
+        <f>""&amp;'1 Affaire'!$C$8</f>
+        <v/>
+      </c>
+      <c r="C6" s="33" t="n"/>
+      <c r="D6" s="32">
+        <f>""&amp;'1 Affaire'!$C$6</f>
+        <v/>
+      </c>
+      <c r="E6" s="33" t="n"/>
+      <c r="F6" s="33" t="n"/>
+      <c r="G6" s="33" t="n"/>
+      <c r="H6" s="32">
+        <f>IF('1 Affaire'!$C$7="","",TEXT('1 Affaire'!$C$7,"dd/mm/yyyy"))</f>
+        <v/>
+      </c>
+      <c r="I6" s="33" t="n"/>
+      <c r="J6" s="33" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="31">
+        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("attn",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <v/>
+      </c>
+      <c r="D7" s="31">
+        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("well",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <v/>
+      </c>
+      <c r="H7" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("by",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="19" customHeight="1">
-      <c r="B6" s="31">
-        <f>""&amp;'1 Affaire'!$C$8</f>
-        <v/>
-      </c>
-      <c r="C6" s="32" t="n"/>
-      <c r="D6" s="31">
-        <f>""&amp;'1 Affaire'!$C$6</f>
-        <v/>
-      </c>
-      <c r="E6" s="32" t="n"/>
-      <c r="F6" s="32" t="n"/>
-      <c r="G6" s="31">
-        <f>IF('1 Affaire'!$C$7="","",TEXT('1 Affaire'!$C$7,"dd/mm/yyyy"))</f>
-        <v/>
-      </c>
-      <c r="H6" s="32" t="n"/>
-      <c r="I6" s="31">
+    <row r="8" ht="19" customHeight="1">
+      <c r="B8" s="32">
+        <f>""&amp;'1 Affaire'!$C$9</f>
+        <v/>
+      </c>
+      <c r="C8" s="33" t="n"/>
+      <c r="D8" s="32">
+        <f>""&amp;'1 Affaire'!$C$10</f>
+        <v/>
+      </c>
+      <c r="E8" s="33" t="n"/>
+      <c r="F8" s="33" t="n"/>
+      <c r="G8" s="33" t="n"/>
+      <c r="H8" s="32">
         <f>""&amp;'1 Affaire'!$F$6</f>
         <v/>
       </c>
-      <c r="J6" s="32" t="n"/>
-      <c r="K6" s="32" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="B7" s="30">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("attn",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
-        <v/>
-      </c>
-      <c r="D7" s="30">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("well",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
-        <v/>
-      </c>
-      <c r="G7" s="30">
+      <c r="I8" s="33" t="n"/>
+      <c r="J8" s="33" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("inco",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
-      <c r="I7" s="30">
+      <c r="D9" s="31">
+        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("valid",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <v/>
+      </c>
+      <c r="H9" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("mail",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
-      <c r="B8" s="31">
-        <f>""&amp;'1 Affaire'!$C$9</f>
-        <v/>
-      </c>
-      <c r="C8" s="32" t="n"/>
-      <c r="D8" s="31">
-        <f>""&amp;'1 Affaire'!$C$10</f>
-        <v/>
-      </c>
-      <c r="E8" s="32" t="n"/>
-      <c r="F8" s="32" t="n"/>
-      <c r="G8" s="31">
+    <row r="10" ht="19" customHeight="1">
+      <c r="B10" s="32">
         <f>""&amp;'1 Affaire'!$F$10</f>
         <v/>
       </c>
-      <c r="H8" s="32" t="n"/>
-      <c r="I8" s="31">
+      <c r="C10" s="33" t="n"/>
+      <c r="D10" s="32">
+        <f>""&amp;'1 Affaire'!$F$9</f>
+        <v/>
+      </c>
+      <c r="E10" s="33" t="n"/>
+      <c r="F10" s="33" t="n"/>
+      <c r="G10" s="33" t="n"/>
+      <c r="H10" s="32">
         <f>""&amp;'1 Affaire'!$F$7</f>
         <v/>
       </c>
-      <c r="J8" s="32" t="n"/>
-      <c r="K8" s="32" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="B9" s="30">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("valid",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
-        <v/>
-      </c>
-      <c r="D9" s="30">
+      <c r="I10" s="33" t="n"/>
+      <c r="J10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="B11" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("lead",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
-      <c r="G9" s="30">
+      <c r="D11" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("we",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
-      <c r="I9" s="30">
+      <c r="H11" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("tel",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
-      <c r="B10" s="31">
-        <f>""&amp;'1 Affaire'!$F$9</f>
-        <v/>
-      </c>
-      <c r="C10" s="32" t="n"/>
-      <c r="D10" s="31">
+    <row r="12" ht="19" customHeight="1">
+      <c r="B12" s="32">
         <f>""&amp;'1 Affaire'!$F$11</f>
         <v/>
       </c>
-      <c r="E10" s="32" t="n"/>
-      <c r="F10" s="32" t="n"/>
-      <c r="G10" s="31">
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="32">
         <f>""&amp;'1 Affaire'!$F$13</f>
         <v/>
       </c>
-      <c r="H10" s="32" t="n"/>
-      <c r="I10" s="31">
+      <c r="E12" s="33" t="n"/>
+      <c r="F12" s="33" t="n"/>
+      <c r="G12" s="33" t="n"/>
+      <c r="H12" s="32">
         <f>""&amp;'1 Affaire'!$F$8</f>
         <v/>
       </c>
-      <c r="J10" s="32" t="n"/>
-      <c r="K10" s="32" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="B11" s="30">
+      <c r="I12" s="33" t="n"/>
+      <c r="J12" s="33" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="31">
         <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("pay",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
-      <c r="B12" s="31">
+    <row r="14" ht="19" customHeight="1">
+      <c r="B14" s="32">
         <f>""&amp;'1 Affaire'!$F$12</f>
         <v/>
       </c>
-      <c r="C12" s="32" t="n"/>
-    </row>
-    <row r="13" ht="8" customHeight="1"/>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="33">
+      <c r="C14" s="33" t="n"/>
+    </row>
+    <row r="15" ht="8" customHeight="1"/>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="34">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("sec_eq",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="C14" s="34" t="n"/>
-      <c r="D14" s="34" t="n"/>
-      <c r="E14" s="34" t="n"/>
-      <c r="F14" s="34" t="n"/>
-      <c r="G14" s="34" t="n"/>
-      <c r="H14" s="34" t="n"/>
-      <c r="I14" s="34" t="n"/>
-      <c r="J14" s="34" t="n"/>
-      <c r="K14" s="34" t="n"/>
-    </row>
-    <row r="15" ht="44" customHeight="1">
-      <c r="B15" s="35">
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="35" t="n"/>
+      <c r="H16" s="35" t="n"/>
+      <c r="I16" s="35" t="n"/>
+      <c r="J16" s="35" t="n"/>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="B17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_n",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="C15" s="36">
+      <c r="C17" s="37">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_desc",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="D15" s="35">
+      <c r="D17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="E15" s="35">
+      <c r="E17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_s",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="F15" s="35">
+      <c r="F17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_o",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="G15" s="35">
+      <c r="G17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_uc",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="H15" s="35">
+      <c r="H17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_lih",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="I15" s="35">
+      <c r="I17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_insp",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="J15" s="35">
+      <c r="J17" s="36">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("h_rest",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="K15" s="35">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_ref",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="21" customHeight="1">
-      <c r="B16" s="13">
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="B18" s="38">
         <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),'2 Matériel'!$A6,"")</f>
         <v/>
       </c>
-      <c r="C16" s="37">
-        <f>IF('2 Matériel'!$L6&gt;0,IF('2 Matériel'!$B6="Oui",UPPER('2 Matériel'!$C6),'2 Matériel'!$C6),"")</f>
-        <v/>
-      </c>
-      <c r="D16" s="38">
+      <c r="C18" s="39">
+        <f>IF('2 Matériel'!$L6&gt;0,IF('2 Matériel'!$B6="Oui",UPPER('2 Matériel'!$C6),'2 Matériel'!$C6&amp;IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D18" s="40">
         <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),'2 Matériel'!$L6,"")</f>
         <v/>
       </c>
-      <c r="E16" s="39">
-        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E6="","",'2 Matériel'!$E6)),"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="39">
-        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F6="","",'2 Matériel'!$F6)),"")</f>
-        <v/>
-      </c>
-      <c r="G16" s="39">
-        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G6="","",'2 Matériel'!$G6)),"")</f>
-        <v/>
-      </c>
-      <c r="H16" s="39">
-        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H6="","",'2 Matériel'!$H6)),"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="39">
-        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I6="","",'2 Matériel'!$I6)),"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="39">
-        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J6="","",'2 Matériel'!$J6)),"")</f>
-        <v/>
-      </c>
-      <c r="K16" s="40">
-        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M16" s="41">
+      <c r="E18" s="41">
+        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E6="","",'2 Matériel'!$E6)),"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="41">
+        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F6="","",'2 Matériel'!$F6)),"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="41">
+        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G6="","",'2 Matériel'!$G6)),"")</f>
+        <v/>
+      </c>
+      <c r="H18" s="41">
+        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H6="","",'2 Matériel'!$H6)),"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="41">
+        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I6="","",'2 Matériel'!$I6)),"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="41">
+        <f>IF(AND('2 Matériel'!$L6&gt;0,NOT('2 Matériel'!$B6="Oui")),IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J6="","",'2 Matériel'!$J6)),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="42">
         <f>IF(AND('2 Matériel'!$L6&gt;0,'2 Matériel'!$B6="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="21" customHeight="1">
-      <c r="B17" s="13">
+    <row r="19" ht="21" customHeight="1">
+      <c r="B19" s="38">
         <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),'2 Matériel'!$A7,"")</f>
         <v/>
       </c>
-      <c r="C17" s="37">
-        <f>IF('2 Matériel'!$L7&gt;0,IF('2 Matériel'!$B7="Oui",UPPER('2 Matériel'!$C7),'2 Matériel'!$C7),"")</f>
-        <v/>
-      </c>
-      <c r="D17" s="38">
+      <c r="C19" s="39">
+        <f>IF('2 Matériel'!$L7&gt;0,IF('2 Matériel'!$B7="Oui",UPPER('2 Matériel'!$C7),'2 Matériel'!$C7&amp;IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D19" s="40">
         <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),'2 Matériel'!$L7,"")</f>
         <v/>
       </c>
-      <c r="E17" s="39">
-        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E7="","",'2 Matériel'!$E7)),"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="39">
-        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F7="","",'2 Matériel'!$F7)),"")</f>
-        <v/>
-      </c>
-      <c r="G17" s="39">
-        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G7="","",'2 Matériel'!$G7)),"")</f>
-        <v/>
-      </c>
-      <c r="H17" s="39">
-        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H7="","",'2 Matériel'!$H7)),"")</f>
-        <v/>
-      </c>
-      <c r="I17" s="39">
-        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I7="","",'2 Matériel'!$I7)),"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="39">
-        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J7="","",'2 Matériel'!$J7)),"")</f>
-        <v/>
-      </c>
-      <c r="K17" s="40">
-        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M17" s="41">
+      <c r="E19" s="41">
+        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E7="","",'2 Matériel'!$E7)),"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="41">
+        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F7="","",'2 Matériel'!$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="41">
+        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G7="","",'2 Matériel'!$G7)),"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="41">
+        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H7="","",'2 Matériel'!$H7)),"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="41">
+        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I7="","",'2 Matériel'!$I7)),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="41">
+        <f>IF(AND('2 Matériel'!$L7&gt;0,NOT('2 Matériel'!$B7="Oui")),IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J7="","",'2 Matériel'!$J7)),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="42">
         <f>IF(AND('2 Matériel'!$L7&gt;0,'2 Matériel'!$B7="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="21" customHeight="1">
-      <c r="B18" s="13">
+    <row r="20" ht="21" customHeight="1">
+      <c r="B20" s="38">
         <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),'2 Matériel'!$A8,"")</f>
         <v/>
       </c>
-      <c r="C18" s="37">
-        <f>IF('2 Matériel'!$L8&gt;0,IF('2 Matériel'!$B8="Oui",UPPER('2 Matériel'!$C8),'2 Matériel'!$C8),"")</f>
-        <v/>
-      </c>
-      <c r="D18" s="38">
+      <c r="C20" s="39">
+        <f>IF('2 Matériel'!$L8&gt;0,IF('2 Matériel'!$B8="Oui",UPPER('2 Matériel'!$C8),'2 Matériel'!$C8&amp;IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D20" s="40">
         <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),'2 Matériel'!$L8,"")</f>
         <v/>
       </c>
-      <c r="E18" s="39">
-        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E8="","",'2 Matériel'!$E8)),"")</f>
-        <v/>
-      </c>
-      <c r="F18" s="39">
-        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F8="","",'2 Matériel'!$F8)),"")</f>
-        <v/>
-      </c>
-      <c r="G18" s="39">
-        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G8="","",'2 Matériel'!$G8)),"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="39">
-        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H8="","",'2 Matériel'!$H8)),"")</f>
-        <v/>
-      </c>
-      <c r="I18" s="39">
-        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I8="","",'2 Matériel'!$I8)),"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="39">
-        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J8="","",'2 Matériel'!$J8)),"")</f>
-        <v/>
-      </c>
-      <c r="K18" s="40">
-        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M18" s="41">
+      <c r="E20" s="41">
+        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E8="","",'2 Matériel'!$E8)),"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="41">
+        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F8="","",'2 Matériel'!$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="41">
+        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G8="","",'2 Matériel'!$G8)),"")</f>
+        <v/>
+      </c>
+      <c r="H20" s="41">
+        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H8="","",'2 Matériel'!$H8)),"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="41">
+        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I8="","",'2 Matériel'!$I8)),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="41">
+        <f>IF(AND('2 Matériel'!$L8&gt;0,NOT('2 Matériel'!$B8="Oui")),IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J8="","",'2 Matériel'!$J8)),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="42">
         <f>IF(AND('2 Matériel'!$L8&gt;0,'2 Matériel'!$B8="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="21" customHeight="1">
-      <c r="B19" s="13">
+    <row r="21" ht="21" customHeight="1">
+      <c r="B21" s="38">
         <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),'2 Matériel'!$A9,"")</f>
         <v/>
       </c>
-      <c r="C19" s="37">
-        <f>IF('2 Matériel'!$L9&gt;0,IF('2 Matériel'!$B9="Oui",UPPER('2 Matériel'!$C9),'2 Matériel'!$C9),"")</f>
-        <v/>
-      </c>
-      <c r="D19" s="38">
+      <c r="C21" s="39">
+        <f>IF('2 Matériel'!$L9&gt;0,IF('2 Matériel'!$B9="Oui",UPPER('2 Matériel'!$C9),'2 Matériel'!$C9&amp;IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D21" s="40">
         <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),'2 Matériel'!$L9,"")</f>
         <v/>
       </c>
-      <c r="E19" s="39">
-        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E9="","",'2 Matériel'!$E9)),"")</f>
-        <v/>
-      </c>
-      <c r="F19" s="39">
-        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F9="","",'2 Matériel'!$F9)),"")</f>
-        <v/>
-      </c>
-      <c r="G19" s="39">
-        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G9="","",'2 Matériel'!$G9)),"")</f>
-        <v/>
-      </c>
-      <c r="H19" s="39">
-        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H9="","",'2 Matériel'!$H9)),"")</f>
-        <v/>
-      </c>
-      <c r="I19" s="39">
-        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I9="","",'2 Matériel'!$I9)),"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="39">
-        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J9="","",'2 Matériel'!$J9)),"")</f>
-        <v/>
-      </c>
-      <c r="K19" s="40">
-        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M19" s="41">
+      <c r="E21" s="41">
+        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E9="","",'2 Matériel'!$E9)),"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="41">
+        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F9="","",'2 Matériel'!$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="41">
+        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G9="","",'2 Matériel'!$G9)),"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="41">
+        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H9="","",'2 Matériel'!$H9)),"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="41">
+        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I9="","",'2 Matériel'!$I9)),"")</f>
+        <v/>
+      </c>
+      <c r="J21" s="41">
+        <f>IF(AND('2 Matériel'!$L9&gt;0,NOT('2 Matériel'!$B9="Oui")),IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J9="","",'2 Matériel'!$J9)),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="42">
         <f>IF(AND('2 Matériel'!$L9&gt;0,'2 Matériel'!$B9="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="21" customHeight="1">
-      <c r="B20" s="13">
+    <row r="22" ht="21" customHeight="1">
+      <c r="B22" s="38">
         <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),'2 Matériel'!$A10,"")</f>
         <v/>
       </c>
-      <c r="C20" s="37">
-        <f>IF('2 Matériel'!$L10&gt;0,IF('2 Matériel'!$B10="Oui",UPPER('2 Matériel'!$C10),'2 Matériel'!$C10),"")</f>
-        <v/>
-      </c>
-      <c r="D20" s="38">
+      <c r="C22" s="39">
+        <f>IF('2 Matériel'!$L10&gt;0,IF('2 Matériel'!$B10="Oui",UPPER('2 Matériel'!$C10),'2 Matériel'!$C10&amp;IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D22" s="40">
         <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),'2 Matériel'!$L10,"")</f>
         <v/>
       </c>
-      <c r="E20" s="39">
-        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E10="","",'2 Matériel'!$E10)),"")</f>
-        <v/>
-      </c>
-      <c r="F20" s="39">
-        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F10="","",'2 Matériel'!$F10)),"")</f>
-        <v/>
-      </c>
-      <c r="G20" s="39">
-        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G10="","",'2 Matériel'!$G10)),"")</f>
-        <v/>
-      </c>
-      <c r="H20" s="39">
-        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H10="","",'2 Matériel'!$H10)),"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="39">
-        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I10="","",'2 Matériel'!$I10)),"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="39">
-        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J10="","",'2 Matériel'!$J10)),"")</f>
-        <v/>
-      </c>
-      <c r="K20" s="40">
-        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="41">
+      <c r="E22" s="41">
+        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E10="","",'2 Matériel'!$E10)),"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="41">
+        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F10="","",'2 Matériel'!$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="41">
+        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G10="","",'2 Matériel'!$G10)),"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="41">
+        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H10="","",'2 Matériel'!$H10)),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="41">
+        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I10="","",'2 Matériel'!$I10)),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="41">
+        <f>IF(AND('2 Matériel'!$L10&gt;0,NOT('2 Matériel'!$B10="Oui")),IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J10="","",'2 Matériel'!$J10)),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="42">
         <f>IF(AND('2 Matériel'!$L10&gt;0,'2 Matériel'!$B10="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="21" customHeight="1">
-      <c r="B21" s="13">
+    <row r="23" ht="21" customHeight="1">
+      <c r="B23" s="38">
         <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),'2 Matériel'!$A11,"")</f>
         <v/>
       </c>
-      <c r="C21" s="37">
-        <f>IF('2 Matériel'!$L11&gt;0,IF('2 Matériel'!$B11="Oui",UPPER('2 Matériel'!$C11),'2 Matériel'!$C11),"")</f>
-        <v/>
-      </c>
-      <c r="D21" s="38">
+      <c r="C23" s="39">
+        <f>IF('2 Matériel'!$L11&gt;0,IF('2 Matériel'!$B11="Oui",UPPER('2 Matériel'!$C11),'2 Matériel'!$C11&amp;IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D23" s="40">
         <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),'2 Matériel'!$L11,"")</f>
         <v/>
       </c>
-      <c r="E21" s="39">
-        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E11="","",'2 Matériel'!$E11)),"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="39">
-        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F11="","",'2 Matériel'!$F11)),"")</f>
-        <v/>
-      </c>
-      <c r="G21" s="39">
-        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G11="","",'2 Matériel'!$G11)),"")</f>
-        <v/>
-      </c>
-      <c r="H21" s="39">
-        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H11="","",'2 Matériel'!$H11)),"")</f>
-        <v/>
-      </c>
-      <c r="I21" s="39">
-        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I11="","",'2 Matériel'!$I11)),"")</f>
-        <v/>
-      </c>
-      <c r="J21" s="39">
-        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J11="","",'2 Matériel'!$J11)),"")</f>
-        <v/>
-      </c>
-      <c r="K21" s="40">
-        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M21" s="41">
+      <c r="E23" s="41">
+        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E11="","",'2 Matériel'!$E11)),"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="41">
+        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F11="","",'2 Matériel'!$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="41">
+        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G11="","",'2 Matériel'!$G11)),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="41">
+        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H11="","",'2 Matériel'!$H11)),"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="41">
+        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I11="","",'2 Matériel'!$I11)),"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="41">
+        <f>IF(AND('2 Matériel'!$L11&gt;0,NOT('2 Matériel'!$B11="Oui")),IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J11="","",'2 Matériel'!$J11)),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="42">
         <f>IF(AND('2 Matériel'!$L11&gt;0,'2 Matériel'!$B11="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="21" customHeight="1">
-      <c r="B22" s="13">
+    <row r="24" ht="21" customHeight="1">
+      <c r="B24" s="38">
         <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),'2 Matériel'!$A12,"")</f>
         <v/>
       </c>
-      <c r="C22" s="37">
-        <f>IF('2 Matériel'!$L12&gt;0,IF('2 Matériel'!$B12="Oui",UPPER('2 Matériel'!$C12),'2 Matériel'!$C12),"")</f>
-        <v/>
-      </c>
-      <c r="D22" s="38">
+      <c r="C24" s="39">
+        <f>IF('2 Matériel'!$L12&gt;0,IF('2 Matériel'!$B12="Oui",UPPER('2 Matériel'!$C12),'2 Matériel'!$C12&amp;IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D24" s="40">
         <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),'2 Matériel'!$L12,"")</f>
         <v/>
       </c>
-      <c r="E22" s="39">
-        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E12="","",'2 Matériel'!$E12)),"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="39">
-        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F12="","",'2 Matériel'!$F12)),"")</f>
-        <v/>
-      </c>
-      <c r="G22" s="39">
-        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G12="","",'2 Matériel'!$G12)),"")</f>
-        <v/>
-      </c>
-      <c r="H22" s="39">
-        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H12="","",'2 Matériel'!$H12)),"")</f>
-        <v/>
-      </c>
-      <c r="I22" s="39">
-        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I12="","",'2 Matériel'!$I12)),"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="39">
-        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J12="","",'2 Matériel'!$J12)),"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="40">
-        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M22" s="41">
+      <c r="E24" s="41">
+        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E12="","",'2 Matériel'!$E12)),"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="41">
+        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F12="","",'2 Matériel'!$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="41">
+        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G12="","",'2 Matériel'!$G12)),"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="41">
+        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H12="","",'2 Matériel'!$H12)),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="41">
+        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I12="","",'2 Matériel'!$I12)),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="41">
+        <f>IF(AND('2 Matériel'!$L12&gt;0,NOT('2 Matériel'!$B12="Oui")),IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J12="","",'2 Matériel'!$J12)),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="42">
         <f>IF(AND('2 Matériel'!$L12&gt;0,'2 Matériel'!$B12="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="21" customHeight="1">
-      <c r="B23" s="13">
+    <row r="25" ht="21" customHeight="1">
+      <c r="B25" s="38">
         <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),'2 Matériel'!$A13,"")</f>
         <v/>
       </c>
-      <c r="C23" s="37">
-        <f>IF('2 Matériel'!$L13&gt;0,IF('2 Matériel'!$B13="Oui",UPPER('2 Matériel'!$C13),'2 Matériel'!$C13),"")</f>
-        <v/>
-      </c>
-      <c r="D23" s="38">
+      <c r="C25" s="39">
+        <f>IF('2 Matériel'!$L13&gt;0,IF('2 Matériel'!$B13="Oui",UPPER('2 Matériel'!$C13),'2 Matériel'!$C13&amp;IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D25" s="40">
         <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),'2 Matériel'!$L13,"")</f>
         <v/>
       </c>
-      <c r="E23" s="39">
-        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E13="","",'2 Matériel'!$E13)),"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="39">
-        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F13="","",'2 Matériel'!$F13)),"")</f>
-        <v/>
-      </c>
-      <c r="G23" s="39">
-        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G13="","",'2 Matériel'!$G13)),"")</f>
-        <v/>
-      </c>
-      <c r="H23" s="39">
-        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H13="","",'2 Matériel'!$H13)),"")</f>
-        <v/>
-      </c>
-      <c r="I23" s="39">
-        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I13="","",'2 Matériel'!$I13)),"")</f>
-        <v/>
-      </c>
-      <c r="J23" s="39">
-        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J13="","",'2 Matériel'!$J13)),"")</f>
-        <v/>
-      </c>
-      <c r="K23" s="40">
-        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M23" s="41">
+      <c r="E25" s="41">
+        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E13="","",'2 Matériel'!$E13)),"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="41">
+        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F13="","",'2 Matériel'!$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="41">
+        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G13="","",'2 Matériel'!$G13)),"")</f>
+        <v/>
+      </c>
+      <c r="H25" s="41">
+        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H13="","",'2 Matériel'!$H13)),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="41">
+        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I13="","",'2 Matériel'!$I13)),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="41">
+        <f>IF(AND('2 Matériel'!$L13&gt;0,NOT('2 Matériel'!$B13="Oui")),IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J13="","",'2 Matériel'!$J13)),"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="42">
         <f>IF(AND('2 Matériel'!$L13&gt;0,'2 Matériel'!$B13="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="21" customHeight="1">
-      <c r="B24" s="13">
+    <row r="26" ht="21" customHeight="1">
+      <c r="B26" s="38">
         <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),'2 Matériel'!$A14,"")</f>
         <v/>
       </c>
-      <c r="C24" s="37">
-        <f>IF('2 Matériel'!$L14&gt;0,IF('2 Matériel'!$B14="Oui",UPPER('2 Matériel'!$C14),'2 Matériel'!$C14),"")</f>
-        <v/>
-      </c>
-      <c r="D24" s="38">
+      <c r="C26" s="39">
+        <f>IF('2 Matériel'!$L14&gt;0,IF('2 Matériel'!$B14="Oui",UPPER('2 Matériel'!$C14),'2 Matériel'!$C14&amp;IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D26" s="40">
         <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),'2 Matériel'!$L14,"")</f>
         <v/>
       </c>
-      <c r="E24" s="39">
-        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E14="","",'2 Matériel'!$E14)),"")</f>
-        <v/>
-      </c>
-      <c r="F24" s="39">
-        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F14="","",'2 Matériel'!$F14)),"")</f>
-        <v/>
-      </c>
-      <c r="G24" s="39">
-        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G14="","",'2 Matériel'!$G14)),"")</f>
-        <v/>
-      </c>
-      <c r="H24" s="39">
-        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H14="","",'2 Matériel'!$H14)),"")</f>
-        <v/>
-      </c>
-      <c r="I24" s="39">
-        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I14="","",'2 Matériel'!$I14)),"")</f>
-        <v/>
-      </c>
-      <c r="J24" s="39">
-        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J14="","",'2 Matériel'!$J14)),"")</f>
-        <v/>
-      </c>
-      <c r="K24" s="40">
-        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M24" s="41">
+      <c r="E26" s="41">
+        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E14="","",'2 Matériel'!$E14)),"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="41">
+        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F14="","",'2 Matériel'!$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="41">
+        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G14="","",'2 Matériel'!$G14)),"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="41">
+        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H14="","",'2 Matériel'!$H14)),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="41">
+        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I14="","",'2 Matériel'!$I14)),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="41">
+        <f>IF(AND('2 Matériel'!$L14&gt;0,NOT('2 Matériel'!$B14="Oui")),IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J14="","",'2 Matériel'!$J14)),"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="42">
         <f>IF(AND('2 Matériel'!$L14&gt;0,'2 Matériel'!$B14="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="25" ht="21" customHeight="1">
-      <c r="B25" s="13">
+    <row r="27" ht="21" customHeight="1">
+      <c r="B27" s="38">
         <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),'2 Matériel'!$A15,"")</f>
         <v/>
       </c>
-      <c r="C25" s="37">
-        <f>IF('2 Matériel'!$L15&gt;0,IF('2 Matériel'!$B15="Oui",UPPER('2 Matériel'!$C15),'2 Matériel'!$C15),"")</f>
-        <v/>
-      </c>
-      <c r="D25" s="38">
+      <c r="C27" s="39">
+        <f>IF('2 Matériel'!$L15&gt;0,IF('2 Matériel'!$B15="Oui",UPPER('2 Matériel'!$C15),'2 Matériel'!$C15&amp;IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D27" s="40">
         <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),'2 Matériel'!$L15,"")</f>
         <v/>
       </c>
-      <c r="E25" s="39">
-        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E15="","",'2 Matériel'!$E15)),"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="39">
-        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F15="","",'2 Matériel'!$F15)),"")</f>
-        <v/>
-      </c>
-      <c r="G25" s="39">
-        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G15="","",'2 Matériel'!$G15)),"")</f>
-        <v/>
-      </c>
-      <c r="H25" s="39">
-        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H15="","",'2 Matériel'!$H15)),"")</f>
-        <v/>
-      </c>
-      <c r="I25" s="39">
-        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I15="","",'2 Matériel'!$I15)),"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="39">
-        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J15="","",'2 Matériel'!$J15)),"")</f>
-        <v/>
-      </c>
-      <c r="K25" s="40">
-        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M25" s="41">
+      <c r="E27" s="41">
+        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E15="","",'2 Matériel'!$E15)),"")</f>
+        <v/>
+      </c>
+      <c r="F27" s="41">
+        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F15="","",'2 Matériel'!$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="41">
+        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G15="","",'2 Matériel'!$G15)),"")</f>
+        <v/>
+      </c>
+      <c r="H27" s="41">
+        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H15="","",'2 Matériel'!$H15)),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="41">
+        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I15="","",'2 Matériel'!$I15)),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="41">
+        <f>IF(AND('2 Matériel'!$L15&gt;0,NOT('2 Matériel'!$B15="Oui")),IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J15="","",'2 Matériel'!$J15)),"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="42">
         <f>IF(AND('2 Matériel'!$L15&gt;0,'2 Matériel'!$B15="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="26" ht="21" customHeight="1">
-      <c r="B26" s="13">
+    <row r="28" ht="21" customHeight="1">
+      <c r="B28" s="38">
         <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),'2 Matériel'!$A16,"")</f>
         <v/>
       </c>
-      <c r="C26" s="37">
-        <f>IF('2 Matériel'!$L16&gt;0,IF('2 Matériel'!$B16="Oui",UPPER('2 Matériel'!$C16),'2 Matériel'!$C16),"")</f>
-        <v/>
-      </c>
-      <c r="D26" s="38">
+      <c r="C28" s="39">
+        <f>IF('2 Matériel'!$L16&gt;0,IF('2 Matériel'!$B16="Oui",UPPER('2 Matériel'!$C16),'2 Matériel'!$C16&amp;IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D28" s="40">
         <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),'2 Matériel'!$L16,"")</f>
         <v/>
       </c>
-      <c r="E26" s="39">
-        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E16="","",'2 Matériel'!$E16)),"")</f>
-        <v/>
-      </c>
-      <c r="F26" s="39">
-        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F16="","",'2 Matériel'!$F16)),"")</f>
-        <v/>
-      </c>
-      <c r="G26" s="39">
-        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G16="","",'2 Matériel'!$G16)),"")</f>
-        <v/>
-      </c>
-      <c r="H26" s="39">
-        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H16="","",'2 Matériel'!$H16)),"")</f>
-        <v/>
-      </c>
-      <c r="I26" s="39">
-        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I16="","",'2 Matériel'!$I16)),"")</f>
-        <v/>
-      </c>
-      <c r="J26" s="39">
-        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J16="","",'2 Matériel'!$J16)),"")</f>
-        <v/>
-      </c>
-      <c r="K26" s="40">
-        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M26" s="41">
+      <c r="E28" s="41">
+        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E16="","",'2 Matériel'!$E16)),"")</f>
+        <v/>
+      </c>
+      <c r="F28" s="41">
+        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F16="","",'2 Matériel'!$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="41">
+        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G16="","",'2 Matériel'!$G16)),"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="41">
+        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H16="","",'2 Matériel'!$H16)),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="41">
+        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I16="","",'2 Matériel'!$I16)),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="41">
+        <f>IF(AND('2 Matériel'!$L16&gt;0,NOT('2 Matériel'!$B16="Oui")),IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J16="","",'2 Matériel'!$J16)),"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="42">
         <f>IF(AND('2 Matériel'!$L16&gt;0,'2 Matériel'!$B16="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="21" customHeight="1">
-      <c r="B27" s="13">
+    <row r="29" ht="21" customHeight="1">
+      <c r="B29" s="38">
         <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),'2 Matériel'!$A17,"")</f>
         <v/>
       </c>
-      <c r="C27" s="37">
-        <f>IF('2 Matériel'!$L17&gt;0,IF('2 Matériel'!$B17="Oui",UPPER('2 Matériel'!$C17),'2 Matériel'!$C17),"")</f>
-        <v/>
-      </c>
-      <c r="D27" s="38">
+      <c r="C29" s="39">
+        <f>IF('2 Matériel'!$L17&gt;0,IF('2 Matériel'!$B17="Oui",UPPER('2 Matériel'!$C17),'2 Matériel'!$C17&amp;IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D29" s="40">
         <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),'2 Matériel'!$L17,"")</f>
         <v/>
       </c>
-      <c r="E27" s="39">
-        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E17="","",'2 Matériel'!$E17)),"")</f>
-        <v/>
-      </c>
-      <c r="F27" s="39">
-        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F17="","",'2 Matériel'!$F17)),"")</f>
-        <v/>
-      </c>
-      <c r="G27" s="39">
-        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G17="","",'2 Matériel'!$G17)),"")</f>
-        <v/>
-      </c>
-      <c r="H27" s="39">
-        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H17="","",'2 Matériel'!$H17)),"")</f>
-        <v/>
-      </c>
-      <c r="I27" s="39">
-        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I17="","",'2 Matériel'!$I17)),"")</f>
-        <v/>
-      </c>
-      <c r="J27" s="39">
-        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J17="","",'2 Matériel'!$J17)),"")</f>
-        <v/>
-      </c>
-      <c r="K27" s="40">
-        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="41">
+      <c r="E29" s="41">
+        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E17="","",'2 Matériel'!$E17)),"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="41">
+        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F17="","",'2 Matériel'!$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="41">
+        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G17="","",'2 Matériel'!$G17)),"")</f>
+        <v/>
+      </c>
+      <c r="H29" s="41">
+        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H17="","",'2 Matériel'!$H17)),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="41">
+        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I17="","",'2 Matériel'!$I17)),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="41">
+        <f>IF(AND('2 Matériel'!$L17&gt;0,NOT('2 Matériel'!$B17="Oui")),IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J17="","",'2 Matériel'!$J17)),"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="42">
         <f>IF(AND('2 Matériel'!$L17&gt;0,'2 Matériel'!$B17="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="21" customHeight="1">
-      <c r="B28" s="13">
+    <row r="30" ht="21" customHeight="1">
+      <c r="B30" s="38">
         <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),'2 Matériel'!$A18,"")</f>
         <v/>
       </c>
-      <c r="C28" s="37">
-        <f>IF('2 Matériel'!$L18&gt;0,IF('2 Matériel'!$B18="Oui",UPPER('2 Matériel'!$C18),'2 Matériel'!$C18),"")</f>
-        <v/>
-      </c>
-      <c r="D28" s="38">
+      <c r="C30" s="39">
+        <f>IF('2 Matériel'!$L18&gt;0,IF('2 Matériel'!$B18="Oui",UPPER('2 Matériel'!$C18),'2 Matériel'!$C18&amp;IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D30" s="40">
         <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),'2 Matériel'!$L18,"")</f>
         <v/>
       </c>
-      <c r="E28" s="39">
-        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E18="","",'2 Matériel'!$E18)),"")</f>
-        <v/>
-      </c>
-      <c r="F28" s="39">
-        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F18="","",'2 Matériel'!$F18)),"")</f>
-        <v/>
-      </c>
-      <c r="G28" s="39">
-        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G18="","",'2 Matériel'!$G18)),"")</f>
-        <v/>
-      </c>
-      <c r="H28" s="39">
-        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H18="","",'2 Matériel'!$H18)),"")</f>
-        <v/>
-      </c>
-      <c r="I28" s="39">
-        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I18="","",'2 Matériel'!$I18)),"")</f>
-        <v/>
-      </c>
-      <c r="J28" s="39">
-        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J18="","",'2 Matériel'!$J18)),"")</f>
-        <v/>
-      </c>
-      <c r="K28" s="40">
-        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="41">
+      <c r="E30" s="41">
+        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E18="","",'2 Matériel'!$E18)),"")</f>
+        <v/>
+      </c>
+      <c r="F30" s="41">
+        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F18="","",'2 Matériel'!$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="G30" s="41">
+        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G18="","",'2 Matériel'!$G18)),"")</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H18="","",'2 Matériel'!$H18)),"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="41">
+        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I18="","",'2 Matériel'!$I18)),"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="41">
+        <f>IF(AND('2 Matériel'!$L18&gt;0,NOT('2 Matériel'!$B18="Oui")),IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J18="","",'2 Matériel'!$J18)),"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="42">
         <f>IF(AND('2 Matériel'!$L18&gt;0,'2 Matériel'!$B18="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="29" ht="21" customHeight="1">
-      <c r="B29" s="13">
+    <row r="31" ht="21" customHeight="1">
+      <c r="B31" s="38">
         <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),'2 Matériel'!$A19,"")</f>
         <v/>
       </c>
-      <c r="C29" s="37">
-        <f>IF('2 Matériel'!$L19&gt;0,IF('2 Matériel'!$B19="Oui",UPPER('2 Matériel'!$C19),'2 Matériel'!$C19),"")</f>
-        <v/>
-      </c>
-      <c r="D29" s="38">
+      <c r="C31" s="39">
+        <f>IF('2 Matériel'!$L19&gt;0,IF('2 Matériel'!$B19="Oui",UPPER('2 Matériel'!$C19),'2 Matériel'!$C19&amp;IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D31" s="40">
         <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),'2 Matériel'!$L19,"")</f>
         <v/>
       </c>
-      <c r="E29" s="39">
-        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E19="","",'2 Matériel'!$E19)),"")</f>
-        <v/>
-      </c>
-      <c r="F29" s="39">
-        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F19="","",'2 Matériel'!$F19)),"")</f>
-        <v/>
-      </c>
-      <c r="G29" s="39">
-        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G19="","",'2 Matériel'!$G19)),"")</f>
-        <v/>
-      </c>
-      <c r="H29" s="39">
-        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H19="","",'2 Matériel'!$H19)),"")</f>
-        <v/>
-      </c>
-      <c r="I29" s="39">
-        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I19="","",'2 Matériel'!$I19)),"")</f>
-        <v/>
-      </c>
-      <c r="J29" s="39">
-        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J19="","",'2 Matériel'!$J19)),"")</f>
-        <v/>
-      </c>
-      <c r="K29" s="40">
-        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="41">
+      <c r="E31" s="41">
+        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E19="","",'2 Matériel'!$E19)),"")</f>
+        <v/>
+      </c>
+      <c r="F31" s="41">
+        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F19="","",'2 Matériel'!$F19)),"")</f>
+        <v/>
+      </c>
+      <c r="G31" s="41">
+        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G19="","",'2 Matériel'!$G19)),"")</f>
+        <v/>
+      </c>
+      <c r="H31" s="41">
+        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H19="","",'2 Matériel'!$H19)),"")</f>
+        <v/>
+      </c>
+      <c r="I31" s="41">
+        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I19="","",'2 Matériel'!$I19)),"")</f>
+        <v/>
+      </c>
+      <c r="J31" s="41">
+        <f>IF(AND('2 Matériel'!$L19&gt;0,NOT('2 Matériel'!$B19="Oui")),IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J19="","",'2 Matériel'!$J19)),"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="42">
         <f>IF(AND('2 Matériel'!$L19&gt;0,'2 Matériel'!$B19="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B30" s="13">
+    <row r="32" ht="21" customHeight="1">
+      <c r="B32" s="38">
         <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),'2 Matériel'!$A20,"")</f>
         <v/>
       </c>
-      <c r="C30" s="37">
-        <f>IF('2 Matériel'!$L20&gt;0,IF('2 Matériel'!$B20="Oui",UPPER('2 Matériel'!$C20),'2 Matériel'!$C20),"")</f>
-        <v/>
-      </c>
-      <c r="D30" s="38">
+      <c r="C32" s="39">
+        <f>IF('2 Matériel'!$L20&gt;0,IF('2 Matériel'!$B20="Oui",UPPER('2 Matériel'!$C20),'2 Matériel'!$C20&amp;IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D32" s="40">
         <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),'2 Matériel'!$L20,"")</f>
         <v/>
       </c>
-      <c r="E30" s="39">
-        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E20="","",'2 Matériel'!$E20)),"")</f>
-        <v/>
-      </c>
-      <c r="F30" s="39">
-        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F20="","",'2 Matériel'!$F20)),"")</f>
-        <v/>
-      </c>
-      <c r="G30" s="39">
-        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G20="","",'2 Matériel'!$G20)),"")</f>
-        <v/>
-      </c>
-      <c r="H30" s="39">
-        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H20="","",'2 Matériel'!$H20)),"")</f>
-        <v/>
-      </c>
-      <c r="I30" s="39">
-        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I20="","",'2 Matériel'!$I20)),"")</f>
-        <v/>
-      </c>
-      <c r="J30" s="39">
-        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J20="","",'2 Matériel'!$J20)),"")</f>
-        <v/>
-      </c>
-      <c r="K30" s="40">
-        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="41">
+      <c r="E32" s="41">
+        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E20="","",'2 Matériel'!$E20)),"")</f>
+        <v/>
+      </c>
+      <c r="F32" s="41">
+        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F20="","",'2 Matériel'!$F20)),"")</f>
+        <v/>
+      </c>
+      <c r="G32" s="41">
+        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G20="","",'2 Matériel'!$G20)),"")</f>
+        <v/>
+      </c>
+      <c r="H32" s="41">
+        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H20="","",'2 Matériel'!$H20)),"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="41">
+        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I20="","",'2 Matériel'!$I20)),"")</f>
+        <v/>
+      </c>
+      <c r="J32" s="41">
+        <f>IF(AND('2 Matériel'!$L20&gt;0,NOT('2 Matériel'!$B20="Oui")),IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J20="","",'2 Matériel'!$J20)),"")</f>
+        <v/>
+      </c>
+      <c r="L32" s="42">
         <f>IF(AND('2 Matériel'!$L20&gt;0,'2 Matériel'!$B20="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B31" s="13">
+    <row r="33" ht="21" customHeight="1">
+      <c r="B33" s="38">
         <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),'2 Matériel'!$A21,"")</f>
         <v/>
       </c>
-      <c r="C31" s="37">
-        <f>IF('2 Matériel'!$L21&gt;0,IF('2 Matériel'!$B21="Oui",UPPER('2 Matériel'!$C21),'2 Matériel'!$C21),"")</f>
-        <v/>
-      </c>
-      <c r="D31" s="38">
+      <c r="C33" s="39">
+        <f>IF('2 Matériel'!$L21&gt;0,IF('2 Matériel'!$B21="Oui",UPPER('2 Matériel'!$C21),'2 Matériel'!$C21&amp;IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D33" s="40">
         <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),'2 Matériel'!$L21,"")</f>
         <v/>
       </c>
-      <c r="E31" s="39">
-        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E21="","",'2 Matériel'!$E21)),"")</f>
-        <v/>
-      </c>
-      <c r="F31" s="39">
-        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F21="","",'2 Matériel'!$F21)),"")</f>
-        <v/>
-      </c>
-      <c r="G31" s="39">
-        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G21="","",'2 Matériel'!$G21)),"")</f>
-        <v/>
-      </c>
-      <c r="H31" s="39">
-        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H21="","",'2 Matériel'!$H21)),"")</f>
-        <v/>
-      </c>
-      <c r="I31" s="39">
-        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I21="","",'2 Matériel'!$I21)),"")</f>
-        <v/>
-      </c>
-      <c r="J31" s="39">
-        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J21="","",'2 Matériel'!$J21)),"")</f>
-        <v/>
-      </c>
-      <c r="K31" s="40">
-        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M31" s="41">
+      <c r="E33" s="41">
+        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E21="","",'2 Matériel'!$E21)),"")</f>
+        <v/>
+      </c>
+      <c r="F33" s="41">
+        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F21="","",'2 Matériel'!$F21)),"")</f>
+        <v/>
+      </c>
+      <c r="G33" s="41">
+        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G21="","",'2 Matériel'!$G21)),"")</f>
+        <v/>
+      </c>
+      <c r="H33" s="41">
+        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H21="","",'2 Matériel'!$H21)),"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="41">
+        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I21="","",'2 Matériel'!$I21)),"")</f>
+        <v/>
+      </c>
+      <c r="J33" s="41">
+        <f>IF(AND('2 Matériel'!$L21&gt;0,NOT('2 Matériel'!$B21="Oui")),IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J21="","",'2 Matériel'!$J21)),"")</f>
+        <v/>
+      </c>
+      <c r="L33" s="42">
         <f>IF(AND('2 Matériel'!$L21&gt;0,'2 Matériel'!$B21="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B32" s="13">
+    <row r="34" ht="21" customHeight="1">
+      <c r="B34" s="38">
         <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),'2 Matériel'!$A22,"")</f>
         <v/>
       </c>
-      <c r="C32" s="37">
-        <f>IF('2 Matériel'!$L22&gt;0,IF('2 Matériel'!$B22="Oui",UPPER('2 Matériel'!$C22),'2 Matériel'!$C22),"")</f>
-        <v/>
-      </c>
-      <c r="D32" s="38">
+      <c r="C34" s="39">
+        <f>IF('2 Matériel'!$L22&gt;0,IF('2 Matériel'!$B22="Oui",UPPER('2 Matériel'!$C22),'2 Matériel'!$C22&amp;IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D34" s="40">
         <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),'2 Matériel'!$L22,"")</f>
         <v/>
       </c>
-      <c r="E32" s="39">
-        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E22="","",'2 Matériel'!$E22)),"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="39">
-        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F22="","",'2 Matériel'!$F22)),"")</f>
-        <v/>
-      </c>
-      <c r="G32" s="39">
-        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G22="","",'2 Matériel'!$G22)),"")</f>
-        <v/>
-      </c>
-      <c r="H32" s="39">
-        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H22="","",'2 Matériel'!$H22)),"")</f>
-        <v/>
-      </c>
-      <c r="I32" s="39">
-        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I22="","",'2 Matériel'!$I22)),"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="39">
-        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J22="","",'2 Matériel'!$J22)),"")</f>
-        <v/>
-      </c>
-      <c r="K32" s="40">
-        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="41">
+      <c r="E34" s="41">
+        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E22="","",'2 Matériel'!$E22)),"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="41">
+        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F22="","",'2 Matériel'!$F22)),"")</f>
+        <v/>
+      </c>
+      <c r="G34" s="41">
+        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G22="","",'2 Matériel'!$G22)),"")</f>
+        <v/>
+      </c>
+      <c r="H34" s="41">
+        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H22="","",'2 Matériel'!$H22)),"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="41">
+        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I22="","",'2 Matériel'!$I22)),"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="41">
+        <f>IF(AND('2 Matériel'!$L22&gt;0,NOT('2 Matériel'!$B22="Oui")),IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J22="","",'2 Matériel'!$J22)),"")</f>
+        <v/>
+      </c>
+      <c r="L34" s="42">
         <f>IF(AND('2 Matériel'!$L22&gt;0,'2 Matériel'!$B22="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="33" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B33" s="13">
+    <row r="35" ht="21" customHeight="1">
+      <c r="B35" s="38">
         <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),'2 Matériel'!$A23,"")</f>
         <v/>
       </c>
-      <c r="C33" s="37">
-        <f>IF('2 Matériel'!$L23&gt;0,IF('2 Matériel'!$B23="Oui",UPPER('2 Matériel'!$C23),'2 Matériel'!$C23),"")</f>
-        <v/>
-      </c>
-      <c r="D33" s="38">
+      <c r="C35" s="39">
+        <f>IF('2 Matériel'!$L23&gt;0,IF('2 Matériel'!$B23="Oui",UPPER('2 Matériel'!$C23),'2 Matériel'!$C23&amp;IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D35" s="40">
         <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),'2 Matériel'!$L23,"")</f>
         <v/>
       </c>
-      <c r="E33" s="39">
-        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E23="","",'2 Matériel'!$E23)),"")</f>
-        <v/>
-      </c>
-      <c r="F33" s="39">
-        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F23="","",'2 Matériel'!$F23)),"")</f>
-        <v/>
-      </c>
-      <c r="G33" s="39">
-        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G23="","",'2 Matériel'!$G23)),"")</f>
-        <v/>
-      </c>
-      <c r="H33" s="39">
-        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H23="","",'2 Matériel'!$H23)),"")</f>
-        <v/>
-      </c>
-      <c r="I33" s="39">
-        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I23="","",'2 Matériel'!$I23)),"")</f>
-        <v/>
-      </c>
-      <c r="J33" s="39">
-        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J23="","",'2 Matériel'!$J23)),"")</f>
-        <v/>
-      </c>
-      <c r="K33" s="40">
-        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="41">
+      <c r="E35" s="41">
+        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E23="","",'2 Matériel'!$E23)),"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="41">
+        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F23="","",'2 Matériel'!$F23)),"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="41">
+        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G23="","",'2 Matériel'!$G23)),"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="41">
+        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H23="","",'2 Matériel'!$H23)),"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="41">
+        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I23="","",'2 Matériel'!$I23)),"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="41">
+        <f>IF(AND('2 Matériel'!$L23&gt;0,NOT('2 Matériel'!$B23="Oui")),IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J23="","",'2 Matériel'!$J23)),"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="42">
         <f>IF(AND('2 Matériel'!$L23&gt;0,'2 Matériel'!$B23="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="34" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B34" s="13">
+    <row r="36" hidden="1" outlineLevel="1" ht="21" customHeight="1">
+      <c r="B36" s="38">
         <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),'2 Matériel'!$A24,"")</f>
         <v/>
       </c>
-      <c r="C34" s="37">
-        <f>IF('2 Matériel'!$L24&gt;0,IF('2 Matériel'!$B24="Oui",UPPER('2 Matériel'!$C24),'2 Matériel'!$C24),"")</f>
-        <v/>
-      </c>
-      <c r="D34" s="38">
+      <c r="C36" s="39">
+        <f>IF('2 Matériel'!$L24&gt;0,IF('2 Matériel'!$B24="Oui",UPPER('2 Matériel'!$C24),'2 Matériel'!$C24&amp;IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D36" s="40">
         <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),'2 Matériel'!$L24,"")</f>
         <v/>
       </c>
-      <c r="E34" s="39">
-        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E24="","",'2 Matériel'!$E24)),"")</f>
-        <v/>
-      </c>
-      <c r="F34" s="39">
-        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F24="","",'2 Matériel'!$F24)),"")</f>
-        <v/>
-      </c>
-      <c r="G34" s="39">
-        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G24="","",'2 Matériel'!$G24)),"")</f>
-        <v/>
-      </c>
-      <c r="H34" s="39">
-        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H24="","",'2 Matériel'!$H24)),"")</f>
-        <v/>
-      </c>
-      <c r="I34" s="39">
-        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I24="","",'2 Matériel'!$I24)),"")</f>
-        <v/>
-      </c>
-      <c r="J34" s="39">
-        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J24="","",'2 Matériel'!$J24)),"")</f>
-        <v/>
-      </c>
-      <c r="K34" s="40">
-        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M34" s="41">
+      <c r="E36" s="41">
+        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E24="","",'2 Matériel'!$E24)),"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="41">
+        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F24="","",'2 Matériel'!$F24)),"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="41">
+        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G24="","",'2 Matériel'!$G24)),"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="41">
+        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H24="","",'2 Matériel'!$H24)),"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="41">
+        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I24="","",'2 Matériel'!$I24)),"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="41">
+        <f>IF(AND('2 Matériel'!$L24&gt;0,NOT('2 Matériel'!$B24="Oui")),IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J24="","",'2 Matériel'!$J24)),"")</f>
+        <v/>
+      </c>
+      <c r="L36" s="42">
         <f>IF(AND('2 Matériel'!$L24&gt;0,'2 Matériel'!$B24="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="35" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B35" s="13">
+    <row r="37" hidden="1" outlineLevel="1" ht="21" customHeight="1">
+      <c r="B37" s="38">
         <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),'2 Matériel'!$A25,"")</f>
         <v/>
       </c>
-      <c r="C35" s="37">
-        <f>IF('2 Matériel'!$L25&gt;0,IF('2 Matériel'!$B25="Oui",UPPER('2 Matériel'!$C25),'2 Matériel'!$C25),"")</f>
-        <v/>
-      </c>
-      <c r="D35" s="38">
+      <c r="C37" s="39">
+        <f>IF('2 Matériel'!$L25&gt;0,IF('2 Matériel'!$B25="Oui",UPPER('2 Matériel'!$C25),'2 Matériel'!$C25&amp;IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D37" s="40">
         <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),'2 Matériel'!$L25,"")</f>
         <v/>
       </c>
-      <c r="E35" s="39">
-        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E25="","",'2 Matériel'!$E25)),"")</f>
-        <v/>
-      </c>
-      <c r="F35" s="39">
-        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F25="","",'2 Matériel'!$F25)),"")</f>
-        <v/>
-      </c>
-      <c r="G35" s="39">
-        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G25="","",'2 Matériel'!$G25)),"")</f>
-        <v/>
-      </c>
-      <c r="H35" s="39">
-        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H25="","",'2 Matériel'!$H25)),"")</f>
-        <v/>
-      </c>
-      <c r="I35" s="39">
-        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I25="","",'2 Matériel'!$I25)),"")</f>
-        <v/>
-      </c>
-      <c r="J35" s="39">
-        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J25="","",'2 Matériel'!$J25)),"")</f>
-        <v/>
-      </c>
-      <c r="K35" s="40">
-        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M35" s="41">
+      <c r="E37" s="41">
+        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E25="","",'2 Matériel'!$E25)),"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="41">
+        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F25="","",'2 Matériel'!$F25)),"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="41">
+        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G25="","",'2 Matériel'!$G25)),"")</f>
+        <v/>
+      </c>
+      <c r="H37" s="41">
+        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H25="","",'2 Matériel'!$H25)),"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="41">
+        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I25="","",'2 Matériel'!$I25)),"")</f>
+        <v/>
+      </c>
+      <c r="J37" s="41">
+        <f>IF(AND('2 Matériel'!$L25&gt;0,NOT('2 Matériel'!$B25="Oui")),IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J25="","",'2 Matériel'!$J25)),"")</f>
+        <v/>
+      </c>
+      <c r="L37" s="42">
         <f>IF(AND('2 Matériel'!$L25&gt;0,'2 Matériel'!$B25="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="36" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B36" s="13">
+    <row r="38" hidden="1" outlineLevel="1" ht="21" customHeight="1">
+      <c r="B38" s="38">
         <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),'2 Matériel'!$A26,"")</f>
         <v/>
       </c>
-      <c r="C36" s="37">
-        <f>IF('2 Matériel'!$L26&gt;0,IF('2 Matériel'!$B26="Oui",UPPER('2 Matériel'!$C26),'2 Matériel'!$C26),"")</f>
-        <v/>
-      </c>
-      <c r="D36" s="38">
+      <c r="C38" s="39">
+        <f>IF('2 Matériel'!$L26&gt;0,IF('2 Matériel'!$B26="Oui",UPPER('2 Matériel'!$C26),'2 Matériel'!$C26&amp;IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D38" s="40">
         <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),'2 Matériel'!$L26,"")</f>
         <v/>
       </c>
-      <c r="E36" s="39">
-        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E26="","",'2 Matériel'!$E26)),"")</f>
-        <v/>
-      </c>
-      <c r="F36" s="39">
-        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F26="","",'2 Matériel'!$F26)),"")</f>
-        <v/>
-      </c>
-      <c r="G36" s="39">
-        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G26="","",'2 Matériel'!$G26)),"")</f>
-        <v/>
-      </c>
-      <c r="H36" s="39">
-        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H26="","",'2 Matériel'!$H26)),"")</f>
-        <v/>
-      </c>
-      <c r="I36" s="39">
-        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I26="","",'2 Matériel'!$I26)),"")</f>
-        <v/>
-      </c>
-      <c r="J36" s="39">
-        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J26="","",'2 Matériel'!$J26)),"")</f>
-        <v/>
-      </c>
-      <c r="K36" s="40">
-        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M36" s="41">
+      <c r="E38" s="41">
+        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E26="","",'2 Matériel'!$E26)),"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="41">
+        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F26="","",'2 Matériel'!$F26)),"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="41">
+        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G26="","",'2 Matériel'!$G26)),"")</f>
+        <v/>
+      </c>
+      <c r="H38" s="41">
+        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H26="","",'2 Matériel'!$H26)),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="41">
+        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I26="","",'2 Matériel'!$I26)),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="41">
+        <f>IF(AND('2 Matériel'!$L26&gt;0,NOT('2 Matériel'!$B26="Oui")),IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J26="","",'2 Matériel'!$J26)),"")</f>
+        <v/>
+      </c>
+      <c r="L38" s="42">
         <f>IF(AND('2 Matériel'!$L26&gt;0,'2 Matériel'!$B26="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="37" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B37" s="13">
+    <row r="39" hidden="1" outlineLevel="1" ht="21" customHeight="1">
+      <c r="B39" s="38">
         <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),'2 Matériel'!$A27,"")</f>
         <v/>
       </c>
-      <c r="C37" s="37">
-        <f>IF('2 Matériel'!$L27&gt;0,IF('2 Matériel'!$B27="Oui",UPPER('2 Matériel'!$C27),'2 Matériel'!$C27),"")</f>
-        <v/>
-      </c>
-      <c r="D37" s="38">
+      <c r="C39" s="39">
+        <f>IF('2 Matériel'!$L27&gt;0,IF('2 Matériel'!$B27="Oui",UPPER('2 Matériel'!$C27),'2 Matériel'!$C27&amp;IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D39" s="40">
         <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),'2 Matériel'!$L27,"")</f>
         <v/>
       </c>
-      <c r="E37" s="39">
-        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E27="","",'2 Matériel'!$E27)),"")</f>
-        <v/>
-      </c>
-      <c r="F37" s="39">
-        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F27="","",'2 Matériel'!$F27)),"")</f>
-        <v/>
-      </c>
-      <c r="G37" s="39">
-        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G27="","",'2 Matériel'!$G27)),"")</f>
-        <v/>
-      </c>
-      <c r="H37" s="39">
-        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H27="","",'2 Matériel'!$H27)),"")</f>
-        <v/>
-      </c>
-      <c r="I37" s="39">
-        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I27="","",'2 Matériel'!$I27)),"")</f>
-        <v/>
-      </c>
-      <c r="J37" s="39">
-        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J27="","",'2 Matériel'!$J27)),"")</f>
-        <v/>
-      </c>
-      <c r="K37" s="40">
-        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M37" s="41">
+      <c r="E39" s="41">
+        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E27="","",'2 Matériel'!$E27)),"")</f>
+        <v/>
+      </c>
+      <c r="F39" s="41">
+        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F27="","",'2 Matériel'!$F27)),"")</f>
+        <v/>
+      </c>
+      <c r="G39" s="41">
+        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G27="","",'2 Matériel'!$G27)),"")</f>
+        <v/>
+      </c>
+      <c r="H39" s="41">
+        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H27="","",'2 Matériel'!$H27)),"")</f>
+        <v/>
+      </c>
+      <c r="I39" s="41">
+        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I27="","",'2 Matériel'!$I27)),"")</f>
+        <v/>
+      </c>
+      <c r="J39" s="41">
+        <f>IF(AND('2 Matériel'!$L27&gt;0,NOT('2 Matériel'!$B27="Oui")),IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J27="","",'2 Matériel'!$J27)),"")</f>
+        <v/>
+      </c>
+      <c r="L39" s="42">
         <f>IF(AND('2 Matériel'!$L27&gt;0,'2 Matériel'!$B27="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="38" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B38" s="13">
+    <row r="40" hidden="1" outlineLevel="1" ht="21" customHeight="1">
+      <c r="B40" s="38">
         <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),'2 Matériel'!$A28,"")</f>
         <v/>
       </c>
-      <c r="C38" s="37">
-        <f>IF('2 Matériel'!$L28&gt;0,IF('2 Matériel'!$B28="Oui",UPPER('2 Matériel'!$C28),'2 Matériel'!$C28),"")</f>
-        <v/>
-      </c>
-      <c r="D38" s="38">
+      <c r="C40" s="39">
+        <f>IF('2 Matériel'!$L28&gt;0,IF('2 Matériel'!$B28="Oui",UPPER('2 Matériel'!$C28),'2 Matériel'!$C28&amp;IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D40" s="40">
         <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),'2 Matériel'!$L28,"")</f>
         <v/>
       </c>
-      <c r="E38" s="39">
-        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E28="","",'2 Matériel'!$E28)),"")</f>
-        <v/>
-      </c>
-      <c r="F38" s="39">
-        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F28="","",'2 Matériel'!$F28)),"")</f>
-        <v/>
-      </c>
-      <c r="G38" s="39">
-        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G28="","",'2 Matériel'!$G28)),"")</f>
-        <v/>
-      </c>
-      <c r="H38" s="39">
-        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H28="","",'2 Matériel'!$H28)),"")</f>
-        <v/>
-      </c>
-      <c r="I38" s="39">
-        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I28="","",'2 Matériel'!$I28)),"")</f>
-        <v/>
-      </c>
-      <c r="J38" s="39">
-        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J28="","",'2 Matériel'!$J28)),"")</f>
-        <v/>
-      </c>
-      <c r="K38" s="40">
-        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M38" s="41">
+      <c r="E40" s="41">
+        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E28="","",'2 Matériel'!$E28)),"")</f>
+        <v/>
+      </c>
+      <c r="F40" s="41">
+        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F28="","",'2 Matériel'!$F28)),"")</f>
+        <v/>
+      </c>
+      <c r="G40" s="41">
+        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G28="","",'2 Matériel'!$G28)),"")</f>
+        <v/>
+      </c>
+      <c r="H40" s="41">
+        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H28="","",'2 Matériel'!$H28)),"")</f>
+        <v/>
+      </c>
+      <c r="I40" s="41">
+        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I28="","",'2 Matériel'!$I28)),"")</f>
+        <v/>
+      </c>
+      <c r="J40" s="41">
+        <f>IF(AND('2 Matériel'!$L28&gt;0,NOT('2 Matériel'!$B28="Oui")),IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J28="","",'2 Matériel'!$J28)),"")</f>
+        <v/>
+      </c>
+      <c r="L40" s="42">
         <f>IF(AND('2 Matériel'!$L28&gt;0,'2 Matériel'!$B28="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="39" hidden="1" outlineLevel="1" ht="21" customHeight="1">
-      <c r="B39" s="13">
+    <row r="41" hidden="1" outlineLevel="1" ht="21" customHeight="1">
+      <c r="B41" s="38">
         <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),'2 Matériel'!$A29,"")</f>
         <v/>
       </c>
-      <c r="C39" s="37">
-        <f>IF('2 Matériel'!$L29&gt;0,IF('2 Matériel'!$B29="Oui",UPPER('2 Matériel'!$C29),'2 Matériel'!$C29),"")</f>
-        <v/>
-      </c>
-      <c r="D39" s="38">
+      <c r="C41" s="39">
+        <f>IF('2 Matériel'!$L29&gt;0,IF('2 Matériel'!$B29="Oui",UPPER('2 Matériel'!$C29),'2 Matériel'!$C29&amp;IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")),"")</f>
+        <v/>
+      </c>
+      <c r="D41" s="40">
         <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),'2 Matériel'!$L29,"")</f>
         <v/>
       </c>
-      <c r="E39" s="39">
-        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E29="","",'2 Matériel'!$E29)),"")</f>
-        <v/>
-      </c>
-      <c r="F39" s="39">
-        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F29="","",'2 Matériel'!$F29)),"")</f>
-        <v/>
-      </c>
-      <c r="G39" s="39">
-        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G29="","",'2 Matériel'!$G29)),"")</f>
-        <v/>
-      </c>
-      <c r="H39" s="39">
-        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H29="","",'2 Matériel'!$H29)),"")</f>
-        <v/>
-      </c>
-      <c r="I39" s="39">
-        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I29="","",'2 Matériel'!$I29)),"")</f>
-        <v/>
-      </c>
-      <c r="J39" s="39">
-        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J29="","",'2 Matériel'!$J29)),"")</f>
-        <v/>
-      </c>
-      <c r="K39" s="40">
-        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),"")</f>
-        <v/>
-      </c>
-      <c r="M39" s="41">
+      <c r="E41" s="41">
+        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E29="","",'2 Matériel'!$E29)),"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="41">
+        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F29="","",'2 Matériel'!$F29)),"")</f>
+        <v/>
+      </c>
+      <c r="G41" s="41">
+        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G29="","",'2 Matériel'!$G29)),"")</f>
+        <v/>
+      </c>
+      <c r="H41" s="41">
+        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H29="","",'2 Matériel'!$H29)),"")</f>
+        <v/>
+      </c>
+      <c r="I41" s="41">
+        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I29="","",'2 Matériel'!$I29)),"")</f>
+        <v/>
+      </c>
+      <c r="J41" s="41">
+        <f>IF(AND('2 Matériel'!$L29&gt;0,NOT('2 Matériel'!$B29="Oui")),IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J29="","",'2 Matériel'!$J29)),"")</f>
+        <v/>
+      </c>
+      <c r="L41" s="42">
         <f>IF(AND('2 Matériel'!$L29&gt;0,'2 Matériel'!$B29="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="B40" s="42">
-        <f>IF(SUM('2 Matériel'!$L$20:$L$29)&gt;0,"⚠  Des lignes de matériel au-delà de la ligne 14 sont masquées : cliquer sur le [+] dans la marge gauche pour les afficher.","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="8" customHeight="1"/>
-    <row r="42" ht="20" customHeight="1">
+    <row r="42" ht="18" customHeight="1">
       <c r="B42" s="43">
+        <f>IF(SUM('2 Matériel'!$L$24:$L$29)&gt;0,"⚠  Des lignes de matériel au-delà de la ligne 18 sont masquées : cliquer sur le [+] dans la marge gauche pour les afficher.","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="8" customHeight="1"/>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="44">
         <f>IF('3 Options'!$C$8="Oui",INDEX(Textes!$B$2:$C$55,MATCH("sec_tight",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="C42" s="44" t="n"/>
-      <c r="D42" s="44">
+      <c r="C44" s="45" t="n"/>
+      <c r="D44" s="45">
         <f>IF('3 Options'!$C$8="Oui",INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="E42" s="44">
+      <c r="E44" s="46">
         <f>IF('3 Options'!$C$8="Oui",INDEX(Textes!$B$2:$C$55,MATCH("h_unit",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="F42" s="44">
+      <c r="F44" s="46">
         <f>IF('3 Options'!$C$8="Oui",INDEX(Textes!$B$2:$C$55,MATCH("h_pu",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="G42" s="44">
+      <c r="G44" s="45">
         <f>IF('3 Options'!$C$8="Oui",INDEX(Textes!$B$2:$C$55,MATCH("h_tot",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="H42" s="43">
+      <c r="H44" s="44">
         <f>IF('3 Options'!$C$8="Oui",INDEX(Textes!$B$2:$C$55,MATCH("h_det",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="M42" s="41">
+      <c r="I44" s="45" t="n"/>
+      <c r="J44" s="45" t="n"/>
+      <c r="L44" s="42">
         <f>IF('3 Options'!$C$8="Oui",1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="43" ht="21" customHeight="1">
-      <c r="C43" s="45">
+    <row r="45" ht="21" customHeight="1">
+      <c r="C45" s="47">
         <f>IF('3 Options'!$C$8="Oui",IF('3 Options'!$D$8&lt;&gt;"",'3 Options'!$D$8,INDEX(Textes!$B$2:$C$55,MATCH("tight",Textes!$A$2:$A$55,0),Listes!$H$1)),"")</f>
         <v/>
       </c>
-      <c r="D43" s="38">
+      <c r="D45" s="48">
         <f>IF('3 Options'!$C$8="Oui",IF('3 Options'!$G$8="Coût réel +15 %","",'3 Options'!$E$8),"")</f>
         <v/>
       </c>
-      <c r="E43" s="38">
+      <c r="E45" s="49">
         <f>IF('3 Options'!$C$8="Oui",IF('3 Options'!$G$8="Coût réel +15 %","",'3 Options'!$G$8),"")</f>
         <v/>
       </c>
-      <c r="F43" s="39">
+      <c r="F45" s="50">
         <f>IF('3 Options'!$C$8="Oui",IF('3 Options'!$G$8="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$8="","",'3 Options'!$F$8)),"")</f>
         <v/>
       </c>
-      <c r="G43" s="46">
+      <c r="G45" s="51">
         <f>IF('3 Options'!$C$8="Oui",IF('3 Options'!$G$8="Coût réel +15 %","—",'3 Options'!$H$8),"")</f>
         <v/>
       </c>
-      <c r="H43" s="47">
+      <c r="H45" s="52">
         <f>""</f>
         <v/>
       </c>
     </row>
-    <row r="44" ht="8" customHeight="1"/>
-    <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="43">
+    <row r="46" ht="8" customHeight="1"/>
+    <row r="47" ht="20" customHeight="1">
+      <c r="B47" s="44">
         <f>IF(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("sec_tr",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="C45" s="44" t="n"/>
-      <c r="D45" s="44">
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45">
         <f>IF(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="E45" s="44">
+      <c r="E47" s="46">
         <f>IF(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_unit",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="F45" s="44">
+      <c r="F47" s="46">
         <f>IF(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_pu",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="G45" s="44">
+      <c r="G47" s="45">
         <f>IF(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_tot",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="H45" s="43">
+      <c r="H47" s="44">
         <f>IF(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_det",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="M45" s="41">
+      <c r="I47" s="45" t="n"/>
+      <c r="J47" s="45" t="n"/>
+      <c r="L47" s="42">
         <f>IF(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="46" ht="21" customHeight="1">
-      <c r="C46" s="45">
+    <row r="48" ht="21" customHeight="1">
+      <c r="C48" s="47">
         <f>IF('3 Options'!$C$9="Oui",IF('3 Options'!$D$9&lt;&gt;"",'3 Options'!$D$9,INDEX(Textes!$B$2:$C$55,MATCH("tr_mob",Textes!$A$2:$A$55,0),Listes!$H$1)),"")</f>
         <v/>
       </c>
-      <c r="D46" s="38">
+      <c r="D48" s="48">
         <f>IF('3 Options'!$C$9="Oui",IF('3 Options'!$G$9="Coût réel +15 %","",'3 Options'!$E$9),"")</f>
         <v/>
       </c>
-      <c r="E46" s="38">
+      <c r="E48" s="49">
         <f>IF('3 Options'!$C$9="Oui",IF('3 Options'!$G$9="Coût réel +15 %","",'3 Options'!$G$9),"")</f>
         <v/>
       </c>
-      <c r="F46" s="39">
+      <c r="F48" s="50">
         <f>IF('3 Options'!$C$9="Oui",IF('3 Options'!$G$9="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$9="","",'3 Options'!$F$9)),"")</f>
         <v/>
       </c>
-      <c r="G46" s="46">
+      <c r="G48" s="51">
         <f>IF('3 Options'!$C$9="Oui",IF('3 Options'!$G$9="Coût réel +15 %","—",'3 Options'!$H$9),"")</f>
         <v/>
       </c>
-      <c r="H46" s="47">
+      <c r="H48" s="52">
         <f>IF('3 Options'!$C$9="Oui",INDEX(Textes!$B$2:$C$55,MATCH("tr_note",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
     </row>
-    <row r="47" ht="21" customHeight="1">
-      <c r="C47" s="45">
+    <row r="49" ht="21" customHeight="1">
+      <c r="C49" s="47">
         <f>IF('3 Options'!$C$10="Oui",IF('3 Options'!$D$10&lt;&gt;"",'3 Options'!$D$10,INDEX(Textes!$B$2:$C$55,MATCH("tr_dem",Textes!$A$2:$A$55,0),Listes!$H$1)),"")</f>
         <v/>
       </c>
-      <c r="D47" s="38">
+      <c r="D49" s="48">
         <f>IF('3 Options'!$C$10="Oui",IF('3 Options'!$G$10="Coût réel +15 %","",'3 Options'!$E$10),"")</f>
         <v/>
       </c>
-      <c r="E47" s="38">
+      <c r="E49" s="49">
         <f>IF('3 Options'!$C$10="Oui",IF('3 Options'!$G$10="Coût réel +15 %","",'3 Options'!$G$10),"")</f>
         <v/>
       </c>
-      <c r="F47" s="39">
+      <c r="F49" s="50">
         <f>IF('3 Options'!$C$10="Oui",IF('3 Options'!$G$10="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$10="","",'3 Options'!$F$10)),"")</f>
         <v/>
       </c>
-      <c r="G47" s="46">
+      <c r="G49" s="51">
         <f>IF('3 Options'!$C$10="Oui",IF('3 Options'!$G$10="Coût réel +15 %","—",'3 Options'!$H$10),"")</f>
         <v/>
       </c>
-      <c r="H47" s="47">
+      <c r="H49" s="52">
         <f>IF('3 Options'!$C$10="Oui",INDEX(Textes!$B$2:$C$55,MATCH("tr_note",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
     </row>
-    <row r="48" ht="8" customHeight="1"/>
-    <row r="49" ht="20" customHeight="1">
-      <c r="B49" s="43">
+    <row r="50" ht="8" customHeight="1"/>
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="44">
         <f>IF(OR('3 Options'!$C$6="Oui",'3 Options'!$C$7="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("sec_op",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="C49" s="44" t="n"/>
-      <c r="D49" s="44">
+      <c r="C51" s="45" t="n"/>
+      <c r="D51" s="45">
         <f>IF(OR('3 Options'!$C$6="Oui",'3 Options'!$C$7="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="E49" s="44">
+      <c r="E51" s="46">
         <f>IF(OR('3 Options'!$C$6="Oui",'3 Options'!$C$7="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_unit",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="F49" s="44">
+      <c r="F51" s="46">
         <f>IF(OR('3 Options'!$C$6="Oui",'3 Options'!$C$7="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_pu",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="G49" s="44">
+      <c r="G51" s="45">
         <f>IF(OR('3 Options'!$C$6="Oui",'3 Options'!$C$7="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_tot",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="H49" s="43">
+      <c r="H51" s="44">
         <f>IF(OR('3 Options'!$C$6="Oui",'3 Options'!$C$7="Oui"),INDEX(Textes!$B$2:$C$55,MATCH("h_det",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
         <v/>
       </c>
-      <c r="M49" s="41">
+      <c r="I51" s="45" t="n"/>
+      <c r="J51" s="45" t="n"/>
+      <c r="L51" s="42">
         <f>IF(OR('3 Options'!$C$6="Oui",'3 Options'!$C$7="Oui"),1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="50" ht="21" customHeight="1">
-      <c r="C50" s="45">
+    <row r="52" ht="21" customHeight="1">
+      <c r="C52" s="47">
         <f>IF('3 Options'!$C$6="Oui",IF('3 Options'!$D$6&lt;&gt;"",'3 Options'!$D$6,INDEX(Textes!$B$2:$C$55,MATCH("op_day",Textes!$A$2:$A$55,0),Listes!$H$1)),"")</f>
         <v/>
       </c>
-      <c r="D50" s="38">
+      <c r="D52" s="48">
         <f>IF('3 Options'!$C$6="Oui",IF('3 Options'!$G$6="Coût réel +15 %","",'3 Options'!$E$6),"")</f>
         <v/>
       </c>
-      <c r="E50" s="38">
+      <c r="E52" s="49">
         <f>IF('3 Options'!$C$6="Oui",IF('3 Options'!$G$6="Coût réel +15 %","",'3 Options'!$G$6),"")</f>
         <v/>
       </c>
-      <c r="F50" s="39">
+      <c r="F52" s="50">
         <f>IF('3 Options'!$C$6="Oui",IF('3 Options'!$G$6="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$6="","",'3 Options'!$F$6)),"")</f>
         <v/>
       </c>
-      <c r="G50" s="46">
+      <c r="G52" s="51">
         <f>IF('3 Options'!$C$6="Oui",IF('3 Options'!$G$6="Coût réel +15 %","—",'3 Options'!$H$6),"")</f>
         <v/>
       </c>
-      <c r="H50" s="47">
+      <c r="H52" s="52">
         <f>""</f>
         <v/>
       </c>
     </row>
-    <row r="51" ht="21" customHeight="1">
-      <c r="C51" s="45">
+    <row r="53" ht="21" customHeight="1">
+      <c r="C53" s="47">
         <f>IF('3 Options'!$C$7="Oui",IF('3 Options'!$D$7&lt;&gt;"",'3 Options'!$D$7,INDEX(Textes!$B$2:$C$55,MATCH("op_mob",Textes!$A$2:$A$55,0),Listes!$H$1)),"")</f>
         <v/>
       </c>
-      <c r="D51" s="38">
+      <c r="D53" s="48">
         <f>IF('3 Options'!$C$7="Oui",IF('3 Options'!$G$7="Coût réel +15 %","",'3 Options'!$E$7),"")</f>
         <v/>
       </c>
-      <c r="E51" s="38">
+      <c r="E53" s="49">
         <f>IF('3 Options'!$C$7="Oui",IF('3 Options'!$G$7="Coût réel +15 %","",'3 Options'!$G$7),"")</f>
         <v/>
       </c>
-      <c r="F51" s="39">
+      <c r="F53" s="50">
         <f>IF('3 Options'!$C$7="Oui",IF('3 Options'!$G$7="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$7="","",'3 Options'!$F$7)),"")</f>
         <v/>
       </c>
-      <c r="G51" s="46">
+      <c r="G53" s="51">
         <f>IF('3 Options'!$C$7="Oui",IF('3 Options'!$G$7="Coût réel +15 %","—",'3 Options'!$H$7),"")</f>
         <v/>
       </c>
-      <c r="H51" s="47">
+      <c r="H53" s="52">
         <f>""</f>
         <v/>
       </c>
     </row>
-    <row r="52" ht="8" customHeight="1"/>
-    <row r="53" ht="40" customHeight="1">
-      <c r="B53" s="48">
+    <row r="54" ht="8" customHeight="1"/>
+    <row r="55" ht="42" customHeight="1">
+      <c r="B55" s="53">
         <f>IF('3 Options'!$C$13="Oui",UPPER(INDEX(Textes!$B$2:$C$55,MATCH("forfait",Textes!$A$2:$A$55,0),Listes!$H$1))&amp;IF('3 Options'!$D$13&lt;&gt;"","   ·   "&amp;'3 Options'!$D$13,""),"")</f>
         <v/>
       </c>
-      <c r="I53" s="49">
+      <c r="H55" s="54">
         <f>IF('3 Options'!$C$13="Oui",'3 Options'!$H$13,"")</f>
         <v/>
       </c>
-      <c r="M53" s="41">
+      <c r="L55" s="42">
         <f>IF('3 Options'!$C$13="Oui",1,0)</f>
         <v/>
       </c>
     </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="B54" s="50">
+    <row r="56" ht="34" customHeight="1">
+      <c r="B56" s="55">
         <f>IF('3 Options'!$C$13="Oui",IF('3 Options'!$G$13="Forfait calculé (S + O + UC)",'3 Options'!$C$15&amp;" "&amp;SUBSTITUTE(INDEX(Textes!$B$2:$C$55,MATCH("calc_det",Textes!$A$2:$A$55,0),Listes!$H$1),"%s",'3 Options'!$C$16)&amp;"   ·   "&amp;INDEX(Textes!$B$2:$C$55,MATCH("ht",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13&amp;" j × "&amp;TEXT('3 Options'!$F$13,"#,##0.00")&amp;" €/j   ·   "&amp;INDEX(Textes!$B$2:$C$55,MATCH("ht",Textes!$A$2:$A$55,0),Listes!$H$1),INDEX(Textes!$B$2:$C$55,MATCH("ht",Textes!$A$2:$A$55,0),Listes!$H$1)))&amp;IF('3 Options'!$D$14&lt;&gt;"","   ·   "&amp;'3 Options'!$D$14,""),"")</f>
         <v/>
       </c>
     </row>
-    <row r="55" ht="10" customHeight="1"/>
-    <row r="56" ht="20" customHeight="1">
-      <c r="B56" s="33">
+    <row r="57" ht="10" customHeight="1"/>
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="34">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("sec_cond",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="C56" s="34" t="n"/>
-      <c r="D56" s="34" t="n"/>
-      <c r="E56" s="34" t="n"/>
-      <c r="F56" s="34" t="n"/>
-      <c r="G56" s="34" t="n"/>
-      <c r="H56" s="34" t="n"/>
-      <c r="I56" s="34" t="n"/>
-      <c r="J56" s="34" t="n"/>
-      <c r="K56" s="34" t="n"/>
-    </row>
-    <row r="57" ht="66" customHeight="1">
-      <c r="B57" s="51" t="inlineStr">
+      <c r="C58" s="35" t="n"/>
+      <c r="D58" s="35" t="n"/>
+      <c r="E58" s="35" t="n"/>
+      <c r="F58" s="35" t="n"/>
+      <c r="G58" s="35" t="n"/>
+      <c r="H58" s="35" t="n"/>
+      <c r="I58" s="35" t="n"/>
+      <c r="J58" s="35" t="n"/>
+    </row>
+    <row r="59" ht="76" customHeight="1">
+      <c r="B59" s="56" t="inlineStr">
         <is>
           <t>La location s'entend depuis le jour de départ de la base d'origine jusqu'à son retour au même endroit.
 Le Wear Charge s'applique pour toute usure liée à un usage normal des équipements. En cas de dommages plus importants liés à un usage anormal, la valeur de remplacement sera facturée sur documentation.
@@ -4083,8 +4041,8 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="66" customHeight="1">
-      <c r="B58" s="51" t="inlineStr">
+    <row r="60" ht="76" customHeight="1">
+      <c r="B60" s="56" t="inlineStr">
         <is>
           <t>The rental is from the day of departure from the base of origin until its return to the same place.
 Wear Charge applies to all wear and tear related to normal use of equipment. In case of greater damage due to abnormal use, the replacement value will be charged based on supporting documentation.
@@ -4093,72 +4051,68 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="10" customHeight="1"/>
-    <row r="60">
-      <c r="B60" s="52">
+    <row r="61" ht="10" customHeight="1"/>
+    <row r="62">
+      <c r="B62" s="57">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("accept",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
     </row>
-    <row r="61" ht="16" customHeight="1">
-      <c r="B61" s="53">
+    <row r="63" ht="17" customHeight="1">
+      <c r="B63" s="58">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("sig_name",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="C61" s="54" t="n"/>
-      <c r="D61" s="55" t="n"/>
-      <c r="E61" s="53">
+      <c r="C63" s="59" t="n"/>
+      <c r="D63" s="58">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("sig_date",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="F61" s="54" t="n"/>
-      <c r="G61" s="55" t="n"/>
-      <c r="H61" s="53">
+      <c r="E63" s="60" t="n"/>
+      <c r="F63" s="60" t="n"/>
+      <c r="G63" s="59" t="n"/>
+      <c r="H63" s="58">
         <f>INDEX(Textes!$B$2:$C$55,MATCH("sig_sig",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="I61" s="54" t="n"/>
-      <c r="J61" s="54" t="n"/>
-      <c r="K61" s="55" t="n"/>
-    </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="B62" s="56" t="n"/>
-      <c r="C62" s="57" t="n"/>
-      <c r="D62" s="58" t="n"/>
-      <c r="E62" s="56" t="n"/>
-      <c r="F62" s="57" t="n"/>
-      <c r="G62" s="58" t="n"/>
-      <c r="H62" s="56" t="n"/>
-      <c r="I62" s="57" t="n"/>
-      <c r="J62" s="57" t="n"/>
-      <c r="K62" s="58" t="n"/>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="B63" s="56" t="n"/>
-      <c r="C63" s="57" t="n"/>
-      <c r="D63" s="58" t="n"/>
-      <c r="E63" s="56" t="n"/>
-      <c r="F63" s="57" t="n"/>
-      <c r="G63" s="58" t="n"/>
-      <c r="H63" s="56" t="n"/>
-      <c r="I63" s="57" t="n"/>
-      <c r="J63" s="57" t="n"/>
-      <c r="K63" s="58" t="n"/>
-    </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="B64" s="59" t="n"/>
-      <c r="C64" s="32" t="n"/>
-      <c r="D64" s="60" t="n"/>
-      <c r="E64" s="59" t="n"/>
-      <c r="F64" s="32" t="n"/>
-      <c r="G64" s="60" t="n"/>
-      <c r="H64" s="59" t="n"/>
-      <c r="I64" s="32" t="n"/>
-      <c r="J64" s="32" t="n"/>
-      <c r="K64" s="60" t="n"/>
-    </row>
-    <row r="66">
-      <c r="B66" s="61" t="inlineStr">
+      <c r="I63" s="60" t="n"/>
+      <c r="J63" s="59" t="n"/>
+    </row>
+    <row r="64" ht="17" customHeight="1">
+      <c r="B64" s="61" t="n"/>
+      <c r="C64" s="62" t="n"/>
+      <c r="D64" s="61" t="n"/>
+      <c r="E64" s="63" t="n"/>
+      <c r="F64" s="63" t="n"/>
+      <c r="G64" s="62" t="n"/>
+      <c r="H64" s="61" t="n"/>
+      <c r="I64" s="63" t="n"/>
+      <c r="J64" s="62" t="n"/>
+    </row>
+    <row r="65" ht="17" customHeight="1">
+      <c r="B65" s="61" t="n"/>
+      <c r="C65" s="62" t="n"/>
+      <c r="D65" s="61" t="n"/>
+      <c r="E65" s="63" t="n"/>
+      <c r="F65" s="63" t="n"/>
+      <c r="G65" s="62" t="n"/>
+      <c r="H65" s="61" t="n"/>
+      <c r="I65" s="63" t="n"/>
+      <c r="J65" s="62" t="n"/>
+    </row>
+    <row r="66" ht="17" customHeight="1">
+      <c r="B66" s="64" t="n"/>
+      <c r="C66" s="65" t="n"/>
+      <c r="D66" s="64" t="n"/>
+      <c r="E66" s="33" t="n"/>
+      <c r="F66" s="33" t="n"/>
+      <c r="G66" s="65" t="n"/>
+      <c r="H66" s="64" t="n"/>
+      <c r="I66" s="33" t="n"/>
+      <c r="J66" s="65" t="n"/>
+    </row>
+    <row r="68" ht="26" customHeight="1">
+      <c r="B68" s="66" t="inlineStr">
         <is>
           <t>ENEDRIL · Z-Induspal · 3 Av. des Lacs · 64140 LONS (France) · SIRET 79464246200020 · TVA FR11794642462</t>
         </is>
@@ -4166,128 +4120,128 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="H49:J49"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="H51:J51"/>
+    <mergeCell ref="D9:G9"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B40:K40"/>
-    <mergeCell ref="H47:K47"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="H42:K42"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="B42:J42"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H52:J52"/>
+    <mergeCell ref="B60:J60"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H45:J45"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G7:H7"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="H61:K64"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="B54:K54"/>
-    <mergeCell ref="H43:K43"/>
-    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="H63:J66"/>
+    <mergeCell ref="H47:J47"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="D1:J1"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B66:K66"/>
-    <mergeCell ref="H50:K50"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="B56:K56"/>
-    <mergeCell ref="B58:K58"/>
+    <mergeCell ref="H48:J48"/>
+    <mergeCell ref="B68:J68"/>
+    <mergeCell ref="B55:G55"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="H5:J5"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="B61:D64"/>
-    <mergeCell ref="H46:K46"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="B63:C66"/>
+    <mergeCell ref="D2:J2"/>
+    <mergeCell ref="D11:G11"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E1:K1"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="H49:K49"/>
-    <mergeCell ref="H51:K51"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="B60:K60"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="B62:J62"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B57:K57"/>
-    <mergeCell ref="B14:K14"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="B59:J59"/>
+    <mergeCell ref="H44:J44"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B53:H53"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="H45:K45"/>
-    <mergeCell ref="E61:G64"/>
-    <mergeCell ref="E2:K2"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="H55:J55"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="B56:J56"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="B58:J58"/>
+    <mergeCell ref="D63:G66"/>
+    <mergeCell ref="H6:J6"/>
   </mergeCells>
-  <conditionalFormatting sqref="B16:K39">
+  <conditionalFormatting sqref="B18:J41">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
-      <formula>$M16=1</formula>
+      <formula>$L18=1</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="2">
-      <formula>$C16&lt;&gt;""</formula>
+      <formula>$C18&lt;&gt;""</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="3">
-      <formula>AND($C16&lt;&gt;"",MOD(ROW(),2)=0)</formula>
+      <formula>AND($C18&lt;&gt;"",MOD(ROW(),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E16:J39">
+  <conditionalFormatting sqref="E18:J41">
     <cfRule type="expression" priority="4" dxfId="4">
-      <formula>E16="incl."</formula>
+      <formula>E18="incl."</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B42:K42">
+  <conditionalFormatting sqref="B44:J44">
     <cfRule type="expression" priority="5" dxfId="5">
-      <formula>$M42=1</formula>
+      <formula>$L44=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43:K43">
+  <conditionalFormatting sqref="B45:J45">
     <cfRule type="expression" priority="6" dxfId="2">
-      <formula>$C43&lt;&gt;""</formula>
+      <formula>$C45&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45:K45">
+  <conditionalFormatting sqref="B47:J47">
     <cfRule type="expression" priority="7" dxfId="5">
-      <formula>$M45=1</formula>
+      <formula>$L47=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B46:K46">
+  <conditionalFormatting sqref="B48:J48">
     <cfRule type="expression" priority="8" dxfId="2">
-      <formula>$C46&lt;&gt;""</formula>
+      <formula>$C48&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B47:K47">
+  <conditionalFormatting sqref="B49:J49">
     <cfRule type="expression" priority="9" dxfId="2">
-      <formula>$C47&lt;&gt;""</formula>
+      <formula>$C49&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B49:K49">
+  <conditionalFormatting sqref="B51:J51">
     <cfRule type="expression" priority="10" dxfId="5">
-      <formula>$M49=1</formula>
+      <formula>$L51=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B50:K50">
+  <conditionalFormatting sqref="B52:J52">
     <cfRule type="expression" priority="11" dxfId="2">
-      <formula>$C50&lt;&gt;""</formula>
+      <formula>$C52&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B51:K51">
+  <conditionalFormatting sqref="B53:J53">
     <cfRule type="expression" priority="12" dxfId="2">
-      <formula>$C51&lt;&gt;""</formula>
+      <formula>$C53&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B53:K53">
+  <conditionalFormatting sqref="B55:J55">
     <cfRule type="expression" priority="13" dxfId="6">
-      <formula>$M$53=1</formula>
+      <formula>$L55=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B54:K54">
+  <conditionalFormatting sqref="B56:J56">
     <cfRule type="expression" priority="14" dxfId="7">
-      <formula>$M$53=1</formula>
+      <formula>$L55=1</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.35" right="0.35" top="0.4" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 Enedril · Devis &amp;P / &amp;N</oddFooter>
@@ -4297,7 +4251,7 @@
     <firstFooter/>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="40" min="0" max="16383" man="1"/>
+    <brk id="42" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -4329,366 +4283,366 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>Contact Enedril</t>
         </is>
       </c>
-      <c r="B1" s="62" t="inlineStr">
+      <c r="B1" s="67" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="D1" s="62" t="inlineStr">
+      <c r="D1" s="67" t="inlineStr">
         <is>
           <t>Incoterm</t>
         </is>
       </c>
-      <c r="E1" s="62" t="inlineStr">
+      <c r="E1" s="67" t="inlineStr">
         <is>
           <t>Validité</t>
         </is>
       </c>
-      <c r="F1" s="62" t="inlineStr">
+      <c r="F1" s="67" t="inlineStr">
         <is>
           <t>Règlement</t>
         </is>
       </c>
-      <c r="G1" s="62" t="inlineStr">
+      <c r="G1" s="67" t="inlineStr">
         <is>
           <t>Oui / Non</t>
         </is>
       </c>
-      <c r="H1" s="63" t="n">
+      <c r="H1" s="68" t="n">
         <v>1</v>
       </c>
-      <c r="J1" s="62" t="inlineStr">
+      <c r="J1" s="67" t="inlineStr">
         <is>
           <t>Support de colisage</t>
         </is>
       </c>
-      <c r="K1" s="62" t="inlineStr">
+      <c r="K1" s="67" t="inlineStr">
         <is>
           <t>N° de colis</t>
         </is>
       </c>
-      <c r="L1" s="62" t="inlineStr">
+      <c r="L1" s="67" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="M1" s="62" t="inlineStr">
+      <c r="M1" s="67" t="inlineStr">
         <is>
           <t>Mode transport</t>
         </is>
       </c>
-      <c r="N1" s="62" t="inlineStr">
+      <c r="N1" s="67" t="inlineStr">
         <is>
           <t>Mode forfait</t>
         </is>
       </c>
-      <c r="P1" s="62" t="inlineStr">
+      <c r="P1" s="67" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="Q1" s="62" t="inlineStr">
+      <c r="Q1" s="67" t="inlineStr">
         <is>
           <t>Test / Taille</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="64" t="inlineStr">
+      <c r="A2" s="69" t="inlineStr">
         <is>
           <t>Fabien JACQUOT</t>
         </is>
       </c>
-      <c r="B2" s="64" t="inlineStr">
+      <c r="B2" s="69" t="inlineStr">
         <is>
           <t>fjacquot@enedril.fr</t>
         </is>
       </c>
-      <c r="D2" s="64" t="inlineStr">
+      <c r="D2" s="69" t="inlineStr">
         <is>
           <t>EXW Lons</t>
         </is>
       </c>
-      <c r="E2" s="64" t="inlineStr">
+      <c r="E2" s="69" t="inlineStr">
         <is>
           <t>15 jours / 15 days</t>
         </is>
       </c>
-      <c r="F2" s="64" t="inlineStr">
+      <c r="F2" s="69" t="inlineStr">
         <is>
           <t>30 jours date de facture / 30 days invoice date</t>
         </is>
       </c>
-      <c r="G2" s="64" t="inlineStr">
+      <c r="G2" s="69" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="H2" s="65" t="inlineStr">
+      <c r="H2" s="70" t="inlineStr">
         <is>
           <t>← langue du devis : 1 = français, 2 = anglais</t>
         </is>
       </c>
-      <c r="J2" s="64" t="inlineStr">
+      <c r="J2" s="69" t="inlineStr">
         <is>
           <t>Palette</t>
         </is>
       </c>
-      <c r="K2" s="64" t="inlineStr">
+      <c r="K2" s="69" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="L2" s="64" t="inlineStr">
+      <c r="L2" s="69" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="M2" s="64" t="inlineStr">
+      <c r="M2" s="69" t="inlineStr">
         <is>
           <t>Coût réel +15 %</t>
         </is>
       </c>
-      <c r="N2" s="64" t="inlineStr">
+      <c r="N2" s="69" t="inlineStr">
         <is>
           <t>Forfait calculé (S + O + UC)</t>
         </is>
       </c>
-      <c r="P2" s="64" t="inlineStr">
+      <c r="P2" s="69" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="Q2" s="64" t="inlineStr">
+      <c r="Q2" s="69" t="inlineStr">
         <is>
           <t>Taille OK</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="64" t="inlineStr">
+      <c r="A3" s="69" t="inlineStr">
         <is>
           <t>Alexis ESTINES</t>
         </is>
       </c>
-      <c r="B3" s="64" t="inlineStr">
+      <c r="B3" s="69" t="inlineStr">
         <is>
           <t>aestines@enedril.fr</t>
         </is>
       </c>
-      <c r="D3" s="64" t="inlineStr">
+      <c r="D3" s="69" t="inlineStr">
         <is>
           <t>FCA Lons</t>
         </is>
       </c>
-      <c r="E3" s="64" t="inlineStr">
+      <c r="E3" s="69" t="inlineStr">
         <is>
           <t>30 jours / 30 days</t>
         </is>
       </c>
-      <c r="F3" s="64" t="inlineStr">
+      <c r="F3" s="69" t="inlineStr">
         <is>
           <t>30 jours fin de mois / 30 days end of month</t>
         </is>
       </c>
-      <c r="G3" s="64" t="inlineStr">
+      <c r="G3" s="69" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="J3" s="64" t="inlineStr">
+      <c r="J3" s="69" t="inlineStr">
         <is>
           <t>Fishing basket</t>
         </is>
       </c>
-      <c r="K3" s="64" t="inlineStr">
+      <c r="K3" s="69" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="L3" s="64" t="inlineStr">
+      <c r="L3" s="69" t="inlineStr">
         <is>
           <t>€/jour</t>
         </is>
       </c>
-      <c r="M3" s="64" t="inlineStr">
+      <c r="M3" s="69" t="inlineStr">
         <is>
           <t>Forfait</t>
         </is>
       </c>
-      <c r="N3" s="64" t="inlineStr">
+      <c r="N3" s="69" t="inlineStr">
         <is>
           <t>Forfait global</t>
         </is>
       </c>
-      <c r="P3" s="64" t="inlineStr">
+      <c r="P3" s="69" t="inlineStr">
         <is>
           <t>En cours</t>
         </is>
       </c>
-      <c r="Q3" s="64" t="inlineStr">
+      <c r="Q3" s="69" t="inlineStr">
         <is>
           <t>Test OK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="64" t="inlineStr">
+      <c r="A4" s="69" t="inlineStr">
         <is>
           <t>Paul HYNDERICK</t>
         </is>
       </c>
-      <c r="B4" s="64" t="inlineStr">
+      <c r="B4" s="69" t="inlineStr">
         <is>
           <t>phynderick@enedril.fr</t>
         </is>
       </c>
-      <c r="D4" s="64" t="inlineStr">
+      <c r="D4" s="69" t="inlineStr">
         <is>
           <t>DAP</t>
         </is>
       </c>
-      <c r="E4" s="64" t="inlineStr">
+      <c r="E4" s="69" t="inlineStr">
         <is>
           <t>60 jours / 60 days</t>
         </is>
       </c>
-      <c r="F4" s="64" t="inlineStr">
+      <c r="F4" s="69" t="inlineStr">
         <is>
           <t>45 jours fin de mois / 45 days end of month</t>
         </is>
       </c>
-      <c r="J4" s="64" t="inlineStr">
+      <c r="J4" s="69" t="inlineStr">
         <is>
           <t>Caisse</t>
         </is>
       </c>
-      <c r="K4" s="64" t="inlineStr">
+      <c r="K4" s="69" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="L4" s="64" t="inlineStr">
+      <c r="L4" s="69" t="inlineStr">
         <is>
           <t>€/jour/pers</t>
         </is>
       </c>
-      <c r="N4" s="64" t="inlineStr">
+      <c r="N4" s="69" t="inlineStr">
         <is>
           <t>Forfait par jour</t>
         </is>
       </c>
-      <c r="Q4" s="64" t="inlineStr">
+      <c r="Q4" s="69" t="inlineStr">
         <is>
           <t>Taille + test OK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="64" t="inlineStr">
+      <c r="A5" s="69" t="inlineStr">
         <is>
           <t>Céline CARDONA</t>
         </is>
       </c>
-      <c r="B5" s="64" t="inlineStr">
+      <c r="B5" s="69" t="inlineStr">
         <is>
           <t>ccardona@enedril.fr</t>
         </is>
       </c>
-      <c r="D5" s="64" t="inlineStr">
+      <c r="D5" s="69" t="inlineStr">
         <is>
           <t>DDP</t>
         </is>
       </c>
-      <c r="E5" s="64" t="inlineStr">
+      <c r="E5" s="69" t="inlineStr">
         <is>
           <t>90 jours / 90 days</t>
         </is>
       </c>
-      <c r="F5" s="64" t="inlineStr">
+      <c r="F5" s="69" t="inlineStr">
         <is>
           <t>À la commande / Upon order</t>
         </is>
       </c>
-      <c r="J5" s="64" t="inlineStr">
+      <c r="J5" s="69" t="inlineStr">
         <is>
           <t>Loose (vrac)</t>
         </is>
       </c>
-      <c r="K5" s="64" t="inlineStr">
+      <c r="K5" s="69" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="L5" s="64" t="inlineStr">
+      <c r="L5" s="69" t="inlineStr">
         <is>
           <t>€/pers</t>
         </is>
       </c>
-      <c r="Q5" s="64" t="inlineStr">
+      <c r="Q5" s="69" t="inlineStr">
         <is>
           <t>À contrôler</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="64" t="inlineStr">
+      <c r="A6" s="69" t="inlineStr">
         <is>
           <t>Koen MONDELAERS</t>
         </is>
       </c>
-      <c r="B6" s="64" t="inlineStr">
+      <c r="B6" s="69" t="inlineStr">
         <is>
           <t>kmondelaers@enedril.fr</t>
         </is>
       </c>
-      <c r="D6" s="64" t="inlineStr">
+      <c r="D6" s="69" t="inlineStr">
         <is>
           <t>FOB</t>
         </is>
       </c>
-      <c r="K6" s="64" t="inlineStr">
+      <c r="K6" s="69" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="L6" s="64" t="inlineStr">
+      <c r="L6" s="69" t="inlineStr">
         <is>
           <t>€/unité</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="64" t="inlineStr">
+      <c r="A7" s="69" t="inlineStr">
         <is>
           <t>Luigi LIBERATORE</t>
         </is>
       </c>
-      <c r="B7" s="64" t="inlineStr">
+      <c r="B7" s="69" t="inlineStr">
         <is>
           <t>lliberatore@enedril.fr</t>
         </is>
       </c>
-      <c r="K7" s="64" t="inlineStr">
+      <c r="K7" s="69" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="K8" s="64" t="inlineStr">
+      <c r="K8" s="69" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="K9" s="64" t="inlineStr">
+      <c r="K9" s="69" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
@@ -4700,21 +4654,21 @@
           <t>Pour ajouter un contact, une validité, etc. : écrire à la suite dans la colonne (les listes déroulantes lisent les 12 premières lignes).</t>
         </is>
       </c>
-      <c r="K10" s="64" t="inlineStr">
+      <c r="K10" s="69" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="K11" s="64" t="inlineStr">
+      <c r="K11" s="69" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="K12" s="64" t="inlineStr">
+      <c r="K12" s="69" t="inlineStr">
         <is>
           <t>Loose</t>
         </is>
@@ -4741,358 +4695,358 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>Clé</t>
         </is>
       </c>
-      <c r="B1" s="62" t="inlineStr">
+      <c r="B1" s="67" t="inlineStr">
         <is>
           <t>Français</t>
         </is>
       </c>
-      <c r="C1" s="62" t="inlineStr">
+      <c r="C1" s="67" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="66" t="inlineStr">
+      <c r="A2" s="71" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B2" s="66" t="inlineStr">
+      <c r="B2" s="71" t="inlineStr">
         <is>
           <t>OFFRE DE LOCATION</t>
         </is>
       </c>
-      <c r="C2" s="66" t="inlineStr">
+      <c r="C2" s="71" t="inlineStr">
         <is>
           <t>EQUIPMENT RENTAL QUOTATION</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="66" t="inlineStr">
+      <c r="A3" s="71" t="inlineStr">
         <is>
           <t>client</t>
         </is>
       </c>
-      <c r="B3" s="66" t="inlineStr">
+      <c r="B3" s="71" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C3" s="66" t="inlineStr">
+      <c r="C3" s="71" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="66" t="inlineStr">
+      <c r="A4" s="71" t="inlineStr">
         <is>
           <t>attn</t>
         </is>
       </c>
-      <c r="B4" s="66" t="inlineStr">
+      <c r="B4" s="71" t="inlineStr">
         <is>
           <t>À l'attention de</t>
         </is>
       </c>
-      <c r="C4" s="66" t="inlineStr">
+      <c r="C4" s="71" t="inlineStr">
         <is>
           <t>Attention</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="66" t="inlineStr">
+      <c r="A5" s="71" t="inlineStr">
         <is>
           <t>well</t>
         </is>
       </c>
-      <c r="B5" s="66" t="inlineStr">
+      <c r="B5" s="71" t="inlineStr">
         <is>
           <t>Puits / Chantier</t>
         </is>
       </c>
-      <c r="C5" s="66" t="inlineStr">
+      <c r="C5" s="71" t="inlineStr">
         <is>
           <t>Well / Location</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="66" t="inlineStr">
+      <c r="A6" s="71" t="inlineStr">
         <is>
           <t>rig</t>
         </is>
       </c>
-      <c r="B6" s="66" t="inlineStr">
+      <c r="B6" s="71" t="inlineStr">
         <is>
           <t>Rig</t>
         </is>
       </c>
-      <c r="C6" s="66" t="inlineStr">
+      <c r="C6" s="71" t="inlineStr">
         <is>
           <t>Rig</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="66" t="inlineStr">
+      <c r="A7" s="71" t="inlineStr">
         <is>
           <t>offer</t>
         </is>
       </c>
-      <c r="B7" s="66" t="inlineStr">
+      <c r="B7" s="71" t="inlineStr">
         <is>
           <t>N° d'offre</t>
         </is>
       </c>
-      <c r="C7" s="66" t="inlineStr">
+      <c r="C7" s="71" t="inlineStr">
         <is>
           <t>Offer N°</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="66" t="inlineStr">
+      <c r="A8" s="71" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B8" s="66" t="inlineStr">
+      <c r="B8" s="71" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C8" s="66" t="inlineStr">
+      <c r="C8" s="71" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="66" t="inlineStr">
+      <c r="A9" s="71" t="inlineStr">
         <is>
           <t>valid</t>
         </is>
       </c>
-      <c r="B9" s="66" t="inlineStr">
+      <c r="B9" s="71" t="inlineStr">
         <is>
           <t>Validité de l'offre</t>
         </is>
       </c>
-      <c r="C9" s="66" t="inlineStr">
+      <c r="C9" s="71" t="inlineStr">
         <is>
           <t>Validity</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="66" t="inlineStr">
+      <c r="A10" s="71" t="inlineStr">
         <is>
           <t>inco</t>
         </is>
       </c>
-      <c r="B10" s="66" t="inlineStr">
+      <c r="B10" s="71" t="inlineStr">
         <is>
           <t>Incoterm</t>
         </is>
       </c>
-      <c r="C10" s="66" t="inlineStr">
+      <c r="C10" s="71" t="inlineStr">
         <is>
           <t>Incoterm</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="66" t="inlineStr">
+      <c r="A11" s="71" t="inlineStr">
         <is>
           <t>lead</t>
         </is>
       </c>
-      <c r="B11" s="66" t="inlineStr">
+      <c r="B11" s="71" t="inlineStr">
         <is>
           <t>Délai de mise à dispo</t>
         </is>
       </c>
-      <c r="C11" s="66" t="inlineStr">
+      <c r="C11" s="71" t="inlineStr">
         <is>
           <t>Lead time</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="66" t="inlineStr">
+      <c r="A12" s="71" t="inlineStr">
         <is>
           <t>pay</t>
         </is>
       </c>
-      <c r="B12" s="66" t="inlineStr">
+      <c r="B12" s="71" t="inlineStr">
         <is>
           <t>Conditions de règlement</t>
         </is>
       </c>
-      <c r="C12" s="66" t="inlineStr">
+      <c r="C12" s="71" t="inlineStr">
         <is>
           <t>Payment terms</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="66" t="inlineStr">
+      <c r="A13" s="71" t="inlineStr">
         <is>
           <t>we</t>
         </is>
       </c>
-      <c r="B13" s="66" t="inlineStr">
+      <c r="B13" s="71" t="inlineStr">
         <is>
           <t>Facturation WE et jours fériés</t>
         </is>
       </c>
-      <c r="C13" s="66" t="inlineStr">
+      <c r="C13" s="71" t="inlineStr">
         <is>
           <t>Weekend &amp; holiday billing</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="66" t="inlineStr">
+      <c r="A14" s="71" t="inlineStr">
         <is>
           <t>by</t>
         </is>
       </c>
-      <c r="B14" s="66" t="inlineStr">
+      <c r="B14" s="71" t="inlineStr">
         <is>
           <t>Établi par</t>
         </is>
       </c>
-      <c r="C14" s="66" t="inlineStr">
+      <c r="C14" s="71" t="inlineStr">
         <is>
           <t>Established by</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="66" t="inlineStr">
+      <c r="A15" s="71" t="inlineStr">
         <is>
           <t>mail</t>
         </is>
       </c>
-      <c r="B15" s="66" t="inlineStr">
+      <c r="B15" s="71" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
-      <c r="C15" s="66" t="inlineStr">
+      <c r="C15" s="71" t="inlineStr">
         <is>
           <t>E-mail</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="66" t="inlineStr">
+      <c r="A16" s="71" t="inlineStr">
         <is>
           <t>tel</t>
         </is>
       </c>
-      <c r="B16" s="66" t="inlineStr">
+      <c r="B16" s="71" t="inlineStr">
         <is>
           <t>Téléphone</t>
         </is>
       </c>
-      <c r="C16" s="66" t="inlineStr">
+      <c r="C16" s="71" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="66" t="inlineStr">
+      <c r="A17" s="71" t="inlineStr">
         <is>
           <t>sec_eq</t>
         </is>
       </c>
-      <c r="B17" s="66" t="inlineStr">
+      <c r="B17" s="71" t="inlineStr">
         <is>
           <t>MATÉRIEL</t>
         </is>
       </c>
-      <c r="C17" s="66" t="inlineStr">
+      <c r="C17" s="71" t="inlineStr">
         <is>
           <t>EQUIPMENT</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="66" t="inlineStr">
+      <c r="A18" s="71" t="inlineStr">
         <is>
           <t>h_n</t>
         </is>
       </c>
-      <c r="B18" s="66" t="inlineStr">
+      <c r="B18" s="71" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C18" s="66" t="inlineStr">
+      <c r="C18" s="71" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="66" t="inlineStr">
+      <c r="A19" s="71" t="inlineStr">
         <is>
           <t>h_desc</t>
         </is>
       </c>
-      <c r="B19" s="66" t="inlineStr">
+      <c r="B19" s="71" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C19" s="66" t="inlineStr">
+      <c r="C19" s="71" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="66" t="inlineStr">
+      <c r="A20" s="71" t="inlineStr">
         <is>
           <t>h_qty</t>
         </is>
       </c>
-      <c r="B20" s="66" t="inlineStr">
+      <c r="B20" s="71" t="inlineStr">
         <is>
           <t>Qté</t>
         </is>
       </c>
-      <c r="C20" s="66" t="inlineStr">
+      <c r="C20" s="71" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="66" t="inlineStr">
+      <c r="A21" s="71" t="inlineStr">
         <is>
           <t>h_s</t>
         </is>
       </c>
-      <c r="B21" s="66" t="inlineStr">
+      <c r="B21" s="71" t="inlineStr">
         <is>
           <t>Stand-by (S)
 € / jour / item</t>
         </is>
       </c>
-      <c r="C21" s="66" t="inlineStr">
+      <c r="C21" s="71" t="inlineStr">
         <is>
           <t>Stand-by (S)
 daily rate / item</t>
@@ -5100,18 +5054,18 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="66" t="inlineStr">
+      <c r="A22" s="71" t="inlineStr">
         <is>
           <t>h_o</t>
         </is>
       </c>
-      <c r="B22" s="66" t="inlineStr">
+      <c r="B22" s="71" t="inlineStr">
         <is>
           <t>Opérations (O)
 € / jour / item</t>
         </is>
       </c>
-      <c r="C22" s="66" t="inlineStr">
+      <c r="C22" s="71" t="inlineStr">
         <is>
           <t>Operations (O)
 daily rate / item</t>
@@ -5119,19 +5073,19 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="66" t="inlineStr">
+      <c r="A23" s="71" t="inlineStr">
         <is>
           <t>h_uc</t>
         </is>
       </c>
-      <c r="B23" s="66" t="inlineStr">
+      <c r="B23" s="71" t="inlineStr">
         <is>
           <t>Utilisation
 Charge (UC)
 € / item</t>
         </is>
       </c>
-      <c r="C23" s="66" t="inlineStr">
+      <c r="C23" s="71" t="inlineStr">
         <is>
           <t>Utilisation
 Charge (UC)
@@ -5140,18 +5094,18 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="66" t="inlineStr">
+      <c r="A24" s="71" t="inlineStr">
         <is>
           <t>h_lih</t>
         </is>
       </c>
-      <c r="B24" s="66" t="inlineStr">
+      <c r="B24" s="71" t="inlineStr">
         <is>
           <t>Valeur de remplacement
 (LIH / DBR) € / item</t>
         </is>
       </c>
-      <c r="C24" s="66" t="inlineStr">
+      <c r="C24" s="71" t="inlineStr">
         <is>
           <t>Replacement value
 (LIH / DBR) per item</t>
@@ -5159,18 +5113,18 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="66" t="inlineStr">
+      <c r="A25" s="71" t="inlineStr">
         <is>
           <t>h_insp</t>
         </is>
       </c>
-      <c r="B25" s="66" t="inlineStr">
+      <c r="B25" s="71" t="inlineStr">
         <is>
           <t>Inspection
 € / item</t>
         </is>
       </c>
-      <c r="C25" s="66" t="inlineStr">
+      <c r="C25" s="71" t="inlineStr">
         <is>
           <t>Inspection
 per item</t>
@@ -5178,18 +5132,18 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="66" t="inlineStr">
+      <c r="A26" s="71" t="inlineStr">
         <is>
           <t>h_rest</t>
         </is>
       </c>
-      <c r="B26" s="66" t="inlineStr">
+      <c r="B26" s="71" t="inlineStr">
         <is>
           <t>Restocking
 €</t>
         </is>
       </c>
-      <c r="C26" s="66" t="inlineStr">
+      <c r="C26" s="71" t="inlineStr">
         <is>
           <t>Restocking
 charge</t>
@@ -5197,493 +5151,493 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="66" t="inlineStr">
+      <c r="A27" s="71" t="inlineStr">
         <is>
           <t>h_ref</t>
         </is>
       </c>
-      <c r="B27" s="66" t="inlineStr">
+      <c r="B27" s="71" t="inlineStr">
         <is>
           <t>Remarques</t>
         </is>
       </c>
-      <c r="C27" s="66" t="inlineStr">
+      <c r="C27" s="71" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="66" t="inlineStr">
+      <c r="A28" s="71" t="inlineStr">
         <is>
           <t>incl</t>
         </is>
       </c>
-      <c r="B28" s="66" t="inlineStr">
+      <c r="B28" s="71" t="inlineStr">
         <is>
           <t>incl.</t>
         </is>
       </c>
-      <c r="C28" s="66" t="inlineStr">
+      <c r="C28" s="71" t="inlineStr">
         <is>
           <t>incl.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="66" t="inlineStr">
+      <c r="A29" s="71" t="inlineStr">
         <is>
           <t>incl_long</t>
         </is>
       </c>
-      <c r="B29" s="66" t="inlineStr">
+      <c r="B29" s="71" t="inlineStr">
         <is>
           <t>Inclus au forfait</t>
         </is>
       </c>
-      <c r="C29" s="66" t="inlineStr">
+      <c r="C29" s="71" t="inlineStr">
         <is>
           <t>Included in lump sum</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="66" t="inlineStr">
+      <c r="A30" s="71" t="inlineStr">
         <is>
           <t>sec_opt</t>
         </is>
       </c>
-      <c r="B30" s="66" t="inlineStr">
+      <c r="B30" s="71" t="inlineStr">
         <is>
           <t>PRESTATIONS ET OPTIONS</t>
         </is>
       </c>
-      <c r="C30" s="66" t="inlineStr">
+      <c r="C30" s="71" t="inlineStr">
         <is>
           <t>SERVICES AND OPTIONS</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="66" t="inlineStr">
+      <c r="A31" s="71" t="inlineStr">
         <is>
           <t>h_label</t>
         </is>
       </c>
-      <c r="B31" s="66" t="inlineStr">
+      <c r="B31" s="71" t="inlineStr">
         <is>
           <t>Prestation</t>
         </is>
       </c>
-      <c r="C31" s="66" t="inlineStr">
+      <c r="C31" s="71" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="66" t="inlineStr">
+      <c r="A32" s="71" t="inlineStr">
         <is>
           <t>h_unit</t>
         </is>
       </c>
-      <c r="B32" s="66" t="inlineStr">
+      <c r="B32" s="71" t="inlineStr">
         <is>
           <t>Unité</t>
         </is>
       </c>
-      <c r="C32" s="66" t="inlineStr">
+      <c r="C32" s="71" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="66" t="inlineStr">
+      <c r="A33" s="71" t="inlineStr">
         <is>
           <t>h_pu</t>
         </is>
       </c>
-      <c r="B33" s="66" t="inlineStr">
+      <c r="B33" s="71" t="inlineStr">
         <is>
           <t>Prix unitaire €</t>
         </is>
       </c>
-      <c r="C33" s="66" t="inlineStr">
+      <c r="C33" s="71" t="inlineStr">
         <is>
           <t>Unit price €</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="66" t="inlineStr">
+      <c r="A34" s="71" t="inlineStr">
         <is>
           <t>h_tot</t>
         </is>
       </c>
-      <c r="B34" s="66" t="inlineStr">
+      <c r="B34" s="71" t="inlineStr">
         <is>
           <t>Total €</t>
         </is>
       </c>
-      <c r="C34" s="66" t="inlineStr">
+      <c r="C34" s="71" t="inlineStr">
         <is>
           <t>Total €</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="66" t="inlineStr">
+      <c r="A35" s="71" t="inlineStr">
         <is>
           <t>h_det</t>
         </is>
       </c>
-      <c r="B35" s="66" t="inlineStr">
+      <c r="B35" s="71" t="inlineStr">
         <is>
           <t>Détail</t>
         </is>
       </c>
-      <c r="C35" s="66" t="inlineStr">
+      <c r="C35" s="71" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="66" t="inlineStr">
+      <c r="A36" s="71" t="inlineStr">
         <is>
           <t>op_day</t>
         </is>
       </c>
-      <c r="B36" s="66" t="inlineStr">
+      <c r="B36" s="71" t="inlineStr">
         <is>
           <t>Opérateur · tarif journalier</t>
         </is>
       </c>
-      <c r="C36" s="66" t="inlineStr">
+      <c r="C36" s="71" t="inlineStr">
         <is>
           <t>Operator · daily rate</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="66" t="inlineStr">
+      <c r="A37" s="71" t="inlineStr">
         <is>
           <t>op_mob</t>
         </is>
       </c>
-      <c r="B37" s="66" t="inlineStr">
+      <c r="B37" s="71" t="inlineStr">
         <is>
           <t>Opérateur · Mob / Demob</t>
         </is>
       </c>
-      <c r="C37" s="66" t="inlineStr">
+      <c r="C37" s="71" t="inlineStr">
         <is>
           <t>Operator · Mob / Demob</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="66" t="inlineStr">
+      <c r="A38" s="71" t="inlineStr">
         <is>
           <t>tight</t>
         </is>
       </c>
-      <c r="B38" s="66" t="inlineStr">
+      <c r="B38" s="71" t="inlineStr">
         <is>
           <t>Serrage · prix par serrage</t>
         </is>
       </c>
-      <c r="C38" s="66" t="inlineStr">
+      <c r="C38" s="71" t="inlineStr">
         <is>
           <t>Tong &amp; make-up service · price per make-up</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="66" t="inlineStr">
+      <c r="A39" s="71" t="inlineStr">
         <is>
           <t>tr_mob</t>
         </is>
       </c>
-      <c r="B39" s="66" t="inlineStr">
+      <c r="B39" s="71" t="inlineStr">
         <is>
           <t>Transport MOB (Lons → chantier)</t>
         </is>
       </c>
-      <c r="C39" s="66" t="inlineStr">
+      <c r="C39" s="71" t="inlineStr">
         <is>
           <t>Transport MOB (Lons → site)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="66" t="inlineStr">
+      <c r="A40" s="71" t="inlineStr">
         <is>
           <t>tr_dem</t>
         </is>
       </c>
-      <c r="B40" s="66" t="inlineStr">
+      <c r="B40" s="71" t="inlineStr">
         <is>
           <t>Transport DEMOB (chantier → Lons)</t>
         </is>
       </c>
-      <c r="C40" s="66" t="inlineStr">
+      <c r="C40" s="71" t="inlineStr">
         <is>
           <t>Transport DEMOB (site → Lons)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="66" t="inlineStr">
+      <c r="A41" s="71" t="inlineStr">
         <is>
           <t>free</t>
         </is>
       </c>
-      <c r="B41" s="66" t="inlineStr">
+      <c r="B41" s="71" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="C41" s="66" t="inlineStr">
+      <c r="C41" s="71" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="66" t="inlineStr">
+      <c r="A42" s="71" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="B42" s="66" t="inlineStr">
+      <c r="B42" s="71" t="inlineStr">
         <is>
           <t>Forfait</t>
         </is>
       </c>
-      <c r="C42" s="66" t="inlineStr">
+      <c r="C42" s="71" t="inlineStr">
         <is>
           <t>Lump sum</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="66" t="inlineStr">
+      <c r="A43" s="71" t="inlineStr">
         <is>
           <t>at_cost</t>
         </is>
       </c>
-      <c r="B43" s="66" t="inlineStr">
+      <c r="B43" s="71" t="inlineStr">
         <is>
           <t>au coût réel +15 %</t>
         </is>
       </c>
-      <c r="C43" s="66" t="inlineStr">
+      <c r="C43" s="71" t="inlineStr">
         <is>
           <t>at cost +15%</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="66" t="inlineStr">
+      <c r="A44" s="71" t="inlineStr">
         <is>
           <t>tr_note</t>
         </is>
       </c>
-      <c r="B44" s="66" t="inlineStr">
+      <c r="B44" s="71" t="inlineStr">
         <is>
           <t>Transport organisé par Enedril</t>
         </is>
       </c>
-      <c r="C44" s="66" t="inlineStr">
+      <c r="C44" s="71" t="inlineStr">
         <is>
           <t>Transport organised by Enedril</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="66" t="inlineStr">
+      <c r="A45" s="71" t="inlineStr">
         <is>
           <t>ht</t>
         </is>
       </c>
-      <c r="B45" s="66" t="inlineStr">
+      <c r="B45" s="71" t="inlineStr">
         <is>
           <t>€ HT</t>
         </is>
       </c>
-      <c r="C45" s="66" t="inlineStr">
+      <c r="C45" s="71" t="inlineStr">
         <is>
           <t>€ excl. VAT</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="66" t="inlineStr">
+      <c r="A46" s="71" t="inlineStr">
         <is>
           <t>calc_det</t>
         </is>
       </c>
-      <c r="B46" s="66" t="inlineStr">
+      <c r="B46" s="71" t="inlineStr">
         <is>
           <t>j stand-by + %s j opérations + utilisations de charge (UC)</t>
         </is>
       </c>
-      <c r="C46" s="66" t="inlineStr">
+      <c r="C46" s="71" t="inlineStr">
         <is>
           <t>stand-by days + %s operation days + utilisation charges (UC)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="66" t="inlineStr">
+      <c r="A47" s="71" t="inlineStr">
         <is>
           <t>sec_cond</t>
         </is>
       </c>
-      <c r="B47" s="66" t="inlineStr">
+      <c r="B47" s="71" t="inlineStr">
         <is>
           <t>CONDITIONS PARTICULIÈRES · SPECIFIC CONDITIONS</t>
         </is>
       </c>
-      <c r="C47" s="66" t="inlineStr">
+      <c r="C47" s="71" t="inlineStr">
         <is>
           <t>SPECIFIC CONDITIONS · CONDITIONS PARTICULIÈRES</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="66" t="inlineStr">
+      <c r="A48" s="71" t="inlineStr">
         <is>
           <t>accept</t>
         </is>
       </c>
-      <c r="B48" s="66" t="inlineStr">
+      <c r="B48" s="71" t="inlineStr">
         <is>
           <t>BON POUR ACCORD</t>
         </is>
       </c>
-      <c r="C48" s="66" t="inlineStr">
+      <c r="C48" s="71" t="inlineStr">
         <is>
           <t>ACCEPTED BY</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="66" t="inlineStr">
+      <c r="A49" s="71" t="inlineStr">
         <is>
           <t>sig_name</t>
         </is>
       </c>
-      <c r="B49" s="66" t="inlineStr">
+      <c r="B49" s="71" t="inlineStr">
         <is>
           <t>Nom et qualité</t>
         </is>
       </c>
-      <c r="C49" s="66" t="inlineStr">
+      <c r="C49" s="71" t="inlineStr">
         <is>
           <t>Name and title</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="66" t="inlineStr">
+      <c r="A50" s="71" t="inlineStr">
         <is>
           <t>sig_date</t>
         </is>
       </c>
-      <c r="B50" s="66" t="inlineStr">
+      <c r="B50" s="71" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C50" s="66" t="inlineStr">
+      <c r="C50" s="71" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="66" t="inlineStr">
+      <c r="A51" s="71" t="inlineStr">
         <is>
           <t>sig_sig</t>
         </is>
       </c>
-      <c r="B51" s="66" t="inlineStr">
+      <c r="B51" s="71" t="inlineStr">
         <is>
           <t>Signature et cachet</t>
         </is>
       </c>
-      <c r="C51" s="66" t="inlineStr">
+      <c r="C51" s="71" t="inlineStr">
         <is>
           <t>Signature and stamp</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="66" t="inlineStr">
+      <c r="A52" s="71" t="inlineStr">
         <is>
           <t>lump</t>
         </is>
       </c>
-      <c r="B52" s="66" t="inlineStr">
+      <c r="B52" s="71" t="inlineStr">
         <is>
           <t>forfait</t>
         </is>
       </c>
-      <c r="C52" s="66" t="inlineStr">
+      <c r="C52" s="71" t="inlineStr">
         <is>
           <t>lump sum</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="66" t="inlineStr">
+      <c r="A53" s="71" t="inlineStr">
         <is>
           <t>sec_tight</t>
         </is>
       </c>
-      <c r="B53" s="66" t="inlineStr">
+      <c r="B53" s="71" t="inlineStr">
         <is>
           <t>SERRAGE · TONG &amp; MAKE-UP</t>
         </is>
       </c>
-      <c r="C53" s="66" t="inlineStr">
+      <c r="C53" s="71" t="inlineStr">
         <is>
           <t>TONG &amp; MAKE-UP SERVICE</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="66" t="inlineStr">
+      <c r="A54" s="71" t="inlineStr">
         <is>
           <t>sec_tr</t>
         </is>
       </c>
-      <c r="B54" s="66" t="inlineStr">
+      <c r="B54" s="71" t="inlineStr">
         <is>
           <t>TRANSPORT</t>
         </is>
       </c>
-      <c r="C54" s="66" t="inlineStr">
+      <c r="C54" s="71" t="inlineStr">
         <is>
           <t>TRANSPORT</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="66" t="inlineStr">
+      <c r="A55" s="71" t="inlineStr">
         <is>
           <t>sec_op</t>
         </is>
       </c>
-      <c r="B55" s="66" t="inlineStr">
+      <c r="B55" s="71" t="inlineStr">
         <is>
           <t>OPÉRATEURS</t>
         </is>
       </c>
-      <c r="C55" s="66" t="inlineStr">
+      <c r="C55" s="71" t="inlineStr">
         <is>
           <t>OPERATORS</t>
         </is>

</xml_diff>

<commit_message>
Devis 2027 : condition transport fournisseur (coût +15 %), forfait N jours avec serrage et transport inclus
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Devis_Enedril_2027.xlsx
+++ b/devis_2027/Devis_Enedril_2027.xlsx
@@ -2491,7 +2491,7 @@
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="29">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("title",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("title",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="K1" s="1" t="n"/>
@@ -2522,15 +2522,15 @@
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("client",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("client",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="D5" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("offer",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("offer",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="H5" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("date",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("date",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
@@ -2556,15 +2556,15 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("attn",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("attn",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="D7" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("well",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("well",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="H7" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("by",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("by",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
@@ -2590,15 +2590,15 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("inco",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("inco",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="D9" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("valid",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("valid",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="H9" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("mail",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("mail",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
@@ -2624,15 +2624,15 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="B11" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("pay",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("pay",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="D11" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("we",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("we",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
       <c r="H11" s="31">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("tel",Textes!$A$2:$A$55,0),Listes!$H$1))</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("tel",Textes!$A$2:$A$59,0),Listes!$H$1))</f>
         <v/>
       </c>
     </row>
@@ -2659,7 +2659,7 @@
     <row r="13" ht="8" customHeight="1"/>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="34">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sec_eq",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sec_eq",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="C14" s="35" t="n"/>
@@ -2673,39 +2673,39 @@
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="B15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_n",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_n",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="C15" s="37">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_desc",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_desc",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="D15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_qty",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="E15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_s",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_s",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="F15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_o",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_o",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="G15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_uc",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_uc",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="H15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_lih",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_lih",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="I15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_insp",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_insp",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="J15" s="36">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_rest",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_rest",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
     </row>
@@ -4558,7 +4558,7 @@
     <row r="57" ht="8" customHeight="1"/>
     <row r="58" ht="20" customHeight="1">
       <c r="B58" s="34">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sec_cond",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sec_cond",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="C58" s="35" t="n"/>
@@ -4570,22 +4570,24 @@
       <c r="I58" s="35" t="n"/>
       <c r="J58" s="35" t="n"/>
     </row>
-    <row r="59" ht="76" customHeight="1">
+    <row r="59" ht="92" customHeight="1">
       <c r="B59" s="44" t="inlineStr">
         <is>
           <t>La location s'entend depuis le jour de départ de la base d'origine jusqu'à son retour au même endroit.
 Le Wear Charge s'applique pour toute usure liée à un usage normal des équipements. En cas de dommages plus importants liés à un usage anormal, la valeur de remplacement sera facturée sur documentation.
 Charges additionnelles à prévoir pour le colisage d'outils destinés à une expédition en aérien ou maritime.
+Tous les transports effectués auprès d'un fournisseur pour la fourniture des équipements sont facturés au coût réel +15 % (idem pour les frais de douane, etc.).
 Conditions générales de vente disponibles sur demande ou sur notre site internet www.enedril.com</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="76" customHeight="1">
+    <row r="60" ht="92" customHeight="1">
       <c r="B60" s="44" t="inlineStr">
         <is>
           <t>The rental is from the day of departure from the base of origin until its return to the same place.
 Wear Charge applies to all wear and tear related to normal use of equipment. In case of greater damage due to abnormal use, the replacement value will be charged based on supporting documentation.
 Additional charges may apply for packing tools intended for air or ocean shipment.
+All transport carried out through a supplier for the supply of equipment is invoiced at cost +15% (same for customs fees, etc.).
 General conditions of sale available upon request or on our website www.enedril.com</t>
         </is>
       </c>
@@ -4593,25 +4595,25 @@
     <row r="61" ht="10" customHeight="1"/>
     <row r="62">
       <c r="B62" s="45">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("accept",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("accept",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
     </row>
     <row r="63" ht="17" customHeight="1">
       <c r="B63" s="46">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sig_name",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sig_name",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="C63" s="47" t="n"/>
       <c r="D63" s="46">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sig_date",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sig_date",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="E63" s="48" t="n"/>
       <c r="F63" s="48" t="n"/>
       <c r="G63" s="47" t="n"/>
       <c r="H63" s="46">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sig_sig",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sig_sig",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="I63" s="48" t="n"/>
@@ -5165,7 +5167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6074,49 +6076,117 @@
     <row r="53">
       <c r="A53" s="59" t="inlineStr">
         <is>
-          <t>sec_tight</t>
+          <t>days</t>
         </is>
       </c>
       <c r="B53" s="59" t="inlineStr">
         <is>
-          <t>SERRAGE · TONG &amp; MAKE-UP</t>
+          <t>JOURS</t>
         </is>
       </c>
       <c r="C53" s="59" t="inlineStr">
         <is>
-          <t>TONG &amp; MAKE-UP SERVICE</t>
+          <t>DAYS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="59" t="inlineStr">
         <is>
-          <t>sec_tr</t>
+          <t>in_tight</t>
         </is>
       </c>
       <c r="B54" s="59" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>serrage inclus</t>
         </is>
       </c>
       <c r="C54" s="59" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>make-up included</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="59" t="inlineStr">
         <is>
+          <t>in_tr</t>
+        </is>
+      </c>
+      <c r="B55" s="59" t="inlineStr">
+        <is>
+          <t>transport inclus</t>
+        </is>
+      </c>
+      <c r="C55" s="59" t="inlineStr">
+        <is>
+          <t>transport included</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="59" t="inlineStr">
+        <is>
+          <t>in_both</t>
+        </is>
+      </c>
+      <c r="B56" s="59" t="inlineStr">
+        <is>
+          <t>serrage et transport inclus</t>
+        </is>
+      </c>
+      <c r="C56" s="59" t="inlineStr">
+        <is>
+          <t>make-up and transport included</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="59" t="inlineStr">
+        <is>
+          <t>sec_tight</t>
+        </is>
+      </c>
+      <c r="B57" s="59" t="inlineStr">
+        <is>
+          <t>SERRAGE · TONG &amp; MAKE-UP</t>
+        </is>
+      </c>
+      <c r="C57" s="59" t="inlineStr">
+        <is>
+          <t>TONG &amp; MAKE-UP SERVICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="59" t="inlineStr">
+        <is>
+          <t>sec_tr</t>
+        </is>
+      </c>
+      <c r="B58" s="59" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="C58" s="59" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="59" t="inlineStr">
+        <is>
           <t>sec_op</t>
         </is>
       </c>
-      <c r="B55" s="59" t="inlineStr">
+      <c r="B59" s="59" t="inlineStr">
         <is>
           <t>OPÉRATEURS</t>
         </is>
       </c>
-      <c r="C55" s="59" t="inlineStr">
+      <c r="C59" s="59" t="inlineStr">
         <is>
           <t>OPERATORS</t>
         </is>
@@ -6217,7 +6287,7 @@
         <v/>
       </c>
       <c r="E2">
-        <f>IF(C2="BAN",UPPER('2 Matériel'!$C6),IF(C2="ITM",'2 Matériel'!$C6&amp;IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C2="BAN",UPPER('2 Matériel'!$C6),IF(C2="ITM",'2 Matériel'!$C6&amp;IF(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F2">
@@ -6225,27 +6295,27 @@
         <v/>
       </c>
       <c r="G2">
-        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E6="","",'2 Matériel'!$E6)),"")</f>
+        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E6="","",'2 Matériel'!$E6)),"")</f>
         <v/>
       </c>
       <c r="H2">
-        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F6="","",'2 Matériel'!$F6)),"")</f>
+        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F6="","",'2 Matériel'!$F6)),"")</f>
         <v/>
       </c>
       <c r="I2">
-        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G6="","",'2 Matériel'!$G6)),"")</f>
+        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G6="","",'2 Matériel'!$G6)),"")</f>
         <v/>
       </c>
       <c r="J2">
-        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H6="","",'2 Matériel'!$H6)),"")</f>
+        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H6="","",'2 Matériel'!$H6)),"")</f>
         <v/>
       </c>
       <c r="K2">
-        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I6="","",'2 Matériel'!$I6)),"")</f>
+        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I6="","",'2 Matériel'!$I6)),"")</f>
         <v/>
       </c>
       <c r="L2">
-        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J6="","",'2 Matériel'!$J6)),"")</f>
+        <f>IF(C2="ITM",IF(AND(AND('2 Matériel'!$K6="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J6="","",'2 Matériel'!$J6)),"")</f>
         <v/>
       </c>
     </row>
@@ -6267,7 +6337,7 @@
         <v/>
       </c>
       <c r="E3">
-        <f>IF(C3="BAN",UPPER('2 Matériel'!$C7),IF(C3="ITM",'2 Matériel'!$C7&amp;IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C3="BAN",UPPER('2 Matériel'!$C7),IF(C3="ITM",'2 Matériel'!$C7&amp;IF(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F3">
@@ -6275,27 +6345,27 @@
         <v/>
       </c>
       <c r="G3">
-        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E7="","",'2 Matériel'!$E7)),"")</f>
+        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E7="","",'2 Matériel'!$E7)),"")</f>
         <v/>
       </c>
       <c r="H3">
-        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F7="","",'2 Matériel'!$F7)),"")</f>
+        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F7="","",'2 Matériel'!$F7)),"")</f>
         <v/>
       </c>
       <c r="I3">
-        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G7="","",'2 Matériel'!$G7)),"")</f>
+        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G7="","",'2 Matériel'!$G7)),"")</f>
         <v/>
       </c>
       <c r="J3">
-        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H7="","",'2 Matériel'!$H7)),"")</f>
+        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H7="","",'2 Matériel'!$H7)),"")</f>
         <v/>
       </c>
       <c r="K3">
-        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I7="","",'2 Matériel'!$I7)),"")</f>
+        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I7="","",'2 Matériel'!$I7)),"")</f>
         <v/>
       </c>
       <c r="L3">
-        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J7="","",'2 Matériel'!$J7)),"")</f>
+        <f>IF(C3="ITM",IF(AND(AND('2 Matériel'!$K7="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J7="","",'2 Matériel'!$J7)),"")</f>
         <v/>
       </c>
     </row>
@@ -6317,7 +6387,7 @@
         <v/>
       </c>
       <c r="E4">
-        <f>IF(C4="BAN",UPPER('2 Matériel'!$C8),IF(C4="ITM",'2 Matériel'!$C8&amp;IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C4="BAN",UPPER('2 Matériel'!$C8),IF(C4="ITM",'2 Matériel'!$C8&amp;IF(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F4">
@@ -6325,27 +6395,27 @@
         <v/>
       </c>
       <c r="G4">
-        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E8="","",'2 Matériel'!$E8)),"")</f>
+        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E8="","",'2 Matériel'!$E8)),"")</f>
         <v/>
       </c>
       <c r="H4">
-        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F8="","",'2 Matériel'!$F8)),"")</f>
+        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F8="","",'2 Matériel'!$F8)),"")</f>
         <v/>
       </c>
       <c r="I4">
-        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G8="","",'2 Matériel'!$G8)),"")</f>
+        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G8="","",'2 Matériel'!$G8)),"")</f>
         <v/>
       </c>
       <c r="J4">
-        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H8="","",'2 Matériel'!$H8)),"")</f>
+        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H8="","",'2 Matériel'!$H8)),"")</f>
         <v/>
       </c>
       <c r="K4">
-        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I8="","",'2 Matériel'!$I8)),"")</f>
+        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I8="","",'2 Matériel'!$I8)),"")</f>
         <v/>
       </c>
       <c r="L4">
-        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J8="","",'2 Matériel'!$J8)),"")</f>
+        <f>IF(C4="ITM",IF(AND(AND('2 Matériel'!$K8="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J8="","",'2 Matériel'!$J8)),"")</f>
         <v/>
       </c>
     </row>
@@ -6367,7 +6437,7 @@
         <v/>
       </c>
       <c r="E5">
-        <f>IF(C5="BAN",UPPER('2 Matériel'!$C9),IF(C5="ITM",'2 Matériel'!$C9&amp;IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C5="BAN",UPPER('2 Matériel'!$C9),IF(C5="ITM",'2 Matériel'!$C9&amp;IF(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F5">
@@ -6375,27 +6445,27 @@
         <v/>
       </c>
       <c r="G5">
-        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E9="","",'2 Matériel'!$E9)),"")</f>
+        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E9="","",'2 Matériel'!$E9)),"")</f>
         <v/>
       </c>
       <c r="H5">
-        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F9="","",'2 Matériel'!$F9)),"")</f>
+        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F9="","",'2 Matériel'!$F9)),"")</f>
         <v/>
       </c>
       <c r="I5">
-        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G9="","",'2 Matériel'!$G9)),"")</f>
+        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G9="","",'2 Matériel'!$G9)),"")</f>
         <v/>
       </c>
       <c r="J5">
-        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H9="","",'2 Matériel'!$H9)),"")</f>
+        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H9="","",'2 Matériel'!$H9)),"")</f>
         <v/>
       </c>
       <c r="K5">
-        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I9="","",'2 Matériel'!$I9)),"")</f>
+        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I9="","",'2 Matériel'!$I9)),"")</f>
         <v/>
       </c>
       <c r="L5">
-        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J9="","",'2 Matériel'!$J9)),"")</f>
+        <f>IF(C5="ITM",IF(AND(AND('2 Matériel'!$K9="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J9="","",'2 Matériel'!$J9)),"")</f>
         <v/>
       </c>
     </row>
@@ -6417,7 +6487,7 @@
         <v/>
       </c>
       <c r="E6">
-        <f>IF(C6="BAN",UPPER('2 Matériel'!$C10),IF(C6="ITM",'2 Matériel'!$C10&amp;IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C6="BAN",UPPER('2 Matériel'!$C10),IF(C6="ITM",'2 Matériel'!$C10&amp;IF(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F6">
@@ -6425,27 +6495,27 @@
         <v/>
       </c>
       <c r="G6">
-        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E10="","",'2 Matériel'!$E10)),"")</f>
+        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E10="","",'2 Matériel'!$E10)),"")</f>
         <v/>
       </c>
       <c r="H6">
-        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F10="","",'2 Matériel'!$F10)),"")</f>
+        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F10="","",'2 Matériel'!$F10)),"")</f>
         <v/>
       </c>
       <c r="I6">
-        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G10="","",'2 Matériel'!$G10)),"")</f>
+        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G10="","",'2 Matériel'!$G10)),"")</f>
         <v/>
       </c>
       <c r="J6">
-        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H10="","",'2 Matériel'!$H10)),"")</f>
+        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H10="","",'2 Matériel'!$H10)),"")</f>
         <v/>
       </c>
       <c r="K6">
-        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I10="","",'2 Matériel'!$I10)),"")</f>
+        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I10="","",'2 Matériel'!$I10)),"")</f>
         <v/>
       </c>
       <c r="L6">
-        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J10="","",'2 Matériel'!$J10)),"")</f>
+        <f>IF(C6="ITM",IF(AND(AND('2 Matériel'!$K10="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J10="","",'2 Matériel'!$J10)),"")</f>
         <v/>
       </c>
     </row>
@@ -6467,7 +6537,7 @@
         <v/>
       </c>
       <c r="E7">
-        <f>IF(C7="BAN",UPPER('2 Matériel'!$C11),IF(C7="ITM",'2 Matériel'!$C11&amp;IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C7="BAN",UPPER('2 Matériel'!$C11),IF(C7="ITM",'2 Matériel'!$C11&amp;IF(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F7">
@@ -6475,27 +6545,27 @@
         <v/>
       </c>
       <c r="G7">
-        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E11="","",'2 Matériel'!$E11)),"")</f>
+        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E11="","",'2 Matériel'!$E11)),"")</f>
         <v/>
       </c>
       <c r="H7">
-        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F11="","",'2 Matériel'!$F11)),"")</f>
+        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F11="","",'2 Matériel'!$F11)),"")</f>
         <v/>
       </c>
       <c r="I7">
-        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G11="","",'2 Matériel'!$G11)),"")</f>
+        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G11="","",'2 Matériel'!$G11)),"")</f>
         <v/>
       </c>
       <c r="J7">
-        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H11="","",'2 Matériel'!$H11)),"")</f>
+        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H11="","",'2 Matériel'!$H11)),"")</f>
         <v/>
       </c>
       <c r="K7">
-        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I11="","",'2 Matériel'!$I11)),"")</f>
+        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I11="","",'2 Matériel'!$I11)),"")</f>
         <v/>
       </c>
       <c r="L7">
-        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J11="","",'2 Matériel'!$J11)),"")</f>
+        <f>IF(C7="ITM",IF(AND(AND('2 Matériel'!$K11="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J11="","",'2 Matériel'!$J11)),"")</f>
         <v/>
       </c>
     </row>
@@ -6517,7 +6587,7 @@
         <v/>
       </c>
       <c r="E8">
-        <f>IF(C8="BAN",UPPER('2 Matériel'!$C12),IF(C8="ITM",'2 Matériel'!$C12&amp;IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C8="BAN",UPPER('2 Matériel'!$C12),IF(C8="ITM",'2 Matériel'!$C12&amp;IF(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F8">
@@ -6525,27 +6595,27 @@
         <v/>
       </c>
       <c r="G8">
-        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E12="","",'2 Matériel'!$E12)),"")</f>
+        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E12="","",'2 Matériel'!$E12)),"")</f>
         <v/>
       </c>
       <c r="H8">
-        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F12="","",'2 Matériel'!$F12)),"")</f>
+        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F12="","",'2 Matériel'!$F12)),"")</f>
         <v/>
       </c>
       <c r="I8">
-        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G12="","",'2 Matériel'!$G12)),"")</f>
+        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G12="","",'2 Matériel'!$G12)),"")</f>
         <v/>
       </c>
       <c r="J8">
-        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H12="","",'2 Matériel'!$H12)),"")</f>
+        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H12="","",'2 Matériel'!$H12)),"")</f>
         <v/>
       </c>
       <c r="K8">
-        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I12="","",'2 Matériel'!$I12)),"")</f>
+        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I12="","",'2 Matériel'!$I12)),"")</f>
         <v/>
       </c>
       <c r="L8">
-        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J12="","",'2 Matériel'!$J12)),"")</f>
+        <f>IF(C8="ITM",IF(AND(AND('2 Matériel'!$K12="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J12="","",'2 Matériel'!$J12)),"")</f>
         <v/>
       </c>
     </row>
@@ -6567,7 +6637,7 @@
         <v/>
       </c>
       <c r="E9">
-        <f>IF(C9="BAN",UPPER('2 Matériel'!$C13),IF(C9="ITM",'2 Matériel'!$C13&amp;IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C9="BAN",UPPER('2 Matériel'!$C13),IF(C9="ITM",'2 Matériel'!$C13&amp;IF(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F9">
@@ -6575,27 +6645,27 @@
         <v/>
       </c>
       <c r="G9">
-        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E13="","",'2 Matériel'!$E13)),"")</f>
+        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E13="","",'2 Matériel'!$E13)),"")</f>
         <v/>
       </c>
       <c r="H9">
-        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F13="","",'2 Matériel'!$F13)),"")</f>
+        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F13="","",'2 Matériel'!$F13)),"")</f>
         <v/>
       </c>
       <c r="I9">
-        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G13="","",'2 Matériel'!$G13)),"")</f>
+        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G13="","",'2 Matériel'!$G13)),"")</f>
         <v/>
       </c>
       <c r="J9">
-        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H13="","",'2 Matériel'!$H13)),"")</f>
+        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H13="","",'2 Matériel'!$H13)),"")</f>
         <v/>
       </c>
       <c r="K9">
-        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I13="","",'2 Matériel'!$I13)),"")</f>
+        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I13="","",'2 Matériel'!$I13)),"")</f>
         <v/>
       </c>
       <c r="L9">
-        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J13="","",'2 Matériel'!$J13)),"")</f>
+        <f>IF(C9="ITM",IF(AND(AND('2 Matériel'!$K13="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J13="","",'2 Matériel'!$J13)),"")</f>
         <v/>
       </c>
     </row>
@@ -6617,7 +6687,7 @@
         <v/>
       </c>
       <c r="E10">
-        <f>IF(C10="BAN",UPPER('2 Matériel'!$C14),IF(C10="ITM",'2 Matériel'!$C14&amp;IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C10="BAN",UPPER('2 Matériel'!$C14),IF(C10="ITM",'2 Matériel'!$C14&amp;IF(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F10">
@@ -6625,27 +6695,27 @@
         <v/>
       </c>
       <c r="G10">
-        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E14="","",'2 Matériel'!$E14)),"")</f>
+        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E14="","",'2 Matériel'!$E14)),"")</f>
         <v/>
       </c>
       <c r="H10">
-        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F14="","",'2 Matériel'!$F14)),"")</f>
+        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F14="","",'2 Matériel'!$F14)),"")</f>
         <v/>
       </c>
       <c r="I10">
-        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G14="","",'2 Matériel'!$G14)),"")</f>
+        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G14="","",'2 Matériel'!$G14)),"")</f>
         <v/>
       </c>
       <c r="J10">
-        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H14="","",'2 Matériel'!$H14)),"")</f>
+        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H14="","",'2 Matériel'!$H14)),"")</f>
         <v/>
       </c>
       <c r="K10">
-        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I14="","",'2 Matériel'!$I14)),"")</f>
+        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I14="","",'2 Matériel'!$I14)),"")</f>
         <v/>
       </c>
       <c r="L10">
-        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J14="","",'2 Matériel'!$J14)),"")</f>
+        <f>IF(C10="ITM",IF(AND(AND('2 Matériel'!$K14="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J14="","",'2 Matériel'!$J14)),"")</f>
         <v/>
       </c>
     </row>
@@ -6667,7 +6737,7 @@
         <v/>
       </c>
       <c r="E11">
-        <f>IF(C11="BAN",UPPER('2 Matériel'!$C15),IF(C11="ITM",'2 Matériel'!$C15&amp;IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C11="BAN",UPPER('2 Matériel'!$C15),IF(C11="ITM",'2 Matériel'!$C15&amp;IF(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F11">
@@ -6675,27 +6745,27 @@
         <v/>
       </c>
       <c r="G11">
-        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E15="","",'2 Matériel'!$E15)),"")</f>
+        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E15="","",'2 Matériel'!$E15)),"")</f>
         <v/>
       </c>
       <c r="H11">
-        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F15="","",'2 Matériel'!$F15)),"")</f>
+        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F15="","",'2 Matériel'!$F15)),"")</f>
         <v/>
       </c>
       <c r="I11">
-        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G15="","",'2 Matériel'!$G15)),"")</f>
+        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G15="","",'2 Matériel'!$G15)),"")</f>
         <v/>
       </c>
       <c r="J11">
-        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H15="","",'2 Matériel'!$H15)),"")</f>
+        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H15="","",'2 Matériel'!$H15)),"")</f>
         <v/>
       </c>
       <c r="K11">
-        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I15="","",'2 Matériel'!$I15)),"")</f>
+        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I15="","",'2 Matériel'!$I15)),"")</f>
         <v/>
       </c>
       <c r="L11">
-        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J15="","",'2 Matériel'!$J15)),"")</f>
+        <f>IF(C11="ITM",IF(AND(AND('2 Matériel'!$K15="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J15="","",'2 Matériel'!$J15)),"")</f>
         <v/>
       </c>
     </row>
@@ -6717,7 +6787,7 @@
         <v/>
       </c>
       <c r="E12">
-        <f>IF(C12="BAN",UPPER('2 Matériel'!$C16),IF(C12="ITM",'2 Matériel'!$C16&amp;IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C12="BAN",UPPER('2 Matériel'!$C16),IF(C12="ITM",'2 Matériel'!$C16&amp;IF(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F12">
@@ -6725,27 +6795,27 @@
         <v/>
       </c>
       <c r="G12">
-        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E16="","",'2 Matériel'!$E16)),"")</f>
+        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E16="","",'2 Matériel'!$E16)),"")</f>
         <v/>
       </c>
       <c r="H12">
-        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F16="","",'2 Matériel'!$F16)),"")</f>
+        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F16="","",'2 Matériel'!$F16)),"")</f>
         <v/>
       </c>
       <c r="I12">
-        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G16="","",'2 Matériel'!$G16)),"")</f>
+        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G16="","",'2 Matériel'!$G16)),"")</f>
         <v/>
       </c>
       <c r="J12">
-        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H16="","",'2 Matériel'!$H16)),"")</f>
+        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H16="","",'2 Matériel'!$H16)),"")</f>
         <v/>
       </c>
       <c r="K12">
-        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I16="","",'2 Matériel'!$I16)),"")</f>
+        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I16="","",'2 Matériel'!$I16)),"")</f>
         <v/>
       </c>
       <c r="L12">
-        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J16="","",'2 Matériel'!$J16)),"")</f>
+        <f>IF(C12="ITM",IF(AND(AND('2 Matériel'!$K16="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J16="","",'2 Matériel'!$J16)),"")</f>
         <v/>
       </c>
     </row>
@@ -6767,7 +6837,7 @@
         <v/>
       </c>
       <c r="E13">
-        <f>IF(C13="BAN",UPPER('2 Matériel'!$C17),IF(C13="ITM",'2 Matériel'!$C17&amp;IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C13="BAN",UPPER('2 Matériel'!$C17),IF(C13="ITM",'2 Matériel'!$C17&amp;IF(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F13">
@@ -6775,27 +6845,27 @@
         <v/>
       </c>
       <c r="G13">
-        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E17="","",'2 Matériel'!$E17)),"")</f>
+        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E17="","",'2 Matériel'!$E17)),"")</f>
         <v/>
       </c>
       <c r="H13">
-        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F17="","",'2 Matériel'!$F17)),"")</f>
+        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F17="","",'2 Matériel'!$F17)),"")</f>
         <v/>
       </c>
       <c r="I13">
-        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G17="","",'2 Matériel'!$G17)),"")</f>
+        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G17="","",'2 Matériel'!$G17)),"")</f>
         <v/>
       </c>
       <c r="J13">
-        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H17="","",'2 Matériel'!$H17)),"")</f>
+        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H17="","",'2 Matériel'!$H17)),"")</f>
         <v/>
       </c>
       <c r="K13">
-        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I17="","",'2 Matériel'!$I17)),"")</f>
+        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I17="","",'2 Matériel'!$I17)),"")</f>
         <v/>
       </c>
       <c r="L13">
-        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J17="","",'2 Matériel'!$J17)),"")</f>
+        <f>IF(C13="ITM",IF(AND(AND('2 Matériel'!$K17="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J17="","",'2 Matériel'!$J17)),"")</f>
         <v/>
       </c>
     </row>
@@ -6817,7 +6887,7 @@
         <v/>
       </c>
       <c r="E14">
-        <f>IF(C14="BAN",UPPER('2 Matériel'!$C18),IF(C14="ITM",'2 Matériel'!$C18&amp;IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C14="BAN",UPPER('2 Matériel'!$C18),IF(C14="ITM",'2 Matériel'!$C18&amp;IF(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F14">
@@ -6825,27 +6895,27 @@
         <v/>
       </c>
       <c r="G14">
-        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E18="","",'2 Matériel'!$E18)),"")</f>
+        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E18="","",'2 Matériel'!$E18)),"")</f>
         <v/>
       </c>
       <c r="H14">
-        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F18="","",'2 Matériel'!$F18)),"")</f>
+        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F18="","",'2 Matériel'!$F18)),"")</f>
         <v/>
       </c>
       <c r="I14">
-        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G18="","",'2 Matériel'!$G18)),"")</f>
+        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G18="","",'2 Matériel'!$G18)),"")</f>
         <v/>
       </c>
       <c r="J14">
-        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H18="","",'2 Matériel'!$H18)),"")</f>
+        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H18="","",'2 Matériel'!$H18)),"")</f>
         <v/>
       </c>
       <c r="K14">
-        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I18="","",'2 Matériel'!$I18)),"")</f>
+        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I18="","",'2 Matériel'!$I18)),"")</f>
         <v/>
       </c>
       <c r="L14">
-        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J18="","",'2 Matériel'!$J18)),"")</f>
+        <f>IF(C14="ITM",IF(AND(AND('2 Matériel'!$K18="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J18="","",'2 Matériel'!$J18)),"")</f>
         <v/>
       </c>
     </row>
@@ -6867,7 +6937,7 @@
         <v/>
       </c>
       <c r="E15">
-        <f>IF(C15="BAN",UPPER('2 Matériel'!$C19),IF(C15="ITM",'2 Matériel'!$C19&amp;IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C15="BAN",UPPER('2 Matériel'!$C19),IF(C15="ITM",'2 Matériel'!$C19&amp;IF(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F15">
@@ -6875,27 +6945,27 @@
         <v/>
       </c>
       <c r="G15">
-        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E19="","",'2 Matériel'!$E19)),"")</f>
+        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E19="","",'2 Matériel'!$E19)),"")</f>
         <v/>
       </c>
       <c r="H15">
-        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F19="","",'2 Matériel'!$F19)),"")</f>
+        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F19="","",'2 Matériel'!$F19)),"")</f>
         <v/>
       </c>
       <c r="I15">
-        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G19="","",'2 Matériel'!$G19)),"")</f>
+        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G19="","",'2 Matériel'!$G19)),"")</f>
         <v/>
       </c>
       <c r="J15">
-        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H19="","",'2 Matériel'!$H19)),"")</f>
+        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H19="","",'2 Matériel'!$H19)),"")</f>
         <v/>
       </c>
       <c r="K15">
-        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I19="","",'2 Matériel'!$I19)),"")</f>
+        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I19="","",'2 Matériel'!$I19)),"")</f>
         <v/>
       </c>
       <c r="L15">
-        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J19="","",'2 Matériel'!$J19)),"")</f>
+        <f>IF(C15="ITM",IF(AND(AND('2 Matériel'!$K19="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J19="","",'2 Matériel'!$J19)),"")</f>
         <v/>
       </c>
     </row>
@@ -6917,7 +6987,7 @@
         <v/>
       </c>
       <c r="E16">
-        <f>IF(C16="BAN",UPPER('2 Matériel'!$C20),IF(C16="ITM",'2 Matériel'!$C20&amp;IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C16="BAN",UPPER('2 Matériel'!$C20),IF(C16="ITM",'2 Matériel'!$C20&amp;IF(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F16">
@@ -6925,27 +6995,27 @@
         <v/>
       </c>
       <c r="G16">
-        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E20="","",'2 Matériel'!$E20)),"")</f>
+        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E20="","",'2 Matériel'!$E20)),"")</f>
         <v/>
       </c>
       <c r="H16">
-        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F20="","",'2 Matériel'!$F20)),"")</f>
+        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F20="","",'2 Matériel'!$F20)),"")</f>
         <v/>
       </c>
       <c r="I16">
-        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G20="","",'2 Matériel'!$G20)),"")</f>
+        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G20="","",'2 Matériel'!$G20)),"")</f>
         <v/>
       </c>
       <c r="J16">
-        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H20="","",'2 Matériel'!$H20)),"")</f>
+        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H20="","",'2 Matériel'!$H20)),"")</f>
         <v/>
       </c>
       <c r="K16">
-        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I20="","",'2 Matériel'!$I20)),"")</f>
+        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I20="","",'2 Matériel'!$I20)),"")</f>
         <v/>
       </c>
       <c r="L16">
-        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J20="","",'2 Matériel'!$J20)),"")</f>
+        <f>IF(C16="ITM",IF(AND(AND('2 Matériel'!$K20="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J20="","",'2 Matériel'!$J20)),"")</f>
         <v/>
       </c>
     </row>
@@ -6967,7 +7037,7 @@
         <v/>
       </c>
       <c r="E17">
-        <f>IF(C17="BAN",UPPER('2 Matériel'!$C21),IF(C17="ITM",'2 Matériel'!$C21&amp;IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C17="BAN",UPPER('2 Matériel'!$C21),IF(C17="ITM",'2 Matériel'!$C21&amp;IF(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F17">
@@ -6975,27 +7045,27 @@
         <v/>
       </c>
       <c r="G17">
-        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E21="","",'2 Matériel'!$E21)),"")</f>
+        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E21="","",'2 Matériel'!$E21)),"")</f>
         <v/>
       </c>
       <c r="H17">
-        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F21="","",'2 Matériel'!$F21)),"")</f>
+        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F21="","",'2 Matériel'!$F21)),"")</f>
         <v/>
       </c>
       <c r="I17">
-        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G21="","",'2 Matériel'!$G21)),"")</f>
+        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G21="","",'2 Matériel'!$G21)),"")</f>
         <v/>
       </c>
       <c r="J17">
-        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H21="","",'2 Matériel'!$H21)),"")</f>
+        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H21="","",'2 Matériel'!$H21)),"")</f>
         <v/>
       </c>
       <c r="K17">
-        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I21="","",'2 Matériel'!$I21)),"")</f>
+        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I21="","",'2 Matériel'!$I21)),"")</f>
         <v/>
       </c>
       <c r="L17">
-        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J21="","",'2 Matériel'!$J21)),"")</f>
+        <f>IF(C17="ITM",IF(AND(AND('2 Matériel'!$K21="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J21="","",'2 Matériel'!$J21)),"")</f>
         <v/>
       </c>
     </row>
@@ -7017,7 +7087,7 @@
         <v/>
       </c>
       <c r="E18">
-        <f>IF(C18="BAN",UPPER('2 Matériel'!$C22),IF(C18="ITM",'2 Matériel'!$C22&amp;IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C18="BAN",UPPER('2 Matériel'!$C22),IF(C18="ITM",'2 Matériel'!$C22&amp;IF(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F18">
@@ -7025,27 +7095,27 @@
         <v/>
       </c>
       <c r="G18">
-        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E22="","",'2 Matériel'!$E22)),"")</f>
+        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E22="","",'2 Matériel'!$E22)),"")</f>
         <v/>
       </c>
       <c r="H18">
-        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F22="","",'2 Matériel'!$F22)),"")</f>
+        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F22="","",'2 Matériel'!$F22)),"")</f>
         <v/>
       </c>
       <c r="I18">
-        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G22="","",'2 Matériel'!$G22)),"")</f>
+        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G22="","",'2 Matériel'!$G22)),"")</f>
         <v/>
       </c>
       <c r="J18">
-        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H22="","",'2 Matériel'!$H22)),"")</f>
+        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H22="","",'2 Matériel'!$H22)),"")</f>
         <v/>
       </c>
       <c r="K18">
-        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I22="","",'2 Matériel'!$I22)),"")</f>
+        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I22="","",'2 Matériel'!$I22)),"")</f>
         <v/>
       </c>
       <c r="L18">
-        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J22="","",'2 Matériel'!$J22)),"")</f>
+        <f>IF(C18="ITM",IF(AND(AND('2 Matériel'!$K22="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J22="","",'2 Matériel'!$J22)),"")</f>
         <v/>
       </c>
     </row>
@@ -7067,7 +7137,7 @@
         <v/>
       </c>
       <c r="E19">
-        <f>IF(C19="BAN",UPPER('2 Matériel'!$C23),IF(C19="ITM",'2 Matériel'!$C23&amp;IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C19="BAN",UPPER('2 Matériel'!$C23),IF(C19="ITM",'2 Matériel'!$C23&amp;IF(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F19">
@@ -7075,27 +7145,27 @@
         <v/>
       </c>
       <c r="G19">
-        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E23="","",'2 Matériel'!$E23)),"")</f>
+        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E23="","",'2 Matériel'!$E23)),"")</f>
         <v/>
       </c>
       <c r="H19">
-        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F23="","",'2 Matériel'!$F23)),"")</f>
+        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F23="","",'2 Matériel'!$F23)),"")</f>
         <v/>
       </c>
       <c r="I19">
-        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G23="","",'2 Matériel'!$G23)),"")</f>
+        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G23="","",'2 Matériel'!$G23)),"")</f>
         <v/>
       </c>
       <c r="J19">
-        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H23="","",'2 Matériel'!$H23)),"")</f>
+        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H23="","",'2 Matériel'!$H23)),"")</f>
         <v/>
       </c>
       <c r="K19">
-        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I23="","",'2 Matériel'!$I23)),"")</f>
+        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I23="","",'2 Matériel'!$I23)),"")</f>
         <v/>
       </c>
       <c r="L19">
-        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J23="","",'2 Matériel'!$J23)),"")</f>
+        <f>IF(C19="ITM",IF(AND(AND('2 Matériel'!$K23="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J23="","",'2 Matériel'!$J23)),"")</f>
         <v/>
       </c>
     </row>
@@ -7117,7 +7187,7 @@
         <v/>
       </c>
       <c r="E20">
-        <f>IF(C20="BAN",UPPER('2 Matériel'!$C24),IF(C20="ITM",'2 Matériel'!$C24&amp;IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C20="BAN",UPPER('2 Matériel'!$C24),IF(C20="ITM",'2 Matériel'!$C24&amp;IF(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F20">
@@ -7125,27 +7195,27 @@
         <v/>
       </c>
       <c r="G20">
-        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E24="","",'2 Matériel'!$E24)),"")</f>
+        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E24="","",'2 Matériel'!$E24)),"")</f>
         <v/>
       </c>
       <c r="H20">
-        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F24="","",'2 Matériel'!$F24)),"")</f>
+        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F24="","",'2 Matériel'!$F24)),"")</f>
         <v/>
       </c>
       <c r="I20">
-        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G24="","",'2 Matériel'!$G24)),"")</f>
+        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G24="","",'2 Matériel'!$G24)),"")</f>
         <v/>
       </c>
       <c r="J20">
-        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H24="","",'2 Matériel'!$H24)),"")</f>
+        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H24="","",'2 Matériel'!$H24)),"")</f>
         <v/>
       </c>
       <c r="K20">
-        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I24="","",'2 Matériel'!$I24)),"")</f>
+        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I24="","",'2 Matériel'!$I24)),"")</f>
         <v/>
       </c>
       <c r="L20">
-        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J24="","",'2 Matériel'!$J24)),"")</f>
+        <f>IF(C20="ITM",IF(AND(AND('2 Matériel'!$K24="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J24="","",'2 Matériel'!$J24)),"")</f>
         <v/>
       </c>
     </row>
@@ -7167,7 +7237,7 @@
         <v/>
       </c>
       <c r="E21">
-        <f>IF(C21="BAN",UPPER('2 Matériel'!$C25),IF(C21="ITM",'2 Matériel'!$C25&amp;IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C21="BAN",UPPER('2 Matériel'!$C25),IF(C21="ITM",'2 Matériel'!$C25&amp;IF(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F21">
@@ -7175,27 +7245,27 @@
         <v/>
       </c>
       <c r="G21">
-        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E25="","",'2 Matériel'!$E25)),"")</f>
+        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E25="","",'2 Matériel'!$E25)),"")</f>
         <v/>
       </c>
       <c r="H21">
-        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F25="","",'2 Matériel'!$F25)),"")</f>
+        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F25="","",'2 Matériel'!$F25)),"")</f>
         <v/>
       </c>
       <c r="I21">
-        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G25="","",'2 Matériel'!$G25)),"")</f>
+        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G25="","",'2 Matériel'!$G25)),"")</f>
         <v/>
       </c>
       <c r="J21">
-        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H25="","",'2 Matériel'!$H25)),"")</f>
+        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H25="","",'2 Matériel'!$H25)),"")</f>
         <v/>
       </c>
       <c r="K21">
-        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I25="","",'2 Matériel'!$I25)),"")</f>
+        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I25="","",'2 Matériel'!$I25)),"")</f>
         <v/>
       </c>
       <c r="L21">
-        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J25="","",'2 Matériel'!$J25)),"")</f>
+        <f>IF(C21="ITM",IF(AND(AND('2 Matériel'!$K25="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J25="","",'2 Matériel'!$J25)),"")</f>
         <v/>
       </c>
     </row>
@@ -7217,7 +7287,7 @@
         <v/>
       </c>
       <c r="E22">
-        <f>IF(C22="BAN",UPPER('2 Matériel'!$C26),IF(C22="ITM",'2 Matériel'!$C26&amp;IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C22="BAN",UPPER('2 Matériel'!$C26),IF(C22="ITM",'2 Matériel'!$C26&amp;IF(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F22">
@@ -7225,27 +7295,27 @@
         <v/>
       </c>
       <c r="G22">
-        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E26="","",'2 Matériel'!$E26)),"")</f>
+        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E26="","",'2 Matériel'!$E26)),"")</f>
         <v/>
       </c>
       <c r="H22">
-        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F26="","",'2 Matériel'!$F26)),"")</f>
+        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F26="","",'2 Matériel'!$F26)),"")</f>
         <v/>
       </c>
       <c r="I22">
-        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G26="","",'2 Matériel'!$G26)),"")</f>
+        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G26="","",'2 Matériel'!$G26)),"")</f>
         <v/>
       </c>
       <c r="J22">
-        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H26="","",'2 Matériel'!$H26)),"")</f>
+        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H26="","",'2 Matériel'!$H26)),"")</f>
         <v/>
       </c>
       <c r="K22">
-        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I26="","",'2 Matériel'!$I26)),"")</f>
+        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I26="","",'2 Matériel'!$I26)),"")</f>
         <v/>
       </c>
       <c r="L22">
-        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J26="","",'2 Matériel'!$J26)),"")</f>
+        <f>IF(C22="ITM",IF(AND(AND('2 Matériel'!$K26="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J26="","",'2 Matériel'!$J26)),"")</f>
         <v/>
       </c>
     </row>
@@ -7267,7 +7337,7 @@
         <v/>
       </c>
       <c r="E23">
-        <f>IF(C23="BAN",UPPER('2 Matériel'!$C27),IF(C23="ITM",'2 Matériel'!$C27&amp;IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C23="BAN",UPPER('2 Matériel'!$C27),IF(C23="ITM",'2 Matériel'!$C27&amp;IF(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F23">
@@ -7275,27 +7345,27 @@
         <v/>
       </c>
       <c r="G23">
-        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E27="","",'2 Matériel'!$E27)),"")</f>
+        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E27="","",'2 Matériel'!$E27)),"")</f>
         <v/>
       </c>
       <c r="H23">
-        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F27="","",'2 Matériel'!$F27)),"")</f>
+        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F27="","",'2 Matériel'!$F27)),"")</f>
         <v/>
       </c>
       <c r="I23">
-        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G27="","",'2 Matériel'!$G27)),"")</f>
+        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G27="","",'2 Matériel'!$G27)),"")</f>
         <v/>
       </c>
       <c r="J23">
-        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H27="","",'2 Matériel'!$H27)),"")</f>
+        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H27="","",'2 Matériel'!$H27)),"")</f>
         <v/>
       </c>
       <c r="K23">
-        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I27="","",'2 Matériel'!$I27)),"")</f>
+        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I27="","",'2 Matériel'!$I27)),"")</f>
         <v/>
       </c>
       <c r="L23">
-        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J27="","",'2 Matériel'!$J27)),"")</f>
+        <f>IF(C23="ITM",IF(AND(AND('2 Matériel'!$K27="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J27="","",'2 Matériel'!$J27)),"")</f>
         <v/>
       </c>
     </row>
@@ -7317,7 +7387,7 @@
         <v/>
       </c>
       <c r="E24">
-        <f>IF(C24="BAN",UPPER('2 Matériel'!$C28),IF(C24="ITM",'2 Matériel'!$C28&amp;IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C24="BAN",UPPER('2 Matériel'!$C28),IF(C24="ITM",'2 Matériel'!$C28&amp;IF(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F24">
@@ -7325,27 +7395,27 @@
         <v/>
       </c>
       <c r="G24">
-        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E28="","",'2 Matériel'!$E28)),"")</f>
+        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E28="","",'2 Matériel'!$E28)),"")</f>
         <v/>
       </c>
       <c r="H24">
-        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F28="","",'2 Matériel'!$F28)),"")</f>
+        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F28="","",'2 Matériel'!$F28)),"")</f>
         <v/>
       </c>
       <c r="I24">
-        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G28="","",'2 Matériel'!$G28)),"")</f>
+        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G28="","",'2 Matériel'!$G28)),"")</f>
         <v/>
       </c>
       <c r="J24">
-        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H28="","",'2 Matériel'!$H28)),"")</f>
+        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H28="","",'2 Matériel'!$H28)),"")</f>
         <v/>
       </c>
       <c r="K24">
-        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I28="","",'2 Matériel'!$I28)),"")</f>
+        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I28="","",'2 Matériel'!$I28)),"")</f>
         <v/>
       </c>
       <c r="L24">
-        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J28="","",'2 Matériel'!$J28)),"")</f>
+        <f>IF(C24="ITM",IF(AND(AND('2 Matériel'!$K28="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J28="","",'2 Matériel'!$J28)),"")</f>
         <v/>
       </c>
     </row>
@@ -7367,7 +7437,7 @@
         <v/>
       </c>
       <c r="E25">
-        <f>IF(C25="BAN",UPPER('2 Matériel'!$C29),IF(C25="ITM",'2 Matériel'!$C29&amp;IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),""),""))</f>
+        <f>IF(C25="BAN",UPPER('2 Matériel'!$C29),IF(C25="ITM",'2 Matériel'!$C29&amp;IF(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),""),""))</f>
         <v/>
       </c>
       <c r="F25">
@@ -7375,27 +7445,27 @@
         <v/>
       </c>
       <c r="G25">
-        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$E29="","",'2 Matériel'!$E29)),"")</f>
+        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$E29="","",'2 Matériel'!$E29)),"")</f>
         <v/>
       </c>
       <c r="H25">
-        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$F29="","",'2 Matériel'!$F29)),"")</f>
+        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$F29="","",'2 Matériel'!$F29)),"")</f>
         <v/>
       </c>
       <c r="I25">
-        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$G29="","",'2 Matériel'!$G29)),"")</f>
+        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$G29="","",'2 Matériel'!$G29)),"")</f>
         <v/>
       </c>
       <c r="J25">
-        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$H29="","",'2 Matériel'!$H29)),"")</f>
+        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$H29="","",'2 Matériel'!$H29)),"")</f>
         <v/>
       </c>
       <c r="K25">
-        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$I29="","",'2 Matériel'!$I29)),"")</f>
+        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$I29="","",'2 Matériel'!$I29)),"")</f>
         <v/>
       </c>
       <c r="L25">
-        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('2 Matériel'!$J29="","",'2 Matériel'!$J29)),"")</f>
+        <f>IF(C25="ITM",IF(AND(AND('2 Matériel'!$K29="Oui",'3 Options'!$C$13="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('2 Matériel'!$J29="","",'2 Matériel'!$J29)),"")</f>
         <v/>
       </c>
     </row>
@@ -7417,23 +7487,23 @@
         <v/>
       </c>
       <c r="E26">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sec_tight",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sec_tight",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="F26">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_qty",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="G26">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_unit",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_unit",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="H26">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_pu",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_pu",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="I26">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_tot",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_tot",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="J26">
@@ -7467,7 +7537,7 @@
         <v/>
       </c>
       <c r="E27">
-        <f>IF('3 Options'!$D$8&lt;&gt;"",'3 Options'!$D$8,INDEX(Textes!$B$2:$C$55,MATCH("tight",Textes!$A$2:$A$55,0),Listes!$H$1))&amp;IF(AND('3 Options'!$C$13="Oui",'3 Options'!$C$19="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
+        <f>IF('3 Options'!$D$8&lt;&gt;"",'3 Options'!$D$8,INDEX(Textes!$B$2:$C$59,MATCH("tight",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(AND('3 Options'!$C$13="Oui",'3 Options'!$C$19="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),"")</f>
         <v/>
       </c>
       <c r="F27">
@@ -7479,11 +7549,11 @@
         <v/>
       </c>
       <c r="H27">
-        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$19="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$8="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$8="","",'3 Options'!$F$8)))</f>
+        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$19="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$8="Coût réel +15 %",INDEX(Textes!$B$2:$C$59,MATCH("at_cost",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$F$8="","",'3 Options'!$F$8)))</f>
         <v/>
       </c>
       <c r="I27">
-        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$19="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$8="Coût réel +15 %","—",'3 Options'!$H$8))</f>
+        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$19="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$8="Coût réel +15 %","—",'3 Options'!$H$8))</f>
         <v/>
       </c>
       <c r="J27">
@@ -7517,23 +7587,23 @@
         <v/>
       </c>
       <c r="E28">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sec_tr",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sec_tr",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="F28">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_qty",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="G28">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_unit",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_unit",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="H28">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_pu",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_pu",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="I28">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_tot",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_tot",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="J28">
@@ -7567,7 +7637,7 @@
         <v/>
       </c>
       <c r="E29">
-        <f>IF('3 Options'!$D$9&lt;&gt;"",'3 Options'!$D$9,INDEX(Textes!$B$2:$C$55,MATCH("tr_mob",Textes!$A$2:$A$55,0),Listes!$H$1))&amp;IF(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
+        <f>IF('3 Options'!$D$9&lt;&gt;"",'3 Options'!$D$9,INDEX(Textes!$B$2:$C$59,MATCH("tr_mob",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),"")</f>
         <v/>
       </c>
       <c r="F29">
@@ -7579,11 +7649,11 @@
         <v/>
       </c>
       <c r="H29">
-        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$9="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$9="","",'3 Options'!$F$9)))</f>
+        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$9="Coût réel +15 %",INDEX(Textes!$B$2:$C$59,MATCH("at_cost",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$F$9="","",'3 Options'!$F$9)))</f>
         <v/>
       </c>
       <c r="I29">
-        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$9="Coût réel +15 %","—",'3 Options'!$H$9))</f>
+        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$9="Coût réel +15 %","—",'3 Options'!$H$9))</f>
         <v/>
       </c>
       <c r="J29">
@@ -7617,7 +7687,7 @@
         <v/>
       </c>
       <c r="E30">
-        <f>IF('3 Options'!$D$10&lt;&gt;"",'3 Options'!$D$10,INDEX(Textes!$B$2:$C$55,MATCH("tr_dem",Textes!$A$2:$A$55,0),Listes!$H$1))&amp;IF(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
+        <f>IF('3 Options'!$D$10&lt;&gt;"",'3 Options'!$D$10,INDEX(Textes!$B$2:$C$59,MATCH("tr_dem",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),"")</f>
         <v/>
       </c>
       <c r="F30">
@@ -7629,11 +7699,11 @@
         <v/>
       </c>
       <c r="H30">
-        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$10="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$10="","",'3 Options'!$F$10)))</f>
+        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$10="Coût réel +15 %",INDEX(Textes!$B$2:$C$59,MATCH("at_cost",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$F$10="","",'3 Options'!$F$10)))</f>
         <v/>
       </c>
       <c r="I30">
-        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$10="Coût réel +15 %","—",'3 Options'!$H$10))</f>
+        <f>IF(AND(AND('3 Options'!$C$13="Oui",'3 Options'!$C$20="Oui"),'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$10="Coût réel +15 %","—",'3 Options'!$H$10))</f>
         <v/>
       </c>
       <c r="J30">
@@ -7667,23 +7737,23 @@
         <v/>
       </c>
       <c r="E31">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("sec_op",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("sec_op",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="F31">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_qty",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_qty",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="G31">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_unit",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_unit",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="H31">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_pu",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_pu",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="I31">
-        <f>INDEX(Textes!$B$2:$C$55,MATCH("h_tot",Textes!$A$2:$A$55,0),Listes!$H$1)</f>
+        <f>INDEX(Textes!$B$2:$C$59,MATCH("h_tot",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
       <c r="J31">
@@ -7717,7 +7787,7 @@
         <v/>
       </c>
       <c r="E32">
-        <f>IF('3 Options'!$D$6&lt;&gt;"",'3 Options'!$D$6,INDEX(Textes!$B$2:$C$55,MATCH("op_day",Textes!$A$2:$A$55,0),Listes!$H$1))&amp;IF(FALSE,"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
+        <f>IF('3 Options'!$D$6&lt;&gt;"",'3 Options'!$D$6,INDEX(Textes!$B$2:$C$59,MATCH("op_day",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(FALSE,"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),"")</f>
         <v/>
       </c>
       <c r="F32">
@@ -7729,11 +7799,11 @@
         <v/>
       </c>
       <c r="H32">
-        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$6="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$6="","",'3 Options'!$F$6)))</f>
+        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$6="Coût réel +15 %",INDEX(Textes!$B$2:$C$59,MATCH("at_cost",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$F$6="","",'3 Options'!$F$6)))</f>
         <v/>
       </c>
       <c r="I32">
-        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$6="Coût réel +15 %","—",'3 Options'!$H$6))</f>
+        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$6="Coût réel +15 %","—",'3 Options'!$H$6))</f>
         <v/>
       </c>
       <c r="J32">
@@ -7767,7 +7837,7 @@
         <v/>
       </c>
       <c r="E33">
-        <f>IF('3 Options'!$D$7&lt;&gt;"",'3 Options'!$D$7,INDEX(Textes!$B$2:$C$55,MATCH("op_mob",Textes!$A$2:$A$55,0),Listes!$H$1))&amp;IF(FALSE,"  ·  "&amp;INDEX(Textes!$B$2:$C$55,MATCH("incl_long",Textes!$A$2:$A$55,0),Listes!$H$1),"")</f>
+        <f>IF('3 Options'!$D$7&lt;&gt;"",'3 Options'!$D$7,INDEX(Textes!$B$2:$C$59,MATCH("op_mob",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(FALSE,"  ·  "&amp;INDEX(Textes!$B$2:$C$59,MATCH("incl_long",Textes!$A$2:$A$59,0),Listes!$H$1),"")</f>
         <v/>
       </c>
       <c r="F33">
@@ -7779,11 +7849,11 @@
         <v/>
       </c>
       <c r="H33">
-        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$7="Coût réel +15 %",INDEX(Textes!$B$2:$C$55,MATCH("at_cost",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$F$7="","",'3 Options'!$F$7)))</f>
+        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$7="Coût réel +15 %",INDEX(Textes!$B$2:$C$59,MATCH("at_cost",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$F$7="","",'3 Options'!$F$7)))</f>
         <v/>
       </c>
       <c r="I33">
-        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$55,MATCH("incl",Textes!$A$2:$A$55,0),Listes!$H$1),IF('3 Options'!$G$7="Coût réel +15 %","—",'3 Options'!$H$7))</f>
+        <f>IF(AND(FALSE,'3 Options'!$C$18&lt;&gt;"Oui"),INDEX(Textes!$B$2:$C$59,MATCH("incl",Textes!$A$2:$A$59,0),Listes!$H$1),IF('3 Options'!$G$7="Coût réel +15 %","—",'3 Options'!$H$7))</f>
         <v/>
       </c>
       <c r="J33">
@@ -7817,7 +7887,7 @@
         <v/>
       </c>
       <c r="E34">
-        <f>UPPER(INDEX(Textes!$B$2:$C$55,MATCH("forfait",Textes!$A$2:$A$55,0),Listes!$H$1))&amp;IF('3 Options'!$D$13&lt;&gt;"","   ·   "&amp;'3 Options'!$D$13,"")</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("forfait",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(IF('3 Options'!$G$13="Forfait calculé (S + O + UC)",'3 Options'!$C$15+'3 Options'!$C$16,IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13,""))&lt;&gt;"","  "&amp;IF('3 Options'!$G$13="Forfait calculé (S + O + UC)",'3 Options'!$C$15+'3 Options'!$C$16,IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13,""))&amp;" "&amp;INDEX(Textes!$B$2:$C$59,MATCH("days",Textes!$A$2:$A$59,0),Listes!$H$1),"")&amp;IF('3 Options'!$D$13&lt;&gt;"","   ·   "&amp;'3 Options'!$D$13,"")</f>
         <v/>
       </c>
       <c r="F34">
@@ -7851,7 +7921,7 @@
     </row>
     <row r="35">
       <c r="A35">
-        <f>IF(AND('3 Options'!$C$13="Oui",OR('3 Options'!$D$14&lt;&gt;"",'3 Options'!$G$13="Forfait par jour")),1,0)</f>
+        <f>IF(AND('3 Options'!$C$13="Oui",E35&lt;&gt;""),1,0)</f>
         <v/>
       </c>
       <c r="B35">
@@ -7867,7 +7937,7 @@
         <v/>
       </c>
       <c r="E35">
-        <f>IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13&amp;" j × "&amp;TEXT('3 Options'!$F$13,"#,##0.00")&amp;" €/j"&amp;IF('3 Options'!$D$14&lt;&gt;"","   ·   "&amp;'3 Options'!$D$14,""),'3 Options'!$D$14)</f>
+        <f>IF(AND(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui")),INDEX(Textes!$B$2:$C$59,MATCH("in_both",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tight",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tr",Textes!$A$2:$A$59,0),Listes!$H$1),"")))&amp;IF(AND(IF(AND(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui")),INDEX(Textes!$B$2:$C$59,MATCH("in_both",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tight",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tr",Textes!$A$2:$A$59,0),Listes!$H$1),"")))&lt;&gt;"",'3 Options'!$D$14&lt;&gt;""),"   ·   ","")&amp;'3 Options'!$D$14</f>
         <v/>
       </c>
       <c r="F35">

</xml_diff>

<commit_message>
Devis 2027 : lignes vides masquées par filtre, conditions juste après le forfait, forfait N jours avec serrage et transport compris
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/devis_2027/Devis_Enedril_2027.xlsx
+++ b/devis_2027/Devis_Enedril_2027.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flux" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Devis'!$B$15:$N$55</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'4 Devis'!$A$1:$K$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -409,6 +410,9 @@
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -419,6 +423,7 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -430,10 +435,6 @@
     </xf>
     <xf numFmtId="4" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
@@ -2468,19 +2469,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
     <col width="4.5" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="5.5" customWidth="1" min="4" max="4"/>
-    <col width="10.5" customWidth="1" min="5" max="5"/>
-    <col width="10.5" customWidth="1" min="6" max="6"/>
-    <col width="10.5" customWidth="1" min="7" max="7"/>
-    <col width="12.5" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="9.5" customWidth="1" min="9" max="9"/>
+    <col width="9.5" customWidth="1" min="10" max="10"/>
     <col width="1.5" customWidth="1" min="11" max="11"/>
     <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
     <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
@@ -2656,1921 +2657,2096 @@
       <c r="I12" s="33" t="n"/>
       <c r="J12" s="33" t="n"/>
     </row>
-    <row r="13" ht="8" customHeight="1"/>
+    <row r="13" ht="14" customHeight="1">
+      <c r="B13" s="34">
+        <f>IF(SUBTOTAL(103,B16:B55)&lt;&gt;SUM(N16:N55),"⚠  Appuyer sur Ctrl + Alt + L pour mettre à jour les lignes du devis (matériel ou options modifiés).","")</f>
+        <v/>
+      </c>
+    </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="34">
+      <c r="B14" s="35">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("sec_eq",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="C14" s="35" t="n"/>
-      <c r="D14" s="35" t="n"/>
-      <c r="E14" s="35" t="n"/>
-      <c r="F14" s="35" t="n"/>
-      <c r="G14" s="35" t="n"/>
-      <c r="H14" s="35" t="n"/>
-      <c r="I14" s="35" t="n"/>
-      <c r="J14" s="35" t="n"/>
+      <c r="C14" s="36" t="n"/>
+      <c r="D14" s="36" t="n"/>
+      <c r="E14" s="36" t="n"/>
+      <c r="F14" s="36" t="n"/>
+      <c r="G14" s="36" t="n"/>
+      <c r="H14" s="36" t="n"/>
+      <c r="I14" s="36" t="n"/>
+      <c r="J14" s="36" t="n"/>
     </row>
     <row r="15" ht="46" customHeight="1">
-      <c r="B15" s="36">
+      <c r="B15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_n",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="C15" s="37">
+      <c r="C15" s="38">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_desc",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="D15" s="36">
+      <c r="D15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_qty",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_s",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="F15" s="36">
+      <c r="F15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_o",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="G15" s="36">
+      <c r="G15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_uc",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="H15" s="36">
+      <c r="H15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_lih",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="I15" s="36">
+      <c r="I15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_insp",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="J15" s="36">
+      <c r="J15" s="37">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("h_rest",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
+      <c r="L15" s="39" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="M15" s="39" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="N15" s="39" t="inlineStr">
+        <is>
+          <t>actif</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="38">
-        <f>IF($L16="","",INDEX(Flux!$D$2:$D$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="C16" s="39">
-        <f>IF($L16="","",INDEX(Flux!$E$2:$E$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="D16" s="40">
-        <f>IF($L16="","",INDEX(Flux!$F$2:$F$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="E16" s="41">
-        <f>IF($L16="","",INDEX(Flux!$G$2:$G$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="F16" s="41">
-        <f>IF($L16="","",INDEX(Flux!$H$2:$H$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="G16" s="41">
-        <f>IF($L16="","",INDEX(Flux!$I$2:$I$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="H16" s="41">
-        <f>IF($L16="","",INDEX(Flux!$J$2:$J$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="I16" s="41">
-        <f>IF($L16="","",INDEX(Flux!$K$2:$K$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="J16" s="41">
-        <f>IF($L16="","",INDEX(Flux!$L$2:$L$35,$L16))</f>
-        <v/>
-      </c>
-      <c r="L16" s="42">
-        <f>IFERROR(MATCH(1,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M16" s="42">
-        <f>IF(L16="","",INDEX(Flux!$C$2:$C$35,L16))</f>
+      <c r="B16" s="40">
+        <f>IF($L16=0,"",INDEX(Flux!$D$2:$D$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="C16" s="41">
+        <f>IF($L16=0,"",INDEX(Flux!$E$2:$E$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="D16" s="42">
+        <f>IF($L16=0,"",INDEX(Flux!$F$2:$F$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="E16" s="43">
+        <f>IF($L16=0,"",INDEX(Flux!$G$2:$G$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="F16" s="43">
+        <f>IF($L16=0,"",INDEX(Flux!$H$2:$H$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="G16" s="43">
+        <f>IF($L16=0,"",INDEX(Flux!$I$2:$I$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="H16" s="43">
+        <f>IF($L16=0,"",INDEX(Flux!$J$2:$J$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="I16" s="43">
+        <f>IF($L16=0,"",INDEX(Flux!$K$2:$K$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="J16" s="43">
+        <f>IF($L16=0,"",INDEX(Flux!$L$2:$L$35,$L16))</f>
+        <v/>
+      </c>
+      <c r="L16" s="39">
+        <f>IFERROR(MATCH(1,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M16" s="39">
+        <f>IF(L16=0,"",INDEX(Flux!$C$2:$C$35,L16))</f>
+        <v/>
+      </c>
+      <c r="N16" s="39">
+        <f>IF(L16&gt;0,1,0)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="38">
-        <f>IF($L17="","",INDEX(Flux!$D$2:$D$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="C17" s="39">
-        <f>IF($L17="","",INDEX(Flux!$E$2:$E$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="D17" s="40">
-        <f>IF($L17="","",INDEX(Flux!$F$2:$F$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="E17" s="41">
-        <f>IF($L17="","",INDEX(Flux!$G$2:$G$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="F17" s="41">
-        <f>IF($L17="","",INDEX(Flux!$H$2:$H$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="G17" s="41">
-        <f>IF($L17="","",INDEX(Flux!$I$2:$I$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="H17" s="41">
-        <f>IF($L17="","",INDEX(Flux!$J$2:$J$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="I17" s="41">
-        <f>IF($L17="","",INDEX(Flux!$K$2:$K$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="J17" s="41">
-        <f>IF($L17="","",INDEX(Flux!$L$2:$L$35,$L17))</f>
-        <v/>
-      </c>
-      <c r="L17" s="42">
-        <f>IFERROR(MATCH(2,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M17" s="42">
-        <f>IF(L17="","",INDEX(Flux!$C$2:$C$35,L17))</f>
+      <c r="B17" s="40">
+        <f>IF($L17=0,"",INDEX(Flux!$D$2:$D$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="C17" s="41">
+        <f>IF($L17=0,"",INDEX(Flux!$E$2:$E$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="D17" s="42">
+        <f>IF($L17=0,"",INDEX(Flux!$F$2:$F$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="E17" s="43">
+        <f>IF($L17=0,"",INDEX(Flux!$G$2:$G$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="F17" s="43">
+        <f>IF($L17=0,"",INDEX(Flux!$H$2:$H$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="G17" s="43">
+        <f>IF($L17=0,"",INDEX(Flux!$I$2:$I$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="H17" s="43">
+        <f>IF($L17=0,"",INDEX(Flux!$J$2:$J$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="I17" s="43">
+        <f>IF($L17=0,"",INDEX(Flux!$K$2:$K$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="J17" s="43">
+        <f>IF($L17=0,"",INDEX(Flux!$L$2:$L$35,$L17))</f>
+        <v/>
+      </c>
+      <c r="L17" s="39">
+        <f>IFERROR(MATCH(2,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M17" s="39">
+        <f>IF(L17=0,"",INDEX(Flux!$C$2:$C$35,L17))</f>
+        <v/>
+      </c>
+      <c r="N17" s="39">
+        <f>IF(L17&gt;0,1,0)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="38">
-        <f>IF($L18="","",INDEX(Flux!$D$2:$D$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="C18" s="39">
-        <f>IF($L18="","",INDEX(Flux!$E$2:$E$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="D18" s="40">
-        <f>IF($L18="","",INDEX(Flux!$F$2:$F$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="E18" s="41">
-        <f>IF($L18="","",INDEX(Flux!$G$2:$G$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="F18" s="41">
-        <f>IF($L18="","",INDEX(Flux!$H$2:$H$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="G18" s="41">
-        <f>IF($L18="","",INDEX(Flux!$I$2:$I$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="H18" s="41">
-        <f>IF($L18="","",INDEX(Flux!$J$2:$J$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="I18" s="41">
-        <f>IF($L18="","",INDEX(Flux!$K$2:$K$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="J18" s="41">
-        <f>IF($L18="","",INDEX(Flux!$L$2:$L$35,$L18))</f>
-        <v/>
-      </c>
-      <c r="L18" s="42">
-        <f>IFERROR(MATCH(3,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M18" s="42">
-        <f>IF(L18="","",INDEX(Flux!$C$2:$C$35,L18))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="38">
-        <f>IF($L19="","",INDEX(Flux!$D$2:$D$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="C19" s="39">
-        <f>IF($L19="","",INDEX(Flux!$E$2:$E$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="D19" s="40">
-        <f>IF($L19="","",INDEX(Flux!$F$2:$F$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="E19" s="41">
-        <f>IF($L19="","",INDEX(Flux!$G$2:$G$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="F19" s="41">
-        <f>IF($L19="","",INDEX(Flux!$H$2:$H$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="G19" s="41">
-        <f>IF($L19="","",INDEX(Flux!$I$2:$I$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="H19" s="41">
-        <f>IF($L19="","",INDEX(Flux!$J$2:$J$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="I19" s="41">
-        <f>IF($L19="","",INDEX(Flux!$K$2:$K$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="J19" s="41">
-        <f>IF($L19="","",INDEX(Flux!$L$2:$L$35,$L19))</f>
-        <v/>
-      </c>
-      <c r="L19" s="42">
-        <f>IFERROR(MATCH(4,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M19" s="42">
-        <f>IF(L19="","",INDEX(Flux!$C$2:$C$35,L19))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="38">
-        <f>IF($L20="","",INDEX(Flux!$D$2:$D$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="C20" s="39">
-        <f>IF($L20="","",INDEX(Flux!$E$2:$E$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="D20" s="40">
-        <f>IF($L20="","",INDEX(Flux!$F$2:$F$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="E20" s="41">
-        <f>IF($L20="","",INDEX(Flux!$G$2:$G$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="F20" s="41">
-        <f>IF($L20="","",INDEX(Flux!$H$2:$H$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="G20" s="41">
-        <f>IF($L20="","",INDEX(Flux!$I$2:$I$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="H20" s="41">
-        <f>IF($L20="","",INDEX(Flux!$J$2:$J$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="I20" s="41">
-        <f>IF($L20="","",INDEX(Flux!$K$2:$K$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="J20" s="41">
-        <f>IF($L20="","",INDEX(Flux!$L$2:$L$35,$L20))</f>
-        <v/>
-      </c>
-      <c r="L20" s="42">
-        <f>IFERROR(MATCH(5,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="42">
-        <f>IF(L20="","",INDEX(Flux!$C$2:$C$35,L20))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="38">
-        <f>IF($L21="","",INDEX(Flux!$D$2:$D$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="C21" s="39">
-        <f>IF($L21="","",INDEX(Flux!$E$2:$E$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="D21" s="40">
-        <f>IF($L21="","",INDEX(Flux!$F$2:$F$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="E21" s="41">
-        <f>IF($L21="","",INDEX(Flux!$G$2:$G$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="F21" s="41">
-        <f>IF($L21="","",INDEX(Flux!$H$2:$H$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="G21" s="41">
-        <f>IF($L21="","",INDEX(Flux!$I$2:$I$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="H21" s="41">
-        <f>IF($L21="","",INDEX(Flux!$J$2:$J$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="I21" s="41">
-        <f>IF($L21="","",INDEX(Flux!$K$2:$K$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="J21" s="41">
-        <f>IF($L21="","",INDEX(Flux!$L$2:$L$35,$L21))</f>
-        <v/>
-      </c>
-      <c r="L21" s="42">
-        <f>IFERROR(MATCH(6,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M21" s="42">
-        <f>IF(L21="","",INDEX(Flux!$C$2:$C$35,L21))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="38">
-        <f>IF($L22="","",INDEX(Flux!$D$2:$D$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="C22" s="39">
-        <f>IF($L22="","",INDEX(Flux!$E$2:$E$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="D22" s="40">
-        <f>IF($L22="","",INDEX(Flux!$F$2:$F$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="E22" s="41">
-        <f>IF($L22="","",INDEX(Flux!$G$2:$G$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="F22" s="41">
-        <f>IF($L22="","",INDEX(Flux!$H$2:$H$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="G22" s="41">
-        <f>IF($L22="","",INDEX(Flux!$I$2:$I$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="H22" s="41">
-        <f>IF($L22="","",INDEX(Flux!$J$2:$J$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="I22" s="41">
-        <f>IF($L22="","",INDEX(Flux!$K$2:$K$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="J22" s="41">
-        <f>IF($L22="","",INDEX(Flux!$L$2:$L$35,$L22))</f>
-        <v/>
-      </c>
-      <c r="L22" s="42">
-        <f>IFERROR(MATCH(7,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M22" s="42">
-        <f>IF(L22="","",INDEX(Flux!$C$2:$C$35,L22))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="38">
-        <f>IF($L23="","",INDEX(Flux!$D$2:$D$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="C23" s="39">
-        <f>IF($L23="","",INDEX(Flux!$E$2:$E$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="D23" s="40">
-        <f>IF($L23="","",INDEX(Flux!$F$2:$F$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="E23" s="41">
-        <f>IF($L23="","",INDEX(Flux!$G$2:$G$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="F23" s="41">
-        <f>IF($L23="","",INDEX(Flux!$H$2:$H$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="G23" s="41">
-        <f>IF($L23="","",INDEX(Flux!$I$2:$I$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="H23" s="41">
-        <f>IF($L23="","",INDEX(Flux!$J$2:$J$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="I23" s="41">
-        <f>IF($L23="","",INDEX(Flux!$K$2:$K$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="J23" s="41">
-        <f>IF($L23="","",INDEX(Flux!$L$2:$L$35,$L23))</f>
-        <v/>
-      </c>
-      <c r="L23" s="42">
-        <f>IFERROR(MATCH(8,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M23" s="42">
-        <f>IF(L23="","",INDEX(Flux!$C$2:$C$35,L23))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="38">
-        <f>IF($L24="","",INDEX(Flux!$D$2:$D$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="C24" s="39">
-        <f>IF($L24="","",INDEX(Flux!$E$2:$E$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="D24" s="40">
-        <f>IF($L24="","",INDEX(Flux!$F$2:$F$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="E24" s="41">
-        <f>IF($L24="","",INDEX(Flux!$G$2:$G$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="F24" s="41">
-        <f>IF($L24="","",INDEX(Flux!$H$2:$H$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="G24" s="41">
-        <f>IF($L24="","",INDEX(Flux!$I$2:$I$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="H24" s="41">
-        <f>IF($L24="","",INDEX(Flux!$J$2:$J$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="I24" s="41">
-        <f>IF($L24="","",INDEX(Flux!$K$2:$K$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="J24" s="41">
-        <f>IF($L24="","",INDEX(Flux!$L$2:$L$35,$L24))</f>
-        <v/>
-      </c>
-      <c r="L24" s="42">
-        <f>IFERROR(MATCH(9,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M24" s="42">
-        <f>IF(L24="","",INDEX(Flux!$C$2:$C$35,L24))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="38">
-        <f>IF($L25="","",INDEX(Flux!$D$2:$D$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="C25" s="39">
-        <f>IF($L25="","",INDEX(Flux!$E$2:$E$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="D25" s="40">
-        <f>IF($L25="","",INDEX(Flux!$F$2:$F$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="E25" s="41">
-        <f>IF($L25="","",INDEX(Flux!$G$2:$G$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="F25" s="41">
-        <f>IF($L25="","",INDEX(Flux!$H$2:$H$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="G25" s="41">
-        <f>IF($L25="","",INDEX(Flux!$I$2:$I$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="H25" s="41">
-        <f>IF($L25="","",INDEX(Flux!$J$2:$J$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="I25" s="41">
-        <f>IF($L25="","",INDEX(Flux!$K$2:$K$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="J25" s="41">
-        <f>IF($L25="","",INDEX(Flux!$L$2:$L$35,$L25))</f>
-        <v/>
-      </c>
-      <c r="L25" s="42">
-        <f>IFERROR(MATCH(10,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M25" s="42">
-        <f>IF(L25="","",INDEX(Flux!$C$2:$C$35,L25))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="38">
-        <f>IF($L26="","",INDEX(Flux!$D$2:$D$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="C26" s="39">
-        <f>IF($L26="","",INDEX(Flux!$E$2:$E$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="D26" s="40">
-        <f>IF($L26="","",INDEX(Flux!$F$2:$F$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="E26" s="41">
-        <f>IF($L26="","",INDEX(Flux!$G$2:$G$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="F26" s="41">
-        <f>IF($L26="","",INDEX(Flux!$H$2:$H$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="G26" s="41">
-        <f>IF($L26="","",INDEX(Flux!$I$2:$I$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="H26" s="41">
-        <f>IF($L26="","",INDEX(Flux!$J$2:$J$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="I26" s="41">
-        <f>IF($L26="","",INDEX(Flux!$K$2:$K$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="J26" s="41">
-        <f>IF($L26="","",INDEX(Flux!$L$2:$L$35,$L26))</f>
-        <v/>
-      </c>
-      <c r="L26" s="42">
-        <f>IFERROR(MATCH(11,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M26" s="42">
-        <f>IF(L26="","",INDEX(Flux!$C$2:$C$35,L26))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="38">
-        <f>IF($L27="","",INDEX(Flux!$D$2:$D$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="C27" s="39">
-        <f>IF($L27="","",INDEX(Flux!$E$2:$E$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="D27" s="40">
-        <f>IF($L27="","",INDEX(Flux!$F$2:$F$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="E27" s="41">
-        <f>IF($L27="","",INDEX(Flux!$G$2:$G$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="F27" s="41">
-        <f>IF($L27="","",INDEX(Flux!$H$2:$H$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="G27" s="41">
-        <f>IF($L27="","",INDEX(Flux!$I$2:$I$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="H27" s="41">
-        <f>IF($L27="","",INDEX(Flux!$J$2:$J$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="I27" s="41">
-        <f>IF($L27="","",INDEX(Flux!$K$2:$K$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="J27" s="41">
-        <f>IF($L27="","",INDEX(Flux!$L$2:$L$35,$L27))</f>
-        <v/>
-      </c>
-      <c r="L27" s="42">
-        <f>IFERROR(MATCH(12,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="42">
-        <f>IF(L27="","",INDEX(Flux!$C$2:$C$35,L27))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="38">
-        <f>IF($L28="","",INDEX(Flux!$D$2:$D$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="C28" s="39">
-        <f>IF($L28="","",INDEX(Flux!$E$2:$E$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="D28" s="40">
-        <f>IF($L28="","",INDEX(Flux!$F$2:$F$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="E28" s="41">
-        <f>IF($L28="","",INDEX(Flux!$G$2:$G$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="F28" s="41">
-        <f>IF($L28="","",INDEX(Flux!$H$2:$H$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="G28" s="41">
-        <f>IF($L28="","",INDEX(Flux!$I$2:$I$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="H28" s="41">
-        <f>IF($L28="","",INDEX(Flux!$J$2:$J$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="I28" s="41">
-        <f>IF($L28="","",INDEX(Flux!$K$2:$K$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="J28" s="41">
-        <f>IF($L28="","",INDEX(Flux!$L$2:$L$35,$L28))</f>
-        <v/>
-      </c>
-      <c r="L28" s="42">
-        <f>IFERROR(MATCH(13,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="42">
-        <f>IF(L28="","",INDEX(Flux!$C$2:$C$35,L28))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="38">
-        <f>IF($L29="","",INDEX(Flux!$D$2:$D$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="C29" s="39">
-        <f>IF($L29="","",INDEX(Flux!$E$2:$E$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="D29" s="40">
-        <f>IF($L29="","",INDEX(Flux!$F$2:$F$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="E29" s="41">
-        <f>IF($L29="","",INDEX(Flux!$G$2:$G$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="F29" s="41">
-        <f>IF($L29="","",INDEX(Flux!$H$2:$H$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="G29" s="41">
-        <f>IF($L29="","",INDEX(Flux!$I$2:$I$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="H29" s="41">
-        <f>IF($L29="","",INDEX(Flux!$J$2:$J$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="I29" s="41">
-        <f>IF($L29="","",INDEX(Flux!$K$2:$K$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="J29" s="41">
-        <f>IF($L29="","",INDEX(Flux!$L$2:$L$35,$L29))</f>
-        <v/>
-      </c>
-      <c r="L29" s="42">
-        <f>IFERROR(MATCH(14,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="42">
-        <f>IF(L29="","",INDEX(Flux!$C$2:$C$35,L29))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="38">
-        <f>IF($L30="","",INDEX(Flux!$D$2:$D$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="C30" s="39">
-        <f>IF($L30="","",INDEX(Flux!$E$2:$E$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="D30" s="40">
-        <f>IF($L30="","",INDEX(Flux!$F$2:$F$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="E30" s="41">
-        <f>IF($L30="","",INDEX(Flux!$G$2:$G$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="F30" s="41">
-        <f>IF($L30="","",INDEX(Flux!$H$2:$H$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="G30" s="41">
-        <f>IF($L30="","",INDEX(Flux!$I$2:$I$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="H30" s="41">
-        <f>IF($L30="","",INDEX(Flux!$J$2:$J$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="I30" s="41">
-        <f>IF($L30="","",INDEX(Flux!$K$2:$K$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="J30" s="41">
-        <f>IF($L30="","",INDEX(Flux!$L$2:$L$35,$L30))</f>
-        <v/>
-      </c>
-      <c r="L30" s="42">
-        <f>IFERROR(MATCH(15,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="42">
-        <f>IF(L30="","",INDEX(Flux!$C$2:$C$35,L30))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="38">
-        <f>IF($L31="","",INDEX(Flux!$D$2:$D$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="C31" s="39">
-        <f>IF($L31="","",INDEX(Flux!$E$2:$E$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="D31" s="40">
-        <f>IF($L31="","",INDEX(Flux!$F$2:$F$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="E31" s="41">
-        <f>IF($L31="","",INDEX(Flux!$G$2:$G$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="F31" s="41">
-        <f>IF($L31="","",INDEX(Flux!$H$2:$H$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="G31" s="41">
-        <f>IF($L31="","",INDEX(Flux!$I$2:$I$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="H31" s="41">
-        <f>IF($L31="","",INDEX(Flux!$J$2:$J$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="I31" s="41">
-        <f>IF($L31="","",INDEX(Flux!$K$2:$K$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="J31" s="41">
-        <f>IF($L31="","",INDEX(Flux!$L$2:$L$35,$L31))</f>
-        <v/>
-      </c>
-      <c r="L31" s="42">
-        <f>IFERROR(MATCH(16,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M31" s="42">
-        <f>IF(L31="","",INDEX(Flux!$C$2:$C$35,L31))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="38">
-        <f>IF($L32="","",INDEX(Flux!$D$2:$D$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="C32" s="39">
-        <f>IF($L32="","",INDEX(Flux!$E$2:$E$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="D32" s="40">
-        <f>IF($L32="","",INDEX(Flux!$F$2:$F$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="E32" s="41">
-        <f>IF($L32="","",INDEX(Flux!$G$2:$G$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="F32" s="41">
-        <f>IF($L32="","",INDEX(Flux!$H$2:$H$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="G32" s="41">
-        <f>IF($L32="","",INDEX(Flux!$I$2:$I$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="H32" s="41">
-        <f>IF($L32="","",INDEX(Flux!$J$2:$J$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="I32" s="41">
-        <f>IF($L32="","",INDEX(Flux!$K$2:$K$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="J32" s="41">
-        <f>IF($L32="","",INDEX(Flux!$L$2:$L$35,$L32))</f>
-        <v/>
-      </c>
-      <c r="L32" s="42">
-        <f>IFERROR(MATCH(17,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="42">
-        <f>IF(L32="","",INDEX(Flux!$C$2:$C$35,L32))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="38">
-        <f>IF($L33="","",INDEX(Flux!$D$2:$D$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="C33" s="39">
-        <f>IF($L33="","",INDEX(Flux!$E$2:$E$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="D33" s="40">
-        <f>IF($L33="","",INDEX(Flux!$F$2:$F$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="E33" s="41">
-        <f>IF($L33="","",INDEX(Flux!$G$2:$G$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="F33" s="41">
-        <f>IF($L33="","",INDEX(Flux!$H$2:$H$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="G33" s="41">
-        <f>IF($L33="","",INDEX(Flux!$I$2:$I$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="H33" s="41">
-        <f>IF($L33="","",INDEX(Flux!$J$2:$J$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="I33" s="41">
-        <f>IF($L33="","",INDEX(Flux!$K$2:$K$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="J33" s="41">
-        <f>IF($L33="","",INDEX(Flux!$L$2:$L$35,$L33))</f>
-        <v/>
-      </c>
-      <c r="L33" s="42">
-        <f>IFERROR(MATCH(18,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="42">
-        <f>IF(L33="","",INDEX(Flux!$C$2:$C$35,L33))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="38">
-        <f>IF($L34="","",INDEX(Flux!$D$2:$D$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="C34" s="39">
-        <f>IF($L34="","",INDEX(Flux!$E$2:$E$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="D34" s="40">
-        <f>IF($L34="","",INDEX(Flux!$F$2:$F$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="E34" s="41">
-        <f>IF($L34="","",INDEX(Flux!$G$2:$G$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="F34" s="41">
-        <f>IF($L34="","",INDEX(Flux!$H$2:$H$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="G34" s="41">
-        <f>IF($L34="","",INDEX(Flux!$I$2:$I$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="H34" s="41">
-        <f>IF($L34="","",INDEX(Flux!$J$2:$J$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="I34" s="41">
-        <f>IF($L34="","",INDEX(Flux!$K$2:$K$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="J34" s="41">
-        <f>IF($L34="","",INDEX(Flux!$L$2:$L$35,$L34))</f>
-        <v/>
-      </c>
-      <c r="L34" s="42">
-        <f>IFERROR(MATCH(19,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M34" s="42">
-        <f>IF(L34="","",INDEX(Flux!$C$2:$C$35,L34))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="38">
-        <f>IF($L35="","",INDEX(Flux!$D$2:$D$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="C35" s="39">
-        <f>IF($L35="","",INDEX(Flux!$E$2:$E$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="D35" s="40">
-        <f>IF($L35="","",INDEX(Flux!$F$2:$F$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="E35" s="41">
-        <f>IF($L35="","",INDEX(Flux!$G$2:$G$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="F35" s="41">
-        <f>IF($L35="","",INDEX(Flux!$H$2:$H$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="G35" s="41">
-        <f>IF($L35="","",INDEX(Flux!$I$2:$I$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="H35" s="41">
-        <f>IF($L35="","",INDEX(Flux!$J$2:$J$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="I35" s="41">
-        <f>IF($L35="","",INDEX(Flux!$K$2:$K$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="J35" s="41">
-        <f>IF($L35="","",INDEX(Flux!$L$2:$L$35,$L35))</f>
-        <v/>
-      </c>
-      <c r="L35" s="42">
-        <f>IFERROR(MATCH(20,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M35" s="42">
-        <f>IF(L35="","",INDEX(Flux!$C$2:$C$35,L35))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="38">
-        <f>IF($L36="","",INDEX(Flux!$D$2:$D$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="C36" s="39">
-        <f>IF($L36="","",INDEX(Flux!$E$2:$E$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="D36" s="40">
-        <f>IF($L36="","",INDEX(Flux!$F$2:$F$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="E36" s="41">
-        <f>IF($L36="","",INDEX(Flux!$G$2:$G$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="F36" s="41">
-        <f>IF($L36="","",INDEX(Flux!$H$2:$H$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="G36" s="41">
-        <f>IF($L36="","",INDEX(Flux!$I$2:$I$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="H36" s="41">
-        <f>IF($L36="","",INDEX(Flux!$J$2:$J$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="I36" s="41">
-        <f>IF($L36="","",INDEX(Flux!$K$2:$K$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="J36" s="41">
-        <f>IF($L36="","",INDEX(Flux!$L$2:$L$35,$L36))</f>
-        <v/>
-      </c>
-      <c r="L36" s="42">
-        <f>IFERROR(MATCH(21,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M36" s="42">
-        <f>IF(L36="","",INDEX(Flux!$C$2:$C$35,L36))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="38">
-        <f>IF($L37="","",INDEX(Flux!$D$2:$D$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="C37" s="39">
-        <f>IF($L37="","",INDEX(Flux!$E$2:$E$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="D37" s="40">
-        <f>IF($L37="","",INDEX(Flux!$F$2:$F$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="E37" s="41">
-        <f>IF($L37="","",INDEX(Flux!$G$2:$G$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="F37" s="41">
-        <f>IF($L37="","",INDEX(Flux!$H$2:$H$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="G37" s="41">
-        <f>IF($L37="","",INDEX(Flux!$I$2:$I$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="H37" s="41">
-        <f>IF($L37="","",INDEX(Flux!$J$2:$J$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="I37" s="41">
-        <f>IF($L37="","",INDEX(Flux!$K$2:$K$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="J37" s="41">
-        <f>IF($L37="","",INDEX(Flux!$L$2:$L$35,$L37))</f>
-        <v/>
-      </c>
-      <c r="L37" s="42">
-        <f>IFERROR(MATCH(22,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M37" s="42">
-        <f>IF(L37="","",INDEX(Flux!$C$2:$C$35,L37))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="B38" s="38">
-        <f>IF($L38="","",INDEX(Flux!$D$2:$D$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="C38" s="39">
-        <f>IF($L38="","",INDEX(Flux!$E$2:$E$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="D38" s="40">
-        <f>IF($L38="","",INDEX(Flux!$F$2:$F$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="E38" s="41">
-        <f>IF($L38="","",INDEX(Flux!$G$2:$G$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="F38" s="41">
-        <f>IF($L38="","",INDEX(Flux!$H$2:$H$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="G38" s="41">
-        <f>IF($L38="","",INDEX(Flux!$I$2:$I$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="H38" s="41">
-        <f>IF($L38="","",INDEX(Flux!$J$2:$J$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="I38" s="41">
-        <f>IF($L38="","",INDEX(Flux!$K$2:$K$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="J38" s="41">
-        <f>IF($L38="","",INDEX(Flux!$L$2:$L$35,$L38))</f>
-        <v/>
-      </c>
-      <c r="L38" s="42">
-        <f>IFERROR(MATCH(23,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M38" s="42">
-        <f>IF(L38="","",INDEX(Flux!$C$2:$C$35,L38))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="B39" s="38">
-        <f>IF($L39="","",INDEX(Flux!$D$2:$D$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="C39" s="39">
-        <f>IF($L39="","",INDEX(Flux!$E$2:$E$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="D39" s="40">
-        <f>IF($L39="","",INDEX(Flux!$F$2:$F$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="E39" s="41">
-        <f>IF($L39="","",INDEX(Flux!$G$2:$G$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="F39" s="41">
-        <f>IF($L39="","",INDEX(Flux!$H$2:$H$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="G39" s="41">
-        <f>IF($L39="","",INDEX(Flux!$I$2:$I$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="H39" s="41">
-        <f>IF($L39="","",INDEX(Flux!$J$2:$J$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="I39" s="41">
-        <f>IF($L39="","",INDEX(Flux!$K$2:$K$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="J39" s="41">
-        <f>IF($L39="","",INDEX(Flux!$L$2:$L$35,$L39))</f>
-        <v/>
-      </c>
-      <c r="L39" s="42">
-        <f>IFERROR(MATCH(24,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M39" s="42">
-        <f>IF(L39="","",INDEX(Flux!$C$2:$C$35,L39))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="B40" s="38">
-        <f>IF($L40="","",INDEX(Flux!$D$2:$D$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="C40" s="39">
-        <f>IF($L40="","",INDEX(Flux!$E$2:$E$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="D40" s="40">
-        <f>IF($L40="","",INDEX(Flux!$F$2:$F$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="E40" s="41">
-        <f>IF($L40="","",INDEX(Flux!$G$2:$G$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="F40" s="41">
-        <f>IF($L40="","",INDEX(Flux!$H$2:$H$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="G40" s="41">
-        <f>IF($L40="","",INDEX(Flux!$I$2:$I$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="H40" s="41">
-        <f>IF($L40="","",INDEX(Flux!$J$2:$J$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="I40" s="41">
-        <f>IF($L40="","",INDEX(Flux!$K$2:$K$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="J40" s="41">
-        <f>IF($L40="","",INDEX(Flux!$L$2:$L$35,$L40))</f>
-        <v/>
-      </c>
-      <c r="L40" s="42">
-        <f>IFERROR(MATCH(25,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M40" s="42">
-        <f>IF(L40="","",INDEX(Flux!$C$2:$C$35,L40))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="38">
-        <f>IF($L41="","",INDEX(Flux!$D$2:$D$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="C41" s="39">
-        <f>IF($L41="","",INDEX(Flux!$E$2:$E$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="D41" s="40">
-        <f>IF($L41="","",INDEX(Flux!$F$2:$F$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="E41" s="41">
-        <f>IF($L41="","",INDEX(Flux!$G$2:$G$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="F41" s="41">
-        <f>IF($L41="","",INDEX(Flux!$H$2:$H$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="G41" s="41">
-        <f>IF($L41="","",INDEX(Flux!$I$2:$I$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="H41" s="41">
-        <f>IF($L41="","",INDEX(Flux!$J$2:$J$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="I41" s="41">
-        <f>IF($L41="","",INDEX(Flux!$K$2:$K$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="J41" s="41">
-        <f>IF($L41="","",INDEX(Flux!$L$2:$L$35,$L41))</f>
-        <v/>
-      </c>
-      <c r="L41" s="42">
-        <f>IFERROR(MATCH(26,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M41" s="42">
-        <f>IF(L41="","",INDEX(Flux!$C$2:$C$35,L41))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B42" s="38">
-        <f>IF($L42="","",INDEX(Flux!$D$2:$D$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="C42" s="39">
-        <f>IF($L42="","",INDEX(Flux!$E$2:$E$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="D42" s="40">
-        <f>IF($L42="","",INDEX(Flux!$F$2:$F$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="E42" s="41">
-        <f>IF($L42="","",INDEX(Flux!$G$2:$G$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="F42" s="41">
-        <f>IF($L42="","",INDEX(Flux!$H$2:$H$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="G42" s="41">
-        <f>IF($L42="","",INDEX(Flux!$I$2:$I$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="H42" s="41">
-        <f>IF($L42="","",INDEX(Flux!$J$2:$J$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="I42" s="41">
-        <f>IF($L42="","",INDEX(Flux!$K$2:$K$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="J42" s="41">
-        <f>IF($L42="","",INDEX(Flux!$L$2:$L$35,$L42))</f>
-        <v/>
-      </c>
-      <c r="L42" s="42">
-        <f>IFERROR(MATCH(27,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M42" s="42">
-        <f>IF(L42="","",INDEX(Flux!$C$2:$C$35,L42))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B43" s="38">
-        <f>IF($L43="","",INDEX(Flux!$D$2:$D$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="C43" s="39">
-        <f>IF($L43="","",INDEX(Flux!$E$2:$E$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="D43" s="40">
-        <f>IF($L43="","",INDEX(Flux!$F$2:$F$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="E43" s="41">
-        <f>IF($L43="","",INDEX(Flux!$G$2:$G$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="F43" s="41">
-        <f>IF($L43="","",INDEX(Flux!$H$2:$H$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="G43" s="41">
-        <f>IF($L43="","",INDEX(Flux!$I$2:$I$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="H43" s="41">
-        <f>IF($L43="","",INDEX(Flux!$J$2:$J$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="I43" s="41">
-        <f>IF($L43="","",INDEX(Flux!$K$2:$K$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="J43" s="41">
-        <f>IF($L43="","",INDEX(Flux!$L$2:$L$35,$L43))</f>
-        <v/>
-      </c>
-      <c r="L43" s="42">
-        <f>IFERROR(MATCH(28,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M43" s="42">
-        <f>IF(L43="","",INDEX(Flux!$C$2:$C$35,L43))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B44" s="38">
-        <f>IF($L44="","",INDEX(Flux!$D$2:$D$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="C44" s="39">
-        <f>IF($L44="","",INDEX(Flux!$E$2:$E$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="D44" s="40">
-        <f>IF($L44="","",INDEX(Flux!$F$2:$F$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="E44" s="41">
-        <f>IF($L44="","",INDEX(Flux!$G$2:$G$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="F44" s="41">
-        <f>IF($L44="","",INDEX(Flux!$H$2:$H$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="G44" s="41">
-        <f>IF($L44="","",INDEX(Flux!$I$2:$I$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="H44" s="41">
-        <f>IF($L44="","",INDEX(Flux!$J$2:$J$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="I44" s="41">
-        <f>IF($L44="","",INDEX(Flux!$K$2:$K$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="J44" s="41">
-        <f>IF($L44="","",INDEX(Flux!$L$2:$L$35,$L44))</f>
-        <v/>
-      </c>
-      <c r="L44" s="42">
-        <f>IFERROR(MATCH(29,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M44" s="42">
-        <f>IF(L44="","",INDEX(Flux!$C$2:$C$35,L44))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B45" s="38">
-        <f>IF($L45="","",INDEX(Flux!$D$2:$D$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="C45" s="39">
-        <f>IF($L45="","",INDEX(Flux!$E$2:$E$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="D45" s="40">
-        <f>IF($L45="","",INDEX(Flux!$F$2:$F$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="E45" s="41">
-        <f>IF($L45="","",INDEX(Flux!$G$2:$G$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="F45" s="41">
-        <f>IF($L45="","",INDEX(Flux!$H$2:$H$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="G45" s="41">
-        <f>IF($L45="","",INDEX(Flux!$I$2:$I$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="H45" s="41">
-        <f>IF($L45="","",INDEX(Flux!$J$2:$J$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="I45" s="41">
-        <f>IF($L45="","",INDEX(Flux!$K$2:$K$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="J45" s="41">
-        <f>IF($L45="","",INDEX(Flux!$L$2:$L$35,$L45))</f>
-        <v/>
-      </c>
-      <c r="L45" s="42">
-        <f>IFERROR(MATCH(30,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M45" s="42">
-        <f>IF(L45="","",INDEX(Flux!$C$2:$C$35,L45))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B46" s="38">
-        <f>IF($L46="","",INDEX(Flux!$D$2:$D$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="C46" s="39">
-        <f>IF($L46="","",INDEX(Flux!$E$2:$E$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="D46" s="40">
-        <f>IF($L46="","",INDEX(Flux!$F$2:$F$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="E46" s="41">
-        <f>IF($L46="","",INDEX(Flux!$G$2:$G$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="F46" s="41">
-        <f>IF($L46="","",INDEX(Flux!$H$2:$H$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="G46" s="41">
-        <f>IF($L46="","",INDEX(Flux!$I$2:$I$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="H46" s="41">
-        <f>IF($L46="","",INDEX(Flux!$J$2:$J$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="I46" s="41">
-        <f>IF($L46="","",INDEX(Flux!$K$2:$K$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="J46" s="41">
-        <f>IF($L46="","",INDEX(Flux!$L$2:$L$35,$L46))</f>
-        <v/>
-      </c>
-      <c r="L46" s="42">
-        <f>IFERROR(MATCH(31,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M46" s="42">
-        <f>IF(L46="","",INDEX(Flux!$C$2:$C$35,L46))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B47" s="38">
-        <f>IF($L47="","",INDEX(Flux!$D$2:$D$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="C47" s="39">
-        <f>IF($L47="","",INDEX(Flux!$E$2:$E$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="D47" s="40">
-        <f>IF($L47="","",INDEX(Flux!$F$2:$F$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="E47" s="41">
-        <f>IF($L47="","",INDEX(Flux!$G$2:$G$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="F47" s="41">
-        <f>IF($L47="","",INDEX(Flux!$H$2:$H$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="G47" s="41">
-        <f>IF($L47="","",INDEX(Flux!$I$2:$I$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="H47" s="41">
-        <f>IF($L47="","",INDEX(Flux!$J$2:$J$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="I47" s="41">
-        <f>IF($L47="","",INDEX(Flux!$K$2:$K$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="J47" s="41">
-        <f>IF($L47="","",INDEX(Flux!$L$2:$L$35,$L47))</f>
-        <v/>
-      </c>
-      <c r="L47" s="42">
-        <f>IFERROR(MATCH(32,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M47" s="42">
-        <f>IF(L47="","",INDEX(Flux!$C$2:$C$35,L47))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B48" s="38">
-        <f>IF($L48="","",INDEX(Flux!$D$2:$D$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="C48" s="39">
-        <f>IF($L48="","",INDEX(Flux!$E$2:$E$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="D48" s="40">
-        <f>IF($L48="","",INDEX(Flux!$F$2:$F$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="E48" s="41">
-        <f>IF($L48="","",INDEX(Flux!$G$2:$G$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="F48" s="41">
-        <f>IF($L48="","",INDEX(Flux!$H$2:$H$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="G48" s="41">
-        <f>IF($L48="","",INDEX(Flux!$I$2:$I$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="H48" s="41">
-        <f>IF($L48="","",INDEX(Flux!$J$2:$J$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="I48" s="41">
-        <f>IF($L48="","",INDEX(Flux!$K$2:$K$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="J48" s="41">
-        <f>IF($L48="","",INDEX(Flux!$L$2:$L$35,$L48))</f>
-        <v/>
-      </c>
-      <c r="L48" s="42">
-        <f>IFERROR(MATCH(33,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M48" s="42">
-        <f>IF(L48="","",INDEX(Flux!$C$2:$C$35,L48))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B49" s="38">
-        <f>IF($L49="","",INDEX(Flux!$D$2:$D$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="C49" s="39">
-        <f>IF($L49="","",INDEX(Flux!$E$2:$E$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="D49" s="40">
-        <f>IF($L49="","",INDEX(Flux!$F$2:$F$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="E49" s="41">
-        <f>IF($L49="","",INDEX(Flux!$G$2:$G$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="F49" s="41">
-        <f>IF($L49="","",INDEX(Flux!$H$2:$H$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="G49" s="41">
-        <f>IF($L49="","",INDEX(Flux!$I$2:$I$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="H49" s="41">
-        <f>IF($L49="","",INDEX(Flux!$J$2:$J$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="I49" s="41">
-        <f>IF($L49="","",INDEX(Flux!$K$2:$K$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="J49" s="41">
-        <f>IF($L49="","",INDEX(Flux!$L$2:$L$35,$L49))</f>
-        <v/>
-      </c>
-      <c r="L49" s="42">
-        <f>IFERROR(MATCH(34,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M49" s="42">
-        <f>IF(L49="","",INDEX(Flux!$C$2:$C$35,L49))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B50" s="38">
-        <f>IF($L50="","",INDEX(Flux!$D$2:$D$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="C50" s="39">
-        <f>IF($L50="","",INDEX(Flux!$E$2:$E$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="D50" s="40">
-        <f>IF($L50="","",INDEX(Flux!$F$2:$F$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="E50" s="41">
-        <f>IF($L50="","",INDEX(Flux!$G$2:$G$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="F50" s="41">
-        <f>IF($L50="","",INDEX(Flux!$H$2:$H$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="G50" s="41">
-        <f>IF($L50="","",INDEX(Flux!$I$2:$I$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="H50" s="41">
-        <f>IF($L50="","",INDEX(Flux!$J$2:$J$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="I50" s="41">
-        <f>IF($L50="","",INDEX(Flux!$K$2:$K$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="J50" s="41">
-        <f>IF($L50="","",INDEX(Flux!$L$2:$L$35,$L50))</f>
-        <v/>
-      </c>
-      <c r="L50" s="42">
-        <f>IFERROR(MATCH(35,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M50" s="42">
-        <f>IF(L50="","",INDEX(Flux!$C$2:$C$35,L50))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B51" s="38">
-        <f>IF($L51="","",INDEX(Flux!$D$2:$D$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="C51" s="39">
-        <f>IF($L51="","",INDEX(Flux!$E$2:$E$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="D51" s="40">
-        <f>IF($L51="","",INDEX(Flux!$F$2:$F$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="E51" s="41">
-        <f>IF($L51="","",INDEX(Flux!$G$2:$G$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="F51" s="41">
-        <f>IF($L51="","",INDEX(Flux!$H$2:$H$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="G51" s="41">
-        <f>IF($L51="","",INDEX(Flux!$I$2:$I$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="H51" s="41">
-        <f>IF($L51="","",INDEX(Flux!$J$2:$J$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="I51" s="41">
-        <f>IF($L51="","",INDEX(Flux!$K$2:$K$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="J51" s="41">
-        <f>IF($L51="","",INDEX(Flux!$L$2:$L$35,$L51))</f>
-        <v/>
-      </c>
-      <c r="L51" s="42">
-        <f>IFERROR(MATCH(36,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M51" s="42">
-        <f>IF(L51="","",INDEX(Flux!$C$2:$C$35,L51))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B52" s="38">
-        <f>IF($L52="","",INDEX(Flux!$D$2:$D$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="C52" s="39">
-        <f>IF($L52="","",INDEX(Flux!$E$2:$E$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="D52" s="40">
-        <f>IF($L52="","",INDEX(Flux!$F$2:$F$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="E52" s="41">
-        <f>IF($L52="","",INDEX(Flux!$G$2:$G$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="F52" s="41">
-        <f>IF($L52="","",INDEX(Flux!$H$2:$H$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="G52" s="41">
-        <f>IF($L52="","",INDEX(Flux!$I$2:$I$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="H52" s="41">
-        <f>IF($L52="","",INDEX(Flux!$J$2:$J$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="I52" s="41">
-        <f>IF($L52="","",INDEX(Flux!$K$2:$K$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="J52" s="41">
-        <f>IF($L52="","",INDEX(Flux!$L$2:$L$35,$L52))</f>
-        <v/>
-      </c>
-      <c r="L52" s="42">
-        <f>IFERROR(MATCH(37,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M52" s="42">
-        <f>IF(L52="","",INDEX(Flux!$C$2:$C$35,L52))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B53" s="38">
-        <f>IF($L53="","",INDEX(Flux!$D$2:$D$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="C53" s="39">
-        <f>IF($L53="","",INDEX(Flux!$E$2:$E$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="D53" s="40">
-        <f>IF($L53="","",INDEX(Flux!$F$2:$F$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="E53" s="41">
-        <f>IF($L53="","",INDEX(Flux!$G$2:$G$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="F53" s="41">
-        <f>IF($L53="","",INDEX(Flux!$H$2:$H$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="G53" s="41">
-        <f>IF($L53="","",INDEX(Flux!$I$2:$I$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="H53" s="41">
-        <f>IF($L53="","",INDEX(Flux!$J$2:$J$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="I53" s="41">
-        <f>IF($L53="","",INDEX(Flux!$K$2:$K$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="J53" s="41">
-        <f>IF($L53="","",INDEX(Flux!$L$2:$L$35,$L53))</f>
-        <v/>
-      </c>
-      <c r="L53" s="42">
-        <f>IFERROR(MATCH(38,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M53" s="42">
-        <f>IF(L53="","",INDEX(Flux!$C$2:$C$35,L53))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B54" s="38">
-        <f>IF($L54="","",INDEX(Flux!$D$2:$D$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="C54" s="39">
-        <f>IF($L54="","",INDEX(Flux!$E$2:$E$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="D54" s="40">
-        <f>IF($L54="","",INDEX(Flux!$F$2:$F$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="E54" s="41">
-        <f>IF($L54="","",INDEX(Flux!$G$2:$G$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="F54" s="41">
-        <f>IF($L54="","",INDEX(Flux!$H$2:$H$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="G54" s="41">
-        <f>IF($L54="","",INDEX(Flux!$I$2:$I$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="H54" s="41">
-        <f>IF($L54="","",INDEX(Flux!$J$2:$J$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="I54" s="41">
-        <f>IF($L54="","",INDEX(Flux!$K$2:$K$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="J54" s="41">
-        <f>IF($L54="","",INDEX(Flux!$L$2:$L$35,$L54))</f>
-        <v/>
-      </c>
-      <c r="L54" s="42">
-        <f>IFERROR(MATCH(39,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M54" s="42">
-        <f>IF(L54="","",INDEX(Flux!$C$2:$C$35,L54))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="B55" s="38">
-        <f>IF($L55="","",INDEX(Flux!$D$2:$D$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="C55" s="39">
-        <f>IF($L55="","",INDEX(Flux!$E$2:$E$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="D55" s="40">
-        <f>IF($L55="","",INDEX(Flux!$F$2:$F$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="E55" s="41">
-        <f>IF($L55="","",INDEX(Flux!$G$2:$G$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="F55" s="41">
-        <f>IF($L55="","",INDEX(Flux!$H$2:$H$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="G55" s="41">
-        <f>IF($L55="","",INDEX(Flux!$I$2:$I$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="H55" s="41">
-        <f>IF($L55="","",INDEX(Flux!$J$2:$J$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="I55" s="41">
-        <f>IF($L55="","",INDEX(Flux!$K$2:$K$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="J55" s="41">
-        <f>IF($L55="","",INDEX(Flux!$L$2:$L$35,$L55))</f>
-        <v/>
-      </c>
-      <c r="L55" s="42">
-        <f>IFERROR(MATCH(40,Flux!$B$2:$B$35,0),"")</f>
-        <v/>
-      </c>
-      <c r="M55" s="42">
-        <f>IF(L55="","",INDEX(Flux!$C$2:$C$35,L55))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="B56" s="43">
-        <f>IF(MAX(Flux!$B$2:$B$35)&gt;26,"⚠  Le devis contient plus de 26 lignes : cliquer sur le [+] dans la marge gauche pour afficher les lignes masquées.","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" ht="8" customHeight="1"/>
+      <c r="B18" s="40">
+        <f>IF($L18=0,"",INDEX(Flux!$D$2:$D$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="C18" s="41">
+        <f>IF($L18=0,"",INDEX(Flux!$E$2:$E$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="D18" s="42">
+        <f>IF($L18=0,"",INDEX(Flux!$F$2:$F$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="E18" s="43">
+        <f>IF($L18=0,"",INDEX(Flux!$G$2:$G$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="F18" s="43">
+        <f>IF($L18=0,"",INDEX(Flux!$H$2:$H$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="G18" s="43">
+        <f>IF($L18=0,"",INDEX(Flux!$I$2:$I$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="H18" s="43">
+        <f>IF($L18=0,"",INDEX(Flux!$J$2:$J$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="I18" s="43">
+        <f>IF($L18=0,"",INDEX(Flux!$K$2:$K$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="J18" s="43">
+        <f>IF($L18=0,"",INDEX(Flux!$L$2:$L$35,$L18))</f>
+        <v/>
+      </c>
+      <c r="L18" s="39">
+        <f>IFERROR(MATCH(3,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M18" s="39">
+        <f>IF(L18=0,"",INDEX(Flux!$C$2:$C$35,L18))</f>
+        <v/>
+      </c>
+      <c r="N18" s="39">
+        <f>IF(L18&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" hidden="1" ht="22" customHeight="1">
+      <c r="B19" s="40">
+        <f>IF($L19=0,"",INDEX(Flux!$D$2:$D$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="C19" s="41">
+        <f>IF($L19=0,"",INDEX(Flux!$E$2:$E$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="D19" s="42">
+        <f>IF($L19=0,"",INDEX(Flux!$F$2:$F$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="E19" s="43">
+        <f>IF($L19=0,"",INDEX(Flux!$G$2:$G$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="F19" s="43">
+        <f>IF($L19=0,"",INDEX(Flux!$H$2:$H$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="G19" s="43">
+        <f>IF($L19=0,"",INDEX(Flux!$I$2:$I$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="H19" s="43">
+        <f>IF($L19=0,"",INDEX(Flux!$J$2:$J$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="I19" s="43">
+        <f>IF($L19=0,"",INDEX(Flux!$K$2:$K$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="J19" s="43">
+        <f>IF($L19=0,"",INDEX(Flux!$L$2:$L$35,$L19))</f>
+        <v/>
+      </c>
+      <c r="L19" s="39">
+        <f>IFERROR(MATCH(4,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M19" s="39">
+        <f>IF(L19=0,"",INDEX(Flux!$C$2:$C$35,L19))</f>
+        <v/>
+      </c>
+      <c r="N19" s="39">
+        <f>IF(L19&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" hidden="1" ht="22" customHeight="1">
+      <c r="B20" s="40">
+        <f>IF($L20=0,"",INDEX(Flux!$D$2:$D$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="C20" s="41">
+        <f>IF($L20=0,"",INDEX(Flux!$E$2:$E$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="D20" s="42">
+        <f>IF($L20=0,"",INDEX(Flux!$F$2:$F$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="E20" s="43">
+        <f>IF($L20=0,"",INDEX(Flux!$G$2:$G$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="F20" s="43">
+        <f>IF($L20=0,"",INDEX(Flux!$H$2:$H$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="G20" s="43">
+        <f>IF($L20=0,"",INDEX(Flux!$I$2:$I$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="H20" s="43">
+        <f>IF($L20=0,"",INDEX(Flux!$J$2:$J$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="I20" s="43">
+        <f>IF($L20=0,"",INDEX(Flux!$K$2:$K$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="J20" s="43">
+        <f>IF($L20=0,"",INDEX(Flux!$L$2:$L$35,$L20))</f>
+        <v/>
+      </c>
+      <c r="L20" s="39">
+        <f>IFERROR(MATCH(5,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M20" s="39">
+        <f>IF(L20=0,"",INDEX(Flux!$C$2:$C$35,L20))</f>
+        <v/>
+      </c>
+      <c r="N20" s="39">
+        <f>IF(L20&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" hidden="1" ht="22" customHeight="1">
+      <c r="B21" s="40">
+        <f>IF($L21=0,"",INDEX(Flux!$D$2:$D$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="C21" s="41">
+        <f>IF($L21=0,"",INDEX(Flux!$E$2:$E$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="D21" s="42">
+        <f>IF($L21=0,"",INDEX(Flux!$F$2:$F$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="E21" s="43">
+        <f>IF($L21=0,"",INDEX(Flux!$G$2:$G$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="F21" s="43">
+        <f>IF($L21=0,"",INDEX(Flux!$H$2:$H$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="G21" s="43">
+        <f>IF($L21=0,"",INDEX(Flux!$I$2:$I$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="H21" s="43">
+        <f>IF($L21=0,"",INDEX(Flux!$J$2:$J$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="I21" s="43">
+        <f>IF($L21=0,"",INDEX(Flux!$K$2:$K$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="J21" s="43">
+        <f>IF($L21=0,"",INDEX(Flux!$L$2:$L$35,$L21))</f>
+        <v/>
+      </c>
+      <c r="L21" s="39">
+        <f>IFERROR(MATCH(6,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M21" s="39">
+        <f>IF(L21=0,"",INDEX(Flux!$C$2:$C$35,L21))</f>
+        <v/>
+      </c>
+      <c r="N21" s="39">
+        <f>IF(L21&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" hidden="1" ht="22" customHeight="1">
+      <c r="B22" s="40">
+        <f>IF($L22=0,"",INDEX(Flux!$D$2:$D$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="C22" s="41">
+        <f>IF($L22=0,"",INDEX(Flux!$E$2:$E$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="D22" s="42">
+        <f>IF($L22=0,"",INDEX(Flux!$F$2:$F$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="E22" s="43">
+        <f>IF($L22=0,"",INDEX(Flux!$G$2:$G$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="F22" s="43">
+        <f>IF($L22=0,"",INDEX(Flux!$H$2:$H$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="G22" s="43">
+        <f>IF($L22=0,"",INDEX(Flux!$I$2:$I$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="H22" s="43">
+        <f>IF($L22=0,"",INDEX(Flux!$J$2:$J$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="I22" s="43">
+        <f>IF($L22=0,"",INDEX(Flux!$K$2:$K$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="J22" s="43">
+        <f>IF($L22=0,"",INDEX(Flux!$L$2:$L$35,$L22))</f>
+        <v/>
+      </c>
+      <c r="L22" s="39">
+        <f>IFERROR(MATCH(7,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M22" s="39">
+        <f>IF(L22=0,"",INDEX(Flux!$C$2:$C$35,L22))</f>
+        <v/>
+      </c>
+      <c r="N22" s="39">
+        <f>IF(L22&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" hidden="1" ht="22" customHeight="1">
+      <c r="B23" s="40">
+        <f>IF($L23=0,"",INDEX(Flux!$D$2:$D$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="C23" s="41">
+        <f>IF($L23=0,"",INDEX(Flux!$E$2:$E$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="D23" s="42">
+        <f>IF($L23=0,"",INDEX(Flux!$F$2:$F$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="E23" s="43">
+        <f>IF($L23=0,"",INDEX(Flux!$G$2:$G$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="F23" s="43">
+        <f>IF($L23=0,"",INDEX(Flux!$H$2:$H$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="G23" s="43">
+        <f>IF($L23=0,"",INDEX(Flux!$I$2:$I$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="H23" s="43">
+        <f>IF($L23=0,"",INDEX(Flux!$J$2:$J$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="I23" s="43">
+        <f>IF($L23=0,"",INDEX(Flux!$K$2:$K$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="J23" s="43">
+        <f>IF($L23=0,"",INDEX(Flux!$L$2:$L$35,$L23))</f>
+        <v/>
+      </c>
+      <c r="L23" s="39">
+        <f>IFERROR(MATCH(8,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M23" s="39">
+        <f>IF(L23=0,"",INDEX(Flux!$C$2:$C$35,L23))</f>
+        <v/>
+      </c>
+      <c r="N23" s="39">
+        <f>IF(L23&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" hidden="1" ht="22" customHeight="1">
+      <c r="B24" s="40">
+        <f>IF($L24=0,"",INDEX(Flux!$D$2:$D$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="C24" s="41">
+        <f>IF($L24=0,"",INDEX(Flux!$E$2:$E$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="D24" s="42">
+        <f>IF($L24=0,"",INDEX(Flux!$F$2:$F$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="E24" s="43">
+        <f>IF($L24=0,"",INDEX(Flux!$G$2:$G$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="F24" s="43">
+        <f>IF($L24=0,"",INDEX(Flux!$H$2:$H$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="G24" s="43">
+        <f>IF($L24=0,"",INDEX(Flux!$I$2:$I$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="H24" s="43">
+        <f>IF($L24=0,"",INDEX(Flux!$J$2:$J$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="I24" s="43">
+        <f>IF($L24=0,"",INDEX(Flux!$K$2:$K$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="J24" s="43">
+        <f>IF($L24=0,"",INDEX(Flux!$L$2:$L$35,$L24))</f>
+        <v/>
+      </c>
+      <c r="L24" s="39">
+        <f>IFERROR(MATCH(9,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M24" s="39">
+        <f>IF(L24=0,"",INDEX(Flux!$C$2:$C$35,L24))</f>
+        <v/>
+      </c>
+      <c r="N24" s="39">
+        <f>IF(L24&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" hidden="1" ht="22" customHeight="1">
+      <c r="B25" s="40">
+        <f>IF($L25=0,"",INDEX(Flux!$D$2:$D$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="C25" s="41">
+        <f>IF($L25=0,"",INDEX(Flux!$E$2:$E$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="D25" s="42">
+        <f>IF($L25=0,"",INDEX(Flux!$F$2:$F$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="E25" s="43">
+        <f>IF($L25=0,"",INDEX(Flux!$G$2:$G$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="F25" s="43">
+        <f>IF($L25=0,"",INDEX(Flux!$H$2:$H$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="G25" s="43">
+        <f>IF($L25=0,"",INDEX(Flux!$I$2:$I$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="H25" s="43">
+        <f>IF($L25=0,"",INDEX(Flux!$J$2:$J$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="I25" s="43">
+        <f>IF($L25=0,"",INDEX(Flux!$K$2:$K$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="J25" s="43">
+        <f>IF($L25=0,"",INDEX(Flux!$L$2:$L$35,$L25))</f>
+        <v/>
+      </c>
+      <c r="L25" s="39">
+        <f>IFERROR(MATCH(10,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M25" s="39">
+        <f>IF(L25=0,"",INDEX(Flux!$C$2:$C$35,L25))</f>
+        <v/>
+      </c>
+      <c r="N25" s="39">
+        <f>IF(L25&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" hidden="1" ht="22" customHeight="1">
+      <c r="B26" s="40">
+        <f>IF($L26=0,"",INDEX(Flux!$D$2:$D$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="C26" s="41">
+        <f>IF($L26=0,"",INDEX(Flux!$E$2:$E$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="D26" s="42">
+        <f>IF($L26=0,"",INDEX(Flux!$F$2:$F$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="E26" s="43">
+        <f>IF($L26=0,"",INDEX(Flux!$G$2:$G$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="F26" s="43">
+        <f>IF($L26=0,"",INDEX(Flux!$H$2:$H$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="G26" s="43">
+        <f>IF($L26=0,"",INDEX(Flux!$I$2:$I$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="H26" s="43">
+        <f>IF($L26=0,"",INDEX(Flux!$J$2:$J$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="I26" s="43">
+        <f>IF($L26=0,"",INDEX(Flux!$K$2:$K$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="J26" s="43">
+        <f>IF($L26=0,"",INDEX(Flux!$L$2:$L$35,$L26))</f>
+        <v/>
+      </c>
+      <c r="L26" s="39">
+        <f>IFERROR(MATCH(11,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M26" s="39">
+        <f>IF(L26=0,"",INDEX(Flux!$C$2:$C$35,L26))</f>
+        <v/>
+      </c>
+      <c r="N26" s="39">
+        <f>IF(L26&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" hidden="1" ht="22" customHeight="1">
+      <c r="B27" s="40">
+        <f>IF($L27=0,"",INDEX(Flux!$D$2:$D$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="C27" s="41">
+        <f>IF($L27=0,"",INDEX(Flux!$E$2:$E$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="D27" s="42">
+        <f>IF($L27=0,"",INDEX(Flux!$F$2:$F$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="E27" s="43">
+        <f>IF($L27=0,"",INDEX(Flux!$G$2:$G$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="F27" s="43">
+        <f>IF($L27=0,"",INDEX(Flux!$H$2:$H$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="G27" s="43">
+        <f>IF($L27=0,"",INDEX(Flux!$I$2:$I$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="H27" s="43">
+        <f>IF($L27=0,"",INDEX(Flux!$J$2:$J$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="I27" s="43">
+        <f>IF($L27=0,"",INDEX(Flux!$K$2:$K$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="J27" s="43">
+        <f>IF($L27=0,"",INDEX(Flux!$L$2:$L$35,$L27))</f>
+        <v/>
+      </c>
+      <c r="L27" s="39">
+        <f>IFERROR(MATCH(12,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M27" s="39">
+        <f>IF(L27=0,"",INDEX(Flux!$C$2:$C$35,L27))</f>
+        <v/>
+      </c>
+      <c r="N27" s="39">
+        <f>IF(L27&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" hidden="1" ht="22" customHeight="1">
+      <c r="B28" s="40">
+        <f>IF($L28=0,"",INDEX(Flux!$D$2:$D$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="C28" s="41">
+        <f>IF($L28=0,"",INDEX(Flux!$E$2:$E$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="D28" s="42">
+        <f>IF($L28=0,"",INDEX(Flux!$F$2:$F$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="E28" s="43">
+        <f>IF($L28=0,"",INDEX(Flux!$G$2:$G$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="F28" s="43">
+        <f>IF($L28=0,"",INDEX(Flux!$H$2:$H$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="G28" s="43">
+        <f>IF($L28=0,"",INDEX(Flux!$I$2:$I$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="H28" s="43">
+        <f>IF($L28=0,"",INDEX(Flux!$J$2:$J$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="I28" s="43">
+        <f>IF($L28=0,"",INDEX(Flux!$K$2:$K$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="J28" s="43">
+        <f>IF($L28=0,"",INDEX(Flux!$L$2:$L$35,$L28))</f>
+        <v/>
+      </c>
+      <c r="L28" s="39">
+        <f>IFERROR(MATCH(13,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M28" s="39">
+        <f>IF(L28=0,"",INDEX(Flux!$C$2:$C$35,L28))</f>
+        <v/>
+      </c>
+      <c r="N28" s="39">
+        <f>IF(L28&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" hidden="1" ht="22" customHeight="1">
+      <c r="B29" s="40">
+        <f>IF($L29=0,"",INDEX(Flux!$D$2:$D$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="C29" s="41">
+        <f>IF($L29=0,"",INDEX(Flux!$E$2:$E$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="D29" s="42">
+        <f>IF($L29=0,"",INDEX(Flux!$F$2:$F$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="E29" s="43">
+        <f>IF($L29=0,"",INDEX(Flux!$G$2:$G$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="F29" s="43">
+        <f>IF($L29=0,"",INDEX(Flux!$H$2:$H$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="G29" s="43">
+        <f>IF($L29=0,"",INDEX(Flux!$I$2:$I$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="H29" s="43">
+        <f>IF($L29=0,"",INDEX(Flux!$J$2:$J$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="I29" s="43">
+        <f>IF($L29=0,"",INDEX(Flux!$K$2:$K$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="J29" s="43">
+        <f>IF($L29=0,"",INDEX(Flux!$L$2:$L$35,$L29))</f>
+        <v/>
+      </c>
+      <c r="L29" s="39">
+        <f>IFERROR(MATCH(14,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M29" s="39">
+        <f>IF(L29=0,"",INDEX(Flux!$C$2:$C$35,L29))</f>
+        <v/>
+      </c>
+      <c r="N29" s="39">
+        <f>IF(L29&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" hidden="1" ht="22" customHeight="1">
+      <c r="B30" s="40">
+        <f>IF($L30=0,"",INDEX(Flux!$D$2:$D$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="C30" s="41">
+        <f>IF($L30=0,"",INDEX(Flux!$E$2:$E$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="D30" s="42">
+        <f>IF($L30=0,"",INDEX(Flux!$F$2:$F$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="E30" s="43">
+        <f>IF($L30=0,"",INDEX(Flux!$G$2:$G$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="F30" s="43">
+        <f>IF($L30=0,"",INDEX(Flux!$H$2:$H$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="G30" s="43">
+        <f>IF($L30=0,"",INDEX(Flux!$I$2:$I$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="H30" s="43">
+        <f>IF($L30=0,"",INDEX(Flux!$J$2:$J$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="I30" s="43">
+        <f>IF($L30=0,"",INDEX(Flux!$K$2:$K$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="J30" s="43">
+        <f>IF($L30=0,"",INDEX(Flux!$L$2:$L$35,$L30))</f>
+        <v/>
+      </c>
+      <c r="L30" s="39">
+        <f>IFERROR(MATCH(15,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M30" s="39">
+        <f>IF(L30=0,"",INDEX(Flux!$C$2:$C$35,L30))</f>
+        <v/>
+      </c>
+      <c r="N30" s="39">
+        <f>IF(L30&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" hidden="1" ht="22" customHeight="1">
+      <c r="B31" s="40">
+        <f>IF($L31=0,"",INDEX(Flux!$D$2:$D$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="C31" s="41">
+        <f>IF($L31=0,"",INDEX(Flux!$E$2:$E$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="D31" s="42">
+        <f>IF($L31=0,"",INDEX(Flux!$F$2:$F$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="E31" s="43">
+        <f>IF($L31=0,"",INDEX(Flux!$G$2:$G$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="F31" s="43">
+        <f>IF($L31=0,"",INDEX(Flux!$H$2:$H$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="G31" s="43">
+        <f>IF($L31=0,"",INDEX(Flux!$I$2:$I$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="H31" s="43">
+        <f>IF($L31=0,"",INDEX(Flux!$J$2:$J$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="I31" s="43">
+        <f>IF($L31=0,"",INDEX(Flux!$K$2:$K$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="J31" s="43">
+        <f>IF($L31=0,"",INDEX(Flux!$L$2:$L$35,$L31))</f>
+        <v/>
+      </c>
+      <c r="L31" s="39">
+        <f>IFERROR(MATCH(16,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M31" s="39">
+        <f>IF(L31=0,"",INDEX(Flux!$C$2:$C$35,L31))</f>
+        <v/>
+      </c>
+      <c r="N31" s="39">
+        <f>IF(L31&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" hidden="1" ht="22" customHeight="1">
+      <c r="B32" s="40">
+        <f>IF($L32=0,"",INDEX(Flux!$D$2:$D$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="C32" s="41">
+        <f>IF($L32=0,"",INDEX(Flux!$E$2:$E$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="D32" s="42">
+        <f>IF($L32=0,"",INDEX(Flux!$F$2:$F$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="E32" s="43">
+        <f>IF($L32=0,"",INDEX(Flux!$G$2:$G$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="F32" s="43">
+        <f>IF($L32=0,"",INDEX(Flux!$H$2:$H$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="G32" s="43">
+        <f>IF($L32=0,"",INDEX(Flux!$I$2:$I$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="H32" s="43">
+        <f>IF($L32=0,"",INDEX(Flux!$J$2:$J$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="I32" s="43">
+        <f>IF($L32=0,"",INDEX(Flux!$K$2:$K$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="J32" s="43">
+        <f>IF($L32=0,"",INDEX(Flux!$L$2:$L$35,$L32))</f>
+        <v/>
+      </c>
+      <c r="L32" s="39">
+        <f>IFERROR(MATCH(17,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M32" s="39">
+        <f>IF(L32=0,"",INDEX(Flux!$C$2:$C$35,L32))</f>
+        <v/>
+      </c>
+      <c r="N32" s="39">
+        <f>IF(L32&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" hidden="1" ht="22" customHeight="1">
+      <c r="B33" s="40">
+        <f>IF($L33=0,"",INDEX(Flux!$D$2:$D$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="C33" s="41">
+        <f>IF($L33=0,"",INDEX(Flux!$E$2:$E$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="D33" s="42">
+        <f>IF($L33=0,"",INDEX(Flux!$F$2:$F$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="E33" s="43">
+        <f>IF($L33=0,"",INDEX(Flux!$G$2:$G$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="F33" s="43">
+        <f>IF($L33=0,"",INDEX(Flux!$H$2:$H$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="G33" s="43">
+        <f>IF($L33=0,"",INDEX(Flux!$I$2:$I$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="H33" s="43">
+        <f>IF($L33=0,"",INDEX(Flux!$J$2:$J$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="I33" s="43">
+        <f>IF($L33=0,"",INDEX(Flux!$K$2:$K$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="J33" s="43">
+        <f>IF($L33=0,"",INDEX(Flux!$L$2:$L$35,$L33))</f>
+        <v/>
+      </c>
+      <c r="L33" s="39">
+        <f>IFERROR(MATCH(18,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M33" s="39">
+        <f>IF(L33=0,"",INDEX(Flux!$C$2:$C$35,L33))</f>
+        <v/>
+      </c>
+      <c r="N33" s="39">
+        <f>IF(L33&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" hidden="1" ht="22" customHeight="1">
+      <c r="B34" s="40">
+        <f>IF($L34=0,"",INDEX(Flux!$D$2:$D$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="C34" s="41">
+        <f>IF($L34=0,"",INDEX(Flux!$E$2:$E$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="D34" s="42">
+        <f>IF($L34=0,"",INDEX(Flux!$F$2:$F$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="E34" s="43">
+        <f>IF($L34=0,"",INDEX(Flux!$G$2:$G$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="F34" s="43">
+        <f>IF($L34=0,"",INDEX(Flux!$H$2:$H$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="G34" s="43">
+        <f>IF($L34=0,"",INDEX(Flux!$I$2:$I$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="H34" s="43">
+        <f>IF($L34=0,"",INDEX(Flux!$J$2:$J$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="I34" s="43">
+        <f>IF($L34=0,"",INDEX(Flux!$K$2:$K$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="J34" s="43">
+        <f>IF($L34=0,"",INDEX(Flux!$L$2:$L$35,$L34))</f>
+        <v/>
+      </c>
+      <c r="L34" s="39">
+        <f>IFERROR(MATCH(19,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M34" s="39">
+        <f>IF(L34=0,"",INDEX(Flux!$C$2:$C$35,L34))</f>
+        <v/>
+      </c>
+      <c r="N34" s="39">
+        <f>IF(L34&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" hidden="1" ht="22" customHeight="1">
+      <c r="B35" s="40">
+        <f>IF($L35=0,"",INDEX(Flux!$D$2:$D$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="C35" s="41">
+        <f>IF($L35=0,"",INDEX(Flux!$E$2:$E$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="D35" s="42">
+        <f>IF($L35=0,"",INDEX(Flux!$F$2:$F$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="E35" s="43">
+        <f>IF($L35=0,"",INDEX(Flux!$G$2:$G$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="F35" s="43">
+        <f>IF($L35=0,"",INDEX(Flux!$H$2:$H$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="G35" s="43">
+        <f>IF($L35=0,"",INDEX(Flux!$I$2:$I$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="H35" s="43">
+        <f>IF($L35=0,"",INDEX(Flux!$J$2:$J$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="I35" s="43">
+        <f>IF($L35=0,"",INDEX(Flux!$K$2:$K$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="J35" s="43">
+        <f>IF($L35=0,"",INDEX(Flux!$L$2:$L$35,$L35))</f>
+        <v/>
+      </c>
+      <c r="L35" s="39">
+        <f>IFERROR(MATCH(20,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M35" s="39">
+        <f>IF(L35=0,"",INDEX(Flux!$C$2:$C$35,L35))</f>
+        <v/>
+      </c>
+      <c r="N35" s="39">
+        <f>IF(L35&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" hidden="1" ht="22" customHeight="1">
+      <c r="B36" s="40">
+        <f>IF($L36=0,"",INDEX(Flux!$D$2:$D$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="C36" s="41">
+        <f>IF($L36=0,"",INDEX(Flux!$E$2:$E$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="D36" s="42">
+        <f>IF($L36=0,"",INDEX(Flux!$F$2:$F$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="E36" s="43">
+        <f>IF($L36=0,"",INDEX(Flux!$G$2:$G$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="F36" s="43">
+        <f>IF($L36=0,"",INDEX(Flux!$H$2:$H$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="G36" s="43">
+        <f>IF($L36=0,"",INDEX(Flux!$I$2:$I$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="H36" s="43">
+        <f>IF($L36=0,"",INDEX(Flux!$J$2:$J$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="I36" s="43">
+        <f>IF($L36=0,"",INDEX(Flux!$K$2:$K$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="J36" s="43">
+        <f>IF($L36=0,"",INDEX(Flux!$L$2:$L$35,$L36))</f>
+        <v/>
+      </c>
+      <c r="L36" s="39">
+        <f>IFERROR(MATCH(21,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M36" s="39">
+        <f>IF(L36=0,"",INDEX(Flux!$C$2:$C$35,L36))</f>
+        <v/>
+      </c>
+      <c r="N36" s="39">
+        <f>IF(L36&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" hidden="1" ht="22" customHeight="1">
+      <c r="B37" s="40">
+        <f>IF($L37=0,"",INDEX(Flux!$D$2:$D$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="C37" s="41">
+        <f>IF($L37=0,"",INDEX(Flux!$E$2:$E$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="D37" s="42">
+        <f>IF($L37=0,"",INDEX(Flux!$F$2:$F$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="E37" s="43">
+        <f>IF($L37=0,"",INDEX(Flux!$G$2:$G$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="F37" s="43">
+        <f>IF($L37=0,"",INDEX(Flux!$H$2:$H$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="G37" s="43">
+        <f>IF($L37=0,"",INDEX(Flux!$I$2:$I$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="H37" s="43">
+        <f>IF($L37=0,"",INDEX(Flux!$J$2:$J$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="I37" s="43">
+        <f>IF($L37=0,"",INDEX(Flux!$K$2:$K$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="J37" s="43">
+        <f>IF($L37=0,"",INDEX(Flux!$L$2:$L$35,$L37))</f>
+        <v/>
+      </c>
+      <c r="L37" s="39">
+        <f>IFERROR(MATCH(22,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M37" s="39">
+        <f>IF(L37=0,"",INDEX(Flux!$C$2:$C$35,L37))</f>
+        <v/>
+      </c>
+      <c r="N37" s="39">
+        <f>IF(L37&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" hidden="1" ht="22" customHeight="1">
+      <c r="B38" s="40">
+        <f>IF($L38=0,"",INDEX(Flux!$D$2:$D$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="C38" s="41">
+        <f>IF($L38=0,"",INDEX(Flux!$E$2:$E$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="D38" s="42">
+        <f>IF($L38=0,"",INDEX(Flux!$F$2:$F$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="E38" s="43">
+        <f>IF($L38=0,"",INDEX(Flux!$G$2:$G$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="F38" s="43">
+        <f>IF($L38=0,"",INDEX(Flux!$H$2:$H$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="G38" s="43">
+        <f>IF($L38=0,"",INDEX(Flux!$I$2:$I$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="H38" s="43">
+        <f>IF($L38=0,"",INDEX(Flux!$J$2:$J$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="I38" s="43">
+        <f>IF($L38=0,"",INDEX(Flux!$K$2:$K$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="J38" s="43">
+        <f>IF($L38=0,"",INDEX(Flux!$L$2:$L$35,$L38))</f>
+        <v/>
+      </c>
+      <c r="L38" s="39">
+        <f>IFERROR(MATCH(23,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M38" s="39">
+        <f>IF(L38=0,"",INDEX(Flux!$C$2:$C$35,L38))</f>
+        <v/>
+      </c>
+      <c r="N38" s="39">
+        <f>IF(L38&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" hidden="1" ht="22" customHeight="1">
+      <c r="B39" s="40">
+        <f>IF($L39=0,"",INDEX(Flux!$D$2:$D$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="C39" s="41">
+        <f>IF($L39=0,"",INDEX(Flux!$E$2:$E$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="D39" s="42">
+        <f>IF($L39=0,"",INDEX(Flux!$F$2:$F$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="E39" s="43">
+        <f>IF($L39=0,"",INDEX(Flux!$G$2:$G$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="F39" s="43">
+        <f>IF($L39=0,"",INDEX(Flux!$H$2:$H$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="G39" s="43">
+        <f>IF($L39=0,"",INDEX(Flux!$I$2:$I$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="H39" s="43">
+        <f>IF($L39=0,"",INDEX(Flux!$J$2:$J$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="I39" s="43">
+        <f>IF($L39=0,"",INDEX(Flux!$K$2:$K$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="J39" s="43">
+        <f>IF($L39=0,"",INDEX(Flux!$L$2:$L$35,$L39))</f>
+        <v/>
+      </c>
+      <c r="L39" s="39">
+        <f>IFERROR(MATCH(24,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M39" s="39">
+        <f>IF(L39=0,"",INDEX(Flux!$C$2:$C$35,L39))</f>
+        <v/>
+      </c>
+      <c r="N39" s="39">
+        <f>IF(L39&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" hidden="1" ht="22" customHeight="1">
+      <c r="B40" s="40">
+        <f>IF($L40=0,"",INDEX(Flux!$D$2:$D$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="C40" s="41">
+        <f>IF($L40=0,"",INDEX(Flux!$E$2:$E$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="D40" s="42">
+        <f>IF($L40=0,"",INDEX(Flux!$F$2:$F$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="E40" s="43">
+        <f>IF($L40=0,"",INDEX(Flux!$G$2:$G$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="F40" s="43">
+        <f>IF($L40=0,"",INDEX(Flux!$H$2:$H$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="G40" s="43">
+        <f>IF($L40=0,"",INDEX(Flux!$I$2:$I$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="H40" s="43">
+        <f>IF($L40=0,"",INDEX(Flux!$J$2:$J$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="I40" s="43">
+        <f>IF($L40=0,"",INDEX(Flux!$K$2:$K$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="J40" s="43">
+        <f>IF($L40=0,"",INDEX(Flux!$L$2:$L$35,$L40))</f>
+        <v/>
+      </c>
+      <c r="L40" s="39">
+        <f>IFERROR(MATCH(25,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M40" s="39">
+        <f>IF(L40=0,"",INDEX(Flux!$C$2:$C$35,L40))</f>
+        <v/>
+      </c>
+      <c r="N40" s="39">
+        <f>IF(L40&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" hidden="1" ht="22" customHeight="1">
+      <c r="B41" s="40">
+        <f>IF($L41=0,"",INDEX(Flux!$D$2:$D$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="C41" s="41">
+        <f>IF($L41=0,"",INDEX(Flux!$E$2:$E$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="D41" s="42">
+        <f>IF($L41=0,"",INDEX(Flux!$F$2:$F$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="E41" s="43">
+        <f>IF($L41=0,"",INDEX(Flux!$G$2:$G$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="F41" s="43">
+        <f>IF($L41=0,"",INDEX(Flux!$H$2:$H$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="G41" s="43">
+        <f>IF($L41=0,"",INDEX(Flux!$I$2:$I$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="H41" s="43">
+        <f>IF($L41=0,"",INDEX(Flux!$J$2:$J$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="I41" s="43">
+        <f>IF($L41=0,"",INDEX(Flux!$K$2:$K$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="J41" s="43">
+        <f>IF($L41=0,"",INDEX(Flux!$L$2:$L$35,$L41))</f>
+        <v/>
+      </c>
+      <c r="L41" s="39">
+        <f>IFERROR(MATCH(26,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M41" s="39">
+        <f>IF(L41=0,"",INDEX(Flux!$C$2:$C$35,L41))</f>
+        <v/>
+      </c>
+      <c r="N41" s="39">
+        <f>IF(L41&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" hidden="1" ht="22" customHeight="1">
+      <c r="B42" s="40">
+        <f>IF($L42=0,"",INDEX(Flux!$D$2:$D$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="C42" s="41">
+        <f>IF($L42=0,"",INDEX(Flux!$E$2:$E$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="D42" s="42">
+        <f>IF($L42=0,"",INDEX(Flux!$F$2:$F$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="E42" s="43">
+        <f>IF($L42=0,"",INDEX(Flux!$G$2:$G$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="F42" s="43">
+        <f>IF($L42=0,"",INDEX(Flux!$H$2:$H$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="G42" s="43">
+        <f>IF($L42=0,"",INDEX(Flux!$I$2:$I$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="H42" s="43">
+        <f>IF($L42=0,"",INDEX(Flux!$J$2:$J$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="I42" s="43">
+        <f>IF($L42=0,"",INDEX(Flux!$K$2:$K$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="J42" s="43">
+        <f>IF($L42=0,"",INDEX(Flux!$L$2:$L$35,$L42))</f>
+        <v/>
+      </c>
+      <c r="L42" s="39">
+        <f>IFERROR(MATCH(27,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M42" s="39">
+        <f>IF(L42=0,"",INDEX(Flux!$C$2:$C$35,L42))</f>
+        <v/>
+      </c>
+      <c r="N42" s="39">
+        <f>IF(L42&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" hidden="1" ht="22" customHeight="1">
+      <c r="B43" s="40">
+        <f>IF($L43=0,"",INDEX(Flux!$D$2:$D$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="C43" s="41">
+        <f>IF($L43=0,"",INDEX(Flux!$E$2:$E$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="D43" s="42">
+        <f>IF($L43=0,"",INDEX(Flux!$F$2:$F$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="E43" s="43">
+        <f>IF($L43=0,"",INDEX(Flux!$G$2:$G$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="F43" s="43">
+        <f>IF($L43=0,"",INDEX(Flux!$H$2:$H$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="G43" s="43">
+        <f>IF($L43=0,"",INDEX(Flux!$I$2:$I$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="H43" s="43">
+        <f>IF($L43=0,"",INDEX(Flux!$J$2:$J$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="I43" s="43">
+        <f>IF($L43=0,"",INDEX(Flux!$K$2:$K$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="J43" s="43">
+        <f>IF($L43=0,"",INDEX(Flux!$L$2:$L$35,$L43))</f>
+        <v/>
+      </c>
+      <c r="L43" s="39">
+        <f>IFERROR(MATCH(28,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M43" s="39">
+        <f>IF(L43=0,"",INDEX(Flux!$C$2:$C$35,L43))</f>
+        <v/>
+      </c>
+      <c r="N43" s="39">
+        <f>IF(L43&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" hidden="1" ht="22" customHeight="1">
+      <c r="B44" s="40">
+        <f>IF($L44=0,"",INDEX(Flux!$D$2:$D$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="C44" s="41">
+        <f>IF($L44=0,"",INDEX(Flux!$E$2:$E$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="D44" s="42">
+        <f>IF($L44=0,"",INDEX(Flux!$F$2:$F$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="E44" s="43">
+        <f>IF($L44=0,"",INDEX(Flux!$G$2:$G$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="F44" s="43">
+        <f>IF($L44=0,"",INDEX(Flux!$H$2:$H$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="G44" s="43">
+        <f>IF($L44=0,"",INDEX(Flux!$I$2:$I$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="H44" s="43">
+        <f>IF($L44=0,"",INDEX(Flux!$J$2:$J$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="I44" s="43">
+        <f>IF($L44=0,"",INDEX(Flux!$K$2:$K$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="J44" s="43">
+        <f>IF($L44=0,"",INDEX(Flux!$L$2:$L$35,$L44))</f>
+        <v/>
+      </c>
+      <c r="L44" s="39">
+        <f>IFERROR(MATCH(29,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M44" s="39">
+        <f>IF(L44=0,"",INDEX(Flux!$C$2:$C$35,L44))</f>
+        <v/>
+      </c>
+      <c r="N44" s="39">
+        <f>IF(L44&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" hidden="1" ht="22" customHeight="1">
+      <c r="B45" s="40">
+        <f>IF($L45=0,"",INDEX(Flux!$D$2:$D$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="C45" s="41">
+        <f>IF($L45=0,"",INDEX(Flux!$E$2:$E$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="D45" s="42">
+        <f>IF($L45=0,"",INDEX(Flux!$F$2:$F$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="E45" s="43">
+        <f>IF($L45=0,"",INDEX(Flux!$G$2:$G$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="F45" s="43">
+        <f>IF($L45=0,"",INDEX(Flux!$H$2:$H$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="G45" s="43">
+        <f>IF($L45=0,"",INDEX(Flux!$I$2:$I$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="H45" s="43">
+        <f>IF($L45=0,"",INDEX(Flux!$J$2:$J$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="I45" s="43">
+        <f>IF($L45=0,"",INDEX(Flux!$K$2:$K$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="J45" s="43">
+        <f>IF($L45=0,"",INDEX(Flux!$L$2:$L$35,$L45))</f>
+        <v/>
+      </c>
+      <c r="L45" s="39">
+        <f>IFERROR(MATCH(30,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M45" s="39">
+        <f>IF(L45=0,"",INDEX(Flux!$C$2:$C$35,L45))</f>
+        <v/>
+      </c>
+      <c r="N45" s="39">
+        <f>IF(L45&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" hidden="1" ht="22" customHeight="1">
+      <c r="B46" s="40">
+        <f>IF($L46=0,"",INDEX(Flux!$D$2:$D$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="C46" s="41">
+        <f>IF($L46=0,"",INDEX(Flux!$E$2:$E$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="D46" s="42">
+        <f>IF($L46=0,"",INDEX(Flux!$F$2:$F$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="E46" s="43">
+        <f>IF($L46=0,"",INDEX(Flux!$G$2:$G$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="F46" s="43">
+        <f>IF($L46=0,"",INDEX(Flux!$H$2:$H$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="G46" s="43">
+        <f>IF($L46=0,"",INDEX(Flux!$I$2:$I$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="H46" s="43">
+        <f>IF($L46=0,"",INDEX(Flux!$J$2:$J$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="I46" s="43">
+        <f>IF($L46=0,"",INDEX(Flux!$K$2:$K$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="J46" s="43">
+        <f>IF($L46=0,"",INDEX(Flux!$L$2:$L$35,$L46))</f>
+        <v/>
+      </c>
+      <c r="L46" s="39">
+        <f>IFERROR(MATCH(31,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M46" s="39">
+        <f>IF(L46=0,"",INDEX(Flux!$C$2:$C$35,L46))</f>
+        <v/>
+      </c>
+      <c r="N46" s="39">
+        <f>IF(L46&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" hidden="1" ht="22" customHeight="1">
+      <c r="B47" s="40">
+        <f>IF($L47=0,"",INDEX(Flux!$D$2:$D$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="C47" s="41">
+        <f>IF($L47=0,"",INDEX(Flux!$E$2:$E$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="D47" s="42">
+        <f>IF($L47=0,"",INDEX(Flux!$F$2:$F$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="E47" s="43">
+        <f>IF($L47=0,"",INDEX(Flux!$G$2:$G$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="F47" s="43">
+        <f>IF($L47=0,"",INDEX(Flux!$H$2:$H$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="G47" s="43">
+        <f>IF($L47=0,"",INDEX(Flux!$I$2:$I$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="H47" s="43">
+        <f>IF($L47=0,"",INDEX(Flux!$J$2:$J$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="I47" s="43">
+        <f>IF($L47=0,"",INDEX(Flux!$K$2:$K$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="J47" s="43">
+        <f>IF($L47=0,"",INDEX(Flux!$L$2:$L$35,$L47))</f>
+        <v/>
+      </c>
+      <c r="L47" s="39">
+        <f>IFERROR(MATCH(32,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M47" s="39">
+        <f>IF(L47=0,"",INDEX(Flux!$C$2:$C$35,L47))</f>
+        <v/>
+      </c>
+      <c r="N47" s="39">
+        <f>IF(L47&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" hidden="1" ht="22" customHeight="1">
+      <c r="B48" s="40">
+        <f>IF($L48=0,"",INDEX(Flux!$D$2:$D$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="C48" s="41">
+        <f>IF($L48=0,"",INDEX(Flux!$E$2:$E$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="D48" s="42">
+        <f>IF($L48=0,"",INDEX(Flux!$F$2:$F$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="E48" s="43">
+        <f>IF($L48=0,"",INDEX(Flux!$G$2:$G$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="F48" s="43">
+        <f>IF($L48=0,"",INDEX(Flux!$H$2:$H$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="G48" s="43">
+        <f>IF($L48=0,"",INDEX(Flux!$I$2:$I$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="H48" s="43">
+        <f>IF($L48=0,"",INDEX(Flux!$J$2:$J$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="I48" s="43">
+        <f>IF($L48=0,"",INDEX(Flux!$K$2:$K$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="J48" s="43">
+        <f>IF($L48=0,"",INDEX(Flux!$L$2:$L$35,$L48))</f>
+        <v/>
+      </c>
+      <c r="L48" s="39">
+        <f>IFERROR(MATCH(33,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M48" s="39">
+        <f>IF(L48=0,"",INDEX(Flux!$C$2:$C$35,L48))</f>
+        <v/>
+      </c>
+      <c r="N48" s="39">
+        <f>IF(L48&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" hidden="1" ht="22" customHeight="1">
+      <c r="B49" s="40">
+        <f>IF($L49=0,"",INDEX(Flux!$D$2:$D$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="C49" s="41">
+        <f>IF($L49=0,"",INDEX(Flux!$E$2:$E$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="D49" s="42">
+        <f>IF($L49=0,"",INDEX(Flux!$F$2:$F$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="E49" s="43">
+        <f>IF($L49=0,"",INDEX(Flux!$G$2:$G$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="F49" s="43">
+        <f>IF($L49=0,"",INDEX(Flux!$H$2:$H$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="G49" s="43">
+        <f>IF($L49=0,"",INDEX(Flux!$I$2:$I$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="H49" s="43">
+        <f>IF($L49=0,"",INDEX(Flux!$J$2:$J$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="I49" s="43">
+        <f>IF($L49=0,"",INDEX(Flux!$K$2:$K$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="J49" s="43">
+        <f>IF($L49=0,"",INDEX(Flux!$L$2:$L$35,$L49))</f>
+        <v/>
+      </c>
+      <c r="L49" s="39">
+        <f>IFERROR(MATCH(34,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M49" s="39">
+        <f>IF(L49=0,"",INDEX(Flux!$C$2:$C$35,L49))</f>
+        <v/>
+      </c>
+      <c r="N49" s="39">
+        <f>IF(L49&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" hidden="1" ht="22" customHeight="1">
+      <c r="B50" s="40">
+        <f>IF($L50=0,"",INDEX(Flux!$D$2:$D$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="C50" s="41">
+        <f>IF($L50=0,"",INDEX(Flux!$E$2:$E$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="D50" s="42">
+        <f>IF($L50=0,"",INDEX(Flux!$F$2:$F$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="E50" s="43">
+        <f>IF($L50=0,"",INDEX(Flux!$G$2:$G$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="F50" s="43">
+        <f>IF($L50=0,"",INDEX(Flux!$H$2:$H$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="G50" s="43">
+        <f>IF($L50=0,"",INDEX(Flux!$I$2:$I$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="H50" s="43">
+        <f>IF($L50=0,"",INDEX(Flux!$J$2:$J$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="I50" s="43">
+        <f>IF($L50=0,"",INDEX(Flux!$K$2:$K$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="J50" s="43">
+        <f>IF($L50=0,"",INDEX(Flux!$L$2:$L$35,$L50))</f>
+        <v/>
+      </c>
+      <c r="L50" s="39">
+        <f>IFERROR(MATCH(35,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M50" s="39">
+        <f>IF(L50=0,"",INDEX(Flux!$C$2:$C$35,L50))</f>
+        <v/>
+      </c>
+      <c r="N50" s="39">
+        <f>IF(L50&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" hidden="1" ht="22" customHeight="1">
+      <c r="B51" s="40">
+        <f>IF($L51=0,"",INDEX(Flux!$D$2:$D$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="C51" s="41">
+        <f>IF($L51=0,"",INDEX(Flux!$E$2:$E$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="D51" s="42">
+        <f>IF($L51=0,"",INDEX(Flux!$F$2:$F$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="E51" s="43">
+        <f>IF($L51=0,"",INDEX(Flux!$G$2:$G$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="F51" s="43">
+        <f>IF($L51=0,"",INDEX(Flux!$H$2:$H$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="G51" s="43">
+        <f>IF($L51=0,"",INDEX(Flux!$I$2:$I$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="H51" s="43">
+        <f>IF($L51=0,"",INDEX(Flux!$J$2:$J$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="I51" s="43">
+        <f>IF($L51=0,"",INDEX(Flux!$K$2:$K$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="J51" s="43">
+        <f>IF($L51=0,"",INDEX(Flux!$L$2:$L$35,$L51))</f>
+        <v/>
+      </c>
+      <c r="L51" s="39">
+        <f>IFERROR(MATCH(36,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M51" s="39">
+        <f>IF(L51=0,"",INDEX(Flux!$C$2:$C$35,L51))</f>
+        <v/>
+      </c>
+      <c r="N51" s="39">
+        <f>IF(L51&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" hidden="1" ht="22" customHeight="1">
+      <c r="B52" s="40">
+        <f>IF($L52=0,"",INDEX(Flux!$D$2:$D$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="C52" s="41">
+        <f>IF($L52=0,"",INDEX(Flux!$E$2:$E$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="D52" s="42">
+        <f>IF($L52=0,"",INDEX(Flux!$F$2:$F$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="E52" s="43">
+        <f>IF($L52=0,"",INDEX(Flux!$G$2:$G$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="F52" s="43">
+        <f>IF($L52=0,"",INDEX(Flux!$H$2:$H$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="G52" s="43">
+        <f>IF($L52=0,"",INDEX(Flux!$I$2:$I$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="H52" s="43">
+        <f>IF($L52=0,"",INDEX(Flux!$J$2:$J$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="I52" s="43">
+        <f>IF($L52=0,"",INDEX(Flux!$K$2:$K$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="J52" s="43">
+        <f>IF($L52=0,"",INDEX(Flux!$L$2:$L$35,$L52))</f>
+        <v/>
+      </c>
+      <c r="L52" s="39">
+        <f>IFERROR(MATCH(37,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M52" s="39">
+        <f>IF(L52=0,"",INDEX(Flux!$C$2:$C$35,L52))</f>
+        <v/>
+      </c>
+      <c r="N52" s="39">
+        <f>IF(L52&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" hidden="1" ht="22" customHeight="1">
+      <c r="B53" s="40">
+        <f>IF($L53=0,"",INDEX(Flux!$D$2:$D$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="C53" s="41">
+        <f>IF($L53=0,"",INDEX(Flux!$E$2:$E$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="D53" s="42">
+        <f>IF($L53=0,"",INDEX(Flux!$F$2:$F$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="E53" s="43">
+        <f>IF($L53=0,"",INDEX(Flux!$G$2:$G$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="F53" s="43">
+        <f>IF($L53=0,"",INDEX(Flux!$H$2:$H$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="G53" s="43">
+        <f>IF($L53=0,"",INDEX(Flux!$I$2:$I$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="H53" s="43">
+        <f>IF($L53=0,"",INDEX(Flux!$J$2:$J$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="I53" s="43">
+        <f>IF($L53=0,"",INDEX(Flux!$K$2:$K$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="J53" s="43">
+        <f>IF($L53=0,"",INDEX(Flux!$L$2:$L$35,$L53))</f>
+        <v/>
+      </c>
+      <c r="L53" s="39">
+        <f>IFERROR(MATCH(38,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M53" s="39">
+        <f>IF(L53=0,"",INDEX(Flux!$C$2:$C$35,L53))</f>
+        <v/>
+      </c>
+      <c r="N53" s="39">
+        <f>IF(L53&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" hidden="1" ht="22" customHeight="1">
+      <c r="B54" s="40">
+        <f>IF($L54=0,"",INDEX(Flux!$D$2:$D$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="C54" s="41">
+        <f>IF($L54=0,"",INDEX(Flux!$E$2:$E$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="D54" s="42">
+        <f>IF($L54=0,"",INDEX(Flux!$F$2:$F$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="E54" s="43">
+        <f>IF($L54=0,"",INDEX(Flux!$G$2:$G$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="F54" s="43">
+        <f>IF($L54=0,"",INDEX(Flux!$H$2:$H$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="G54" s="43">
+        <f>IF($L54=0,"",INDEX(Flux!$I$2:$I$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="H54" s="43">
+        <f>IF($L54=0,"",INDEX(Flux!$J$2:$J$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="I54" s="43">
+        <f>IF($L54=0,"",INDEX(Flux!$K$2:$K$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="J54" s="43">
+        <f>IF($L54=0,"",INDEX(Flux!$L$2:$L$35,$L54))</f>
+        <v/>
+      </c>
+      <c r="L54" s="39">
+        <f>IFERROR(MATCH(39,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M54" s="39">
+        <f>IF(L54=0,"",INDEX(Flux!$C$2:$C$35,L54))</f>
+        <v/>
+      </c>
+      <c r="N54" s="39">
+        <f>IF(L54&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" hidden="1" ht="22" customHeight="1">
+      <c r="B55" s="40">
+        <f>IF($L55=0,"",INDEX(Flux!$D$2:$D$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="C55" s="41">
+        <f>IF($L55=0,"",INDEX(Flux!$E$2:$E$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="D55" s="42">
+        <f>IF($L55=0,"",INDEX(Flux!$F$2:$F$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="E55" s="43">
+        <f>IF($L55=0,"",INDEX(Flux!$G$2:$G$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="F55" s="43">
+        <f>IF($L55=0,"",INDEX(Flux!$H$2:$H$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="G55" s="43">
+        <f>IF($L55=0,"",INDEX(Flux!$I$2:$I$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="H55" s="43">
+        <f>IF($L55=0,"",INDEX(Flux!$J$2:$J$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="I55" s="43">
+        <f>IF($L55=0,"",INDEX(Flux!$K$2:$K$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="J55" s="43">
+        <f>IF($L55=0,"",INDEX(Flux!$L$2:$L$35,$L55))</f>
+        <v/>
+      </c>
+      <c r="L55" s="39">
+        <f>IFERROR(MATCH(40,Flux!$B$2:$B$35,0),0)</f>
+        <v/>
+      </c>
+      <c r="M55" s="39">
+        <f>IF(L55=0,"",INDEX(Flux!$C$2:$C$35,L55))</f>
+        <v/>
+      </c>
+      <c r="N55" s="39">
+        <f>IF(L55&gt;0,1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1"/>
+    <row r="57" ht="22" customHeight="1"/>
     <row r="58" ht="20" customHeight="1">
-      <c r="B58" s="34">
+      <c r="B58" s="35">
         <f>INDEX(Textes!$B$2:$C$59,MATCH("sec_cond",Textes!$A$2:$A$59,0),Listes!$H$1)</f>
         <v/>
       </c>
-      <c r="C58" s="35" t="n"/>
-      <c r="D58" s="35" t="n"/>
-      <c r="E58" s="35" t="n"/>
-      <c r="F58" s="35" t="n"/>
-      <c r="G58" s="35" t="n"/>
-      <c r="H58" s="35" t="n"/>
-      <c r="I58" s="35" t="n"/>
-      <c r="J58" s="35" t="n"/>
-    </row>
-    <row r="59" ht="92" customHeight="1">
+      <c r="C58" s="36" t="n"/>
+      <c r="D58" s="36" t="n"/>
+      <c r="E58" s="36" t="n"/>
+      <c r="F58" s="36" t="n"/>
+      <c r="G58" s="36" t="n"/>
+      <c r="H58" s="36" t="n"/>
+      <c r="I58" s="36" t="n"/>
+      <c r="J58" s="36" t="n"/>
+    </row>
+    <row r="59" ht="80" customHeight="1">
       <c r="B59" s="44" t="inlineStr">
         <is>
           <t>La location s'entend depuis le jour de départ de la base d'origine jusqu'à son retour au même endroit.
@@ -4581,7 +4757,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="92" customHeight="1">
+    <row r="60" ht="80" customHeight="1">
       <c r="B60" s="44" t="inlineStr">
         <is>
           <t>The rental is from the day of departure from the base of origin until its return to the same place.
@@ -4660,6 +4836,25 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B15:N55">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0">
+      <customFilters>
+        <customFilter val="0" operator="greaterThan"/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="12" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <mergeCells count="36">
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="B7:C7"/>
@@ -4668,6 +4863,7 @@
     <mergeCell ref="B14:J14"/>
     <mergeCell ref="B60:J60"/>
     <mergeCell ref="D5:G5"/>
+    <mergeCell ref="B13:J13"/>
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="B12:C12"/>
@@ -4692,7 +4888,6 @@
     <mergeCell ref="B59:J59"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D7:G7"/>
-    <mergeCell ref="B56:J56"/>
     <mergeCell ref="H9:J9"/>
     <mergeCell ref="B58:J58"/>
     <mergeCell ref="D63:G66"/>
@@ -4731,9 +4926,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="56" min="0" max="16383" man="1"/>
-  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -6098,7 +6290,7 @@
       </c>
       <c r="B54" s="59" t="inlineStr">
         <is>
-          <t>serrage inclus</t>
+          <t>serrage compris</t>
         </is>
       </c>
       <c r="C54" s="59" t="inlineStr">
@@ -6115,7 +6307,7 @@
       </c>
       <c r="B55" s="59" t="inlineStr">
         <is>
-          <t>transport inclus</t>
+          <t>transport compris</t>
         </is>
       </c>
       <c r="C55" s="59" t="inlineStr">
@@ -6132,7 +6324,7 @@
       </c>
       <c r="B56" s="59" t="inlineStr">
         <is>
-          <t>serrage et transport inclus</t>
+          <t>serrage et transport compris</t>
         </is>
       </c>
       <c r="C56" s="59" t="inlineStr">
@@ -7887,7 +8079,7 @@
         <v/>
       </c>
       <c r="E34">
-        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("forfait",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(IF('3 Options'!$G$13="Forfait calculé (S + O + UC)",'3 Options'!$C$15+'3 Options'!$C$16,IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13,""))&lt;&gt;"","  "&amp;IF('3 Options'!$G$13="Forfait calculé (S + O + UC)",'3 Options'!$C$15+'3 Options'!$C$16,IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13,""))&amp;" "&amp;INDEX(Textes!$B$2:$C$59,MATCH("days",Textes!$A$2:$A$59,0),Listes!$H$1),"")&amp;IF('3 Options'!$D$13&lt;&gt;"","   ·   "&amp;'3 Options'!$D$13,"")</f>
+        <f>UPPER(INDEX(Textes!$B$2:$C$59,MATCH("forfait",Textes!$A$2:$A$59,0),Listes!$H$1))&amp;IF(IF('3 Options'!$G$13="Forfait calculé (S + O + UC)",'3 Options'!$C$15+'3 Options'!$C$16,IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13,""))&lt;&gt;"","  "&amp;IF('3 Options'!$G$13="Forfait calculé (S + O + UC)",'3 Options'!$C$15+'3 Options'!$C$16,IF('3 Options'!$G$13="Forfait par jour",'3 Options'!$E$13,""))&amp;" "&amp;INDEX(Textes!$B$2:$C$59,MATCH("days",Textes!$A$2:$A$59,0),Listes!$H$1),"")&amp;IF(IF(AND(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui")),INDEX(Textes!$B$2:$C$59,MATCH("in_both",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tight",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tr",Textes!$A$2:$A$59,0),Listes!$H$1),"")))&lt;&gt;"","   ·   "&amp;IF(AND(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui")),INDEX(Textes!$B$2:$C$59,MATCH("in_both",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tight",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tr",Textes!$A$2:$A$59,0),Listes!$H$1),""))),"")&amp;IF('3 Options'!$D$13&lt;&gt;"","   ·   "&amp;'3 Options'!$D$13,"")</f>
         <v/>
       </c>
       <c r="F34">
@@ -7937,7 +8129,7 @@
         <v/>
       </c>
       <c r="E35">
-        <f>IF(AND(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui")),INDEX(Textes!$B$2:$C$59,MATCH("in_both",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tight",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tr",Textes!$A$2:$A$59,0),Listes!$H$1),"")))&amp;IF(AND(IF(AND(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui")),INDEX(Textes!$B$2:$C$59,MATCH("in_both",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND('3 Options'!$C$8="Oui",'3 Options'!$C$19="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tight",Textes!$A$2:$A$59,0),Listes!$H$1),IF(AND(OR('3 Options'!$C$9="Oui",'3 Options'!$C$10="Oui"),'3 Options'!$C$20="Oui"),INDEX(Textes!$B$2:$C$59,MATCH("in_tr",Textes!$A$2:$A$59,0),Listes!$H$1),"")))&lt;&gt;"",'3 Options'!$D$14&lt;&gt;""),"   ·   ","")&amp;'3 Options'!$D$14</f>
+        <f>'3 Options'!$D$14</f>
         <v/>
       </c>
       <c r="F35">

</xml_diff>